<commit_message>
docs(11377): cap nhat testcase + design theo cac quyet dinh chot 30/09
Testcase (93 TC, 121 dong):
- TC_05.004 / TC_05.005 (N <= M khong canh bao): GIU NGUYEN, von dung spec
- TC_01.004, TC_09.001, TC_09.002: viet lai theo N chup luc tao - doi N o danh
  muc KHONG con doi han cua nhu cau da co
- TC_05.006: nguoi nhan canh bao gom ca 3 vai, kiem ca viec khong nhan trung
- Them TC_08.006..010: bo trong ca 3 o bao loi, cau bao loi chuan, chan so am o
  o M, chan ky tu e/E/+, cot han hien du chu khong bi cat
- 13 cho "Khong thoi han" -> "Khong gioi han thoi gian hieu luc" (chot 24/09)
- Bo sach emoji khoi noi dung o theo rule tc_engine (user chot 15/09): 22 dau
  canh bao -> chu "LUU Y:", 14 mui nhon -> "->", dau tru/nho hon bang -> ASCII

design.md: them muc "Quyet dinh da chot (30/09/2026)" ghi ro spec la nguon, phan
hoi QA khong phai can cu doi nghiep vu; ghi lai 3 diem lech spec con lai.

Refs #11377

Co-Authored-By: Claude Opus 5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/hrm/.plans/canh-bao-tu-dong-dong-nhu-cau/testcase.xlsx
+++ b/hrm/.plans/canh-bao-tu-dong-dong-nhu-cau/testcase.xlsx
@@ -567,7 +567,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q116"/>
+  <dimension ref="A1:Q121"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26.9" customWidth="1" min="1" max="1"/>
@@ -609,7 +609,7 @@
 - Danh mục › Lĩnh vực Công ty kinh doanh: khai N = 'Thời gian hiệu lực nhu cầu (ngày)' cho từng lĩnh vực.
 - Cấu hình › Cấu hình chung › thẻ Quản lý dự án › thẻ con Cấu hình hạn: khai M = 'Cảnh báo trước khi đóng nhu cầu' (ngày), dùng chung, mặc định 3.
 - Nhu cầu khách hàng (và thẻ 'Nhu cầu của khách hàng' ở màn Công việc của tôi): cột 'Thời gian hết hạn nhu cầu' + nút Tạo Dự án TKT.
-Công thức: T = thời điểm cuộc họp phát sinh nhu cầu chuyển sang Hoàn thành · cảnh báo tại T + N − M (chỉ khi N &gt; M) · tự đóng tại T + N.</t>
+Công thức: T = thời điểm cuộc họp phát sinh nhu cầu chuyển sang Hoàn thành · cảnh báo tại T + N - M (chỉ khi N &gt; M) · tự đóng tại T + N.</t>
         </is>
       </c>
       <c r="C2" s="4" t="n"/>
@@ -662,12 +662,12 @@
       </c>
       <c r="B4" s="3" t="inlineStr">
         <is>
-          <t>Không bao giờ tự cảnh báo và không bao giờ tự đóng (cột hạn ghi 'Không thời hạn'):
+          <t>Không bao giờ tự cảnh báo và không bao giờ tự đóng (cột hạn ghi 'Không giới hạn thời gian hiệu lực'):
 - Nhu cầu của lĩnh vực đang để N = 0 (đây là giá trị mặc định sau khi bổ sung trường này);
 - Nhu cầu mà cuộc họp chưa Hoàn thành (chưa có mốc T);
 - Nhu cầu đã lập Dự án TKT;
 - Nhu cầu đã ở trạng thái Đóng (do người dùng đóng tay hoặc hệ thống đã đóng trước đó).
-Riêng luồng CẢNH BÁO còn bị bỏ qua khi N ≤ M, hoặc khi M = 0, hoặc khi nhu cầu đó đã được cảnh báo một lần rồi (không nhắc lại mỗi ngày).</t>
+Riêng luồng CẢNH BÁO còn bị bỏ qua khi N &lt;= M, hoặc khi M = 0, hoặc khi nhu cầu đó đã được cảnh báo một lần rồi (không nhắc lại mỗi ngày).</t>
         </is>
       </c>
       <c r="C4" s="4" t="n"/>
@@ -719,9 +719,9 @@
       </c>
       <c r="B6" s="3" t="inlineStr">
         <is>
-          <t>Cuộc họp (có khảo sát nhu cầu) → nhiều Nhu cầu khách hàng → mỗi nhu cầu thuộc 1 Lĩnh vực Công ty kinh doanh và 1 Nhóm ngành → nhu cầu có thể được chuyển thành 1 Dự án TKT.
+          <t>Cuộc họp (có khảo sát nhu cầu) -&gt; nhiều Nhu cầu khách hàng -&gt; mỗi nhu cầu thuộc 1 Lĩnh vực Công ty kinh doanh và 1 Nhóm ngành -&gt; nhu cầu có thể được chuyển thành 1 Dự án TKT.
 N nằm ở bản ghi Lĩnh vực; M nằm ở Cấu hình chung theo công ty (công ty chưa khai thì hiểu là 3).
-Ngày hết hạn KHÔNG được lưu sẵn mà tính lại mỗi lần đọc: sửa N ở danh mục là hạn của mọi nhu cầu thuộc lĩnh vực đó đổi theo ngay.</t>
+Ngày hết hạn tính theo N ĐƯỢC CHỤP LẠI LÚC TẠO nhu cầu, không phải N hiện tại của lĩnh vực: sửa N ở danh mục thì nhu cầu đã có GIỮ NGUYÊN hạn cũ, chỉ nhu cầu tạo sau mới theo N mới. Vì vậy KHÔNG gia hạn được nhu cầu đang chạy bằng cách sửa N.</t>
         </is>
       </c>
       <c r="C6" s="4" t="n"/>
@@ -827,11 +827,11 @@
         <is>
           <t>Bẫy dễ sai nhất của đợt này:
 - N = 0 nghĩa là KHÔNG đặt thời hạn, không phải 'hết hạn ngay'. Mặc định sau khi lên bản mới, mọi lĩnh vực đều là 0, tức chưa nhu cầu nào bị đóng cho tới khi người quản trị khai N.
-- N ≤ M thì KHÔNG có bước cảnh báo, nhu cầu vẫn bị đóng đúng hạn. Đừng báo lỗi 'thiếu thông báo'.
+- N &lt;= M thì KHÔNG có bước cảnh báo, nhu cầu vẫn bị đóng đúng hạn. Đừng báo lỗi 'thiếu thông báo'.
 - Nhu cầu quá hạn vẫn nằm trong danh sách cho tới lần quét kế tiếp (01:20 hôm sau) mới chuyển sang Đóng — trong khoảng đó cột hạn hiện '(quá hạn X ngày)' là đúng.
 - Ngày đóng là ngày HẾT HẠN chứ không phải ngày chạy quét.
 - Sửa N ở danh mục làm hạn của mọi nhu cầu thuộc lĩnh vực đó đổi ngay, kể cả nhu cầu cũ.
-- ⚠️ Yêu cầu gốc viết badge là 'Đã đóng', hệ thống đang hiển thị 'Đóng' (nhãn có sẵn của màn nhu cầu). Ghi nhận là điểm cần chốt lại với người viết yêu cầu, không tự sửa.
+- LƯU Ý: Yêu cầu gốc viết badge là 'Đã đóng', hệ thống đang hiển thị 'Đóng' (nhãn có sẵn của màn nhu cầu). Ghi nhận là điểm cần chốt lại với người viết yêu cầu, không tự sửa.
 - Nút Tạo Dự án TKT với nhu cầu đã đóng bị ẩn hẳn (quy ước dự án: không hiện nút mờ), khác với câu chữ 'làm mờ kèm tooltip' trong yêu cầu gốc.</t>
         </is>
       </c>
@@ -1226,7 +1226,7 @@
       <c r="P20" s="16" t="inlineStr"/>
       <c r="Q20" s="16" t="inlineStr"/>
     </row>
-    <row r="21" ht="35" customHeight="1">
+    <row r="21" ht="37" customHeight="1">
       <c r="A21" s="15" t="inlineStr">
         <is>
           <t>Hạn xử lý nhu cầu KH</t>
@@ -1271,7 +1271,7 @@
       <c r="I21" s="15" t="inlineStr">
         <is>
           <t>- Hệ thống từ chối vì không có quyền
-- Cột 'Thời gian hiệu lực (ngày)' vẫn là 'Không thời hạn'</t>
+- Cột 'Thời gian hiệu lực (ngày)' vẫn là 'Không giới hạn thời gian hiệu lực'</t>
         </is>
       </c>
       <c r="J21" s="15" t="inlineStr"/>
@@ -1667,7 +1667,7 @@
       <c r="P27" s="4" t="n"/>
       <c r="Q27" s="5" t="n"/>
     </row>
-    <row r="28" ht="58" customHeight="1">
+    <row r="28" ht="66" customHeight="1">
       <c r="A28" s="15" t="inlineStr">
         <is>
           <t>Hạn xử lý nhu cầu KH</t>
@@ -1713,8 +1713,8 @@
         <is>
           <t>- Có cột 'Thời gian hiệu lực (ngày)' nằm ngay sau cột Tên, căn phải
 - Dòng LVCTKD.0001 hiện số 30
-- Dòng LVCTKD.KHAC hiện chữ 'Không thời hạn' màu xám
-- ⚠️ Không để số 0 trơ ra</t>
+- Dòng LVCTKD.KHAC hiện chữ 'Không giới hạn thời gian hiệu lực' màu xám
+- LƯU Ý: Không để số 0 trơ ra</t>
         </is>
       </c>
       <c r="J28" s="15" t="inlineStr"/>
@@ -1879,7 +1879,7 @@
       <c r="P30" s="16" t="inlineStr"/>
       <c r="Q30" s="16" t="inlineStr"/>
     </row>
-    <row r="31" ht="42" customHeight="1">
+    <row r="31" ht="56" customHeight="1">
       <c r="A31" s="15" t="inlineStr">
         <is>
           <t>Hạn xử lý nhu cầu KH</t>
@@ -1915,18 +1915,20 @@
           <t>1. Bấm Sửa dòng LVCTKD.0001
 2. Đổi N thành 60
 3. Bấm Lưu
-4. Sang màn Nhu cầu khách hàng, xem 5 nhu cầu đó</t>
+4. Sang màn Nhu cầu khách hàng, xem 5 nhu cầu cũ
+5. Tạo 1 nhu cầu mới thuộc lĩnh vực này rồi xem hạn của nó</t>
         </is>
       </c>
       <c r="H31" s="15" t="inlineStr">
         <is>
-          <t>Thời gian hiệu lực nhu cầu: 30 → 60</t>
+          <t>Thời gian hiệu lực nhu cầu: 30 -&gt; 60</t>
         </is>
       </c>
       <c r="I31" s="15" t="inlineStr">
         <is>
           <t>- Lưu thành công
-- ⚠️ Hạn của cả 5 nhu cầu tự lùi thêm 30 ngày ngay lập tức (hạn được tính lại, không lưu cứng theo giá trị cũ)</t>
+- LƯU Ý: Hạn của cả 5 nhu cầu cũ GIỮ NGUYÊN, không lùi ngày nào (N được chụp lại lúc tạo nhu cầu)
+- Riêng nhu cầu tạo MỚI ở bước 5 mới tính theo N = 60</t>
         </is>
       </c>
       <c r="J31" s="15" t="inlineStr"/>
@@ -1950,7 +1952,7 @@
       <c r="P31" s="16" t="inlineStr"/>
       <c r="Q31" s="16" t="inlineStr"/>
     </row>
-    <row r="32" ht="34" customHeight="1">
+    <row r="32" ht="37" customHeight="1">
       <c r="A32" s="15" t="inlineStr">
         <is>
           <t>Hạn xử lý nhu cầu KH</t>
@@ -1994,7 +1996,7 @@
       </c>
       <c r="I32" s="15" t="inlineStr">
         <is>
-          <t>- Cột hạn của nhu cầu #101 chuyển thành 'Không thời hạn'
+          <t>- Cột hạn của nhu cầu #101 chuyển thành 'Không giới hạn thời gian hiệu lực'
 - Nhu cầu không còn bị quét đóng nữa</t>
         </is>
       </c>
@@ -2019,7 +2021,7 @@
       <c r="P32" s="16" t="inlineStr"/>
       <c r="Q32" s="16" t="inlineStr"/>
     </row>
-    <row r="33" ht="47" customHeight="1">
+    <row r="33" ht="48" customHeight="1">
       <c r="A33" s="15" t="inlineStr">
         <is>
           <t>Hạn xử lý nhu cầu KH</t>
@@ -2065,7 +2067,7 @@
         <is>
           <t>- Ô viền đỏ kèm dòng chữ 'Bắt buộc phải nhập' ngay dưới ô
 - Cửa sổ không đóng, không tạo bản ghi
-- ⚠️ Ô để trống KHÔNG được ngầm hiểu thành 0</t>
+- LƯU Ý: Ô để trống KHÔNG được ngầm hiểu thành 0</t>
         </is>
       </c>
       <c r="J33" s="15" t="inlineStr"/>
@@ -2203,7 +2205,7 @@
       <c r="I35" s="15" t="inlineStr">
         <is>
           <t>- Báo lỗi ngay dưới ô, không lưu
-- ⚠️ Hệ thống không được tự đổi thành 0 hay 5</t>
+- LƯU Ý: Hệ thống không được tự đổi thành 0 hay 5</t>
         </is>
       </c>
       <c r="J35" s="15" t="inlineStr"/>
@@ -3005,7 +3007,7 @@
       <c r="P47" s="16" t="inlineStr"/>
       <c r="Q47" s="16" t="inlineStr"/>
     </row>
-    <row r="48" ht="42" customHeight="1">
+    <row r="48" ht="44" customHeight="1">
       <c r="A48" s="15" t="inlineStr">
         <is>
           <t>Hạn xử lý nhu cầu KH</t>
@@ -3051,7 +3053,7 @@
       <c r="I48" s="15" t="inlineStr">
         <is>
           <t>- Hệ thống không nhận số âm: ô báo lỗi, hoặc sau khi lưu giá trị về 0
-- ⚠️ Không được lưu ra số âm rồi dùng để tính mốc cảnh báo</t>
+- LƯU Ý: Không được lưu ra số âm rồi dùng để tính mốc cảnh báo</t>
         </is>
       </c>
       <c r="J48" s="15" t="inlineStr"/>
@@ -3114,7 +3116,7 @@
       </c>
       <c r="H49" s="15" t="inlineStr">
         <is>
-          <t>Cảnh báo trước khi đóng nhu cầu: 3 → 7</t>
+          <t>Cảnh báo trước khi đóng nhu cầu: 3 -&gt; 7</t>
         </is>
       </c>
       <c r="I49" s="15" t="inlineStr">
@@ -3348,7 +3350,7 @@
       </c>
       <c r="I53" s="15" t="inlineStr">
         <is>
-          <t>- Trước bước 1, cột hạn ghi 'Không thời hạn'
+          <t>- Trước bước 1, cột hạn ghi 'Không giới hạn thời gian hiệu lực'
 - Sau bước 1, cột hạn hiện đúng ngày = ngày hoàn thành + 30 ngày</t>
         </is>
       </c>
@@ -3418,7 +3420,7 @@
       <c r="I54" s="15" t="inlineStr">
         <is>
           <t>- Hạn vẫn là 01/10/2026
-- ⚠️ Không được nhảy thành ngày sửa + 30</t>
+- LƯU Ý: Không được nhảy thành ngày sửa + 30</t>
         </is>
       </c>
       <c r="J54" s="15" t="inlineStr"/>
@@ -3510,7 +3512,7 @@
       <c r="P55" s="16" t="inlineStr"/>
       <c r="Q55" s="16" t="inlineStr"/>
     </row>
-    <row r="56" ht="39" customHeight="1">
+    <row r="56" ht="40" customHeight="1">
       <c r="A56" s="15" t="inlineStr">
         <is>
           <t>Hạn xử lý nhu cầu KH</t>
@@ -3555,7 +3557,7 @@
       <c r="I56" s="15" t="inlineStr">
         <is>
           <t>- Hạn hiện 19/09/2026 (tính từ ngày kết thúc cuộc họp + 30 ngày)
-- ⚠️ Không lấy ngày sửa gần nhất của biên bản làm mốc</t>
+- LƯU Ý: Không lấy ngày sửa gần nhất của biên bản làm mốc</t>
         </is>
       </c>
       <c r="J56" s="15" t="inlineStr"/>
@@ -3579,7 +3581,7 @@
       <c r="P56" s="16" t="inlineStr"/>
       <c r="Q56" s="16" t="inlineStr"/>
     </row>
-    <row r="57" ht="34" customHeight="1">
+    <row r="57" ht="40" customHeight="1">
       <c r="A57" s="15" t="inlineStr">
         <is>
           <t>Hạn xử lý nhu cầu KH</t>
@@ -3622,7 +3624,7 @@
       </c>
       <c r="I57" s="15" t="inlineStr">
         <is>
-          <t>- Cột hạn ghi 'Không thời hạn'
+          <t>- Cột hạn ghi 'Không giới hạn thời gian hiệu lực'
 - Nhu cầu không bao giờ bị hệ thống tự đóng khi cuộc họp chưa Hoàn thành</t>
         </is>
       </c>
@@ -3670,7 +3672,7 @@
       <c r="P58" s="4" t="n"/>
       <c r="Q58" s="5" t="n"/>
     </row>
-    <row r="59" ht="51" customHeight="1">
+    <row r="59" ht="52" customHeight="1">
       <c r="A59" s="15" t="inlineStr">
         <is>
           <t>Hạn xử lý nhu cầu KH</t>
@@ -3715,7 +3717,7 @@
       <c r="I59" s="15" t="inlineStr">
         <is>
           <t>- Có cột 'Thời gian hết hạn nhu cầu', nằm sau cột 'Thời gian khánh thành dự án'
-- ⚠️ Không nhầm với cột 'Thời gian khánh thành dự án' (hai cột khác nhau)</t>
+- LƯU Ý: Không nhầm với cột 'Thời gian khánh thành dự án' (hai cột khác nhau)</t>
         </is>
       </c>
       <c r="J59" s="15" t="inlineStr"/>
@@ -3806,7 +3808,7 @@
       <c r="P60" s="16" t="inlineStr"/>
       <c r="Q60" s="16" t="inlineStr"/>
     </row>
-    <row r="61" ht="44" customHeight="1">
+    <row r="61" ht="46" customHeight="1">
       <c r="A61" s="15" t="inlineStr">
         <is>
           <t>Hạn xử lý nhu cầu KH</t>
@@ -3850,7 +3852,7 @@
       <c r="I61" s="15" t="inlineStr">
         <is>
           <t>- Hiện '17/09/2026 (còn 2 ngày)' màu CAM, đậm, có biểu tượng chuông báo
-- ⚠️ Màu cam chứ không phải đỏ (đỏ chỉ dành cho lỗi nhập liệu)</t>
+- LƯU Ý: Màu cam chứ không phải đỏ (đỏ chỉ dành cho lỗi nhập liệu)</t>
         </is>
       </c>
       <c r="J61" s="15" t="inlineStr"/>
@@ -3985,7 +3987,7 @@
       <c r="I63" s="15" t="inlineStr">
         <is>
           <t>- Hiện '12/09/2026 (quá hạn 3 ngày)' tô cam
-- ⚠️ TUYỆT ĐỐI không được hiện '(còn -3 ngày)'</t>
+- LƯU Ý: TUYỆT ĐỐI không được hiện '(còn -3 ngày)'</t>
         </is>
       </c>
       <c r="J63" s="15" t="inlineStr"/>
@@ -4052,7 +4054,7 @@
       </c>
       <c r="I64" s="15" t="inlineStr">
         <is>
-          <t>- Cột hạn ghi 'Không thời hạn' màu xám nhạt</t>
+          <t>- Cột hạn ghi 'Không giới hạn thời gian hiệu lực' màu xám nhạt</t>
         </is>
       </c>
       <c r="J64" s="15" t="inlineStr"/>
@@ -4119,7 +4121,7 @@
       </c>
       <c r="I65" s="15" t="inlineStr">
         <is>
-          <t>- Cột hạn ghi 'Không thời hạn'
+          <t>- Cột hạn ghi 'Không giới hạn thời gian hiệu lực'
 - Cột Trạng thái là 'Đã lập dự án TKT'</t>
         </is>
       </c>
@@ -4187,7 +4189,7 @@
       </c>
       <c r="I66" s="15" t="inlineStr">
         <is>
-          <t>- Cột hạn ghi 'Không thời hạn'
+          <t>- Cột hạn ghi 'Không giới hạn thời gian hiệu lực'
 - Badge trạng thái hiện 'Đóng' màu xám</t>
         </is>
       </c>
@@ -4459,7 +4461,7 @@
       </c>
       <c r="D71" s="15" t="inlineStr">
         <is>
-          <t>Cảnh báo đúng mốc T + N − M</t>
+          <t>Cảnh báo đúng mốc T + N - M</t>
         </is>
       </c>
       <c r="E71" s="16" t="inlineStr">
@@ -4469,7 +4471,7 @@
       </c>
       <c r="F71" s="15" t="inlineStr">
         <is>
-          <t>M = 3, lĩnh vực N = 30. Cuộc họp Hoàn thành 16/08/2026 → nhu cầu #201 hết hạn 15/09/2026. Hôm nay 12/09/2026. Nhu cầu chưa từng được cảnh báo, chưa lập dự án.</t>
+          <t>M = 3, lĩnh vực N = 30. Cuộc họp Hoàn thành 16/08/2026 -&gt; nhu cầu #201 hết hạn 15/09/2026. Hôm nay 12/09/2026. Nhu cầu chưa từng được cảnh báo, chưa lập dự án.</t>
         </is>
       </c>
       <c r="G71" s="15" t="inlineStr">
@@ -4650,7 +4652,7 @@
       <c r="P73" s="16" t="inlineStr"/>
       <c r="Q73" s="16" t="inlineStr"/>
     </row>
-    <row r="74" ht="66" customHeight="1">
+    <row r="74" ht="67" customHeight="1">
       <c r="A74" s="15" t="inlineStr">
         <is>
           <t>Hạn xử lý nhu cầu KH</t>
@@ -4668,7 +4670,7 @@
       </c>
       <c r="D74" s="15" t="inlineStr">
         <is>
-          <t>N ≤ M thì bỏ qua cảnh báo</t>
+          <t>N &lt;= M thì bỏ qua cảnh báo</t>
         </is>
       </c>
       <c r="E74" s="16" t="inlineStr">
@@ -4678,7 +4680,7 @@
       </c>
       <c r="F74" s="15" t="inlineStr">
         <is>
-          <t>M = 3, lĩnh vực đặt N = 2. Cuộc họp Hoàn thành hôm qua → nhu cầu #202 hết hạn ngày mai.</t>
+          <t>M = 3, lĩnh vực đặt N = 2. Cuộc họp Hoàn thành hôm qua -&gt; nhu cầu #202 hết hạn ngày mai.</t>
         </is>
       </c>
       <c r="G74" s="15" t="inlineStr">
@@ -4695,7 +4697,7 @@
       <c r="I74" s="15" t="inlineStr">
         <is>
           <t>- Không có dòng cảnh báo cho #202
-- ⚠️ Đây là đúng yêu cầu (thời gian hiệu lực ngắn hơn thời gian cảnh báo thì bỏ cảnh báo), không phải lỗi thiếu thông báo
+- LƯU Ý: Đây là đúng yêu cầu (thời gian hiệu lực ngắn hơn thời gian cảnh báo thì bỏ cảnh báo), không phải lỗi thiếu thông báo
 - Nhu cầu vẫn sẽ bị đóng đúng ngày hết hạn</t>
         </is>
       </c>
@@ -4788,7 +4790,7 @@
       <c r="P75" s="16" t="inlineStr"/>
       <c r="Q75" s="16" t="inlineStr"/>
     </row>
-    <row r="76" ht="37" customHeight="1">
+    <row r="76" ht="101" customHeight="1">
       <c r="A76" s="15" t="inlineStr">
         <is>
           <t>Hạn xử lý nhu cầu KH</t>
@@ -4806,7 +4808,7 @@
       </c>
       <c r="D76" s="15" t="inlineStr">
         <is>
-          <t>Người nhận cảnh báo là người chủ trì cuộc họp</t>
+          <t>Người nhận cảnh báo gồm cả 3 vai</t>
         </is>
       </c>
       <c r="E76" s="16" t="inlineStr">
@@ -4816,13 +4818,13 @@
       </c>
       <c r="F76" s="15" t="inlineStr">
         <is>
-          <t>Cuộc họp M-01 do Nguyễn Thị Cần chủ trì, do Trần Văn B tạo. Nhu cầu #201 vào vùng cảnh báo.</t>
+          <t>Cuộc họp M-01 do Nguyễn Thị Cần chủ trì, do Trần Văn B tạo hộ. Nhu cầu #201 đã bàn giao cho Lê Thị C phụ trách, đang trong vùng cảnh báo.</t>
         </is>
       </c>
       <c r="G76" s="15" t="inlineStr">
         <is>
           <t>1. Chạy lệnh quét hạn nhu cầu
-2. Kiểm tra chuông thông báo của cả 2 tài khoản</t>
+2. Kiểm tra chuông thông báo của cả 3 tài khoản</t>
         </is>
       </c>
       <c r="H76" s="15" t="inlineStr">
@@ -4832,8 +4834,9 @@
       </c>
       <c r="I76" s="15" t="inlineStr">
         <is>
-          <t>- Nguyễn Thị Cần nhận thông báo
-- Trần Văn B không nhận (chỉ nhận khi cuộc họp không xác định được người chủ trì)</t>
+          <t>- CẢ 3 đều nhận thông báo: Lê Thị C (nhân sự phụ trách nhu cầu), Trần Văn B (người tạo cuộc họp), Nguyễn Thị Cần (người chủ trì)
+- Mỗi người nhận ĐÚNG 1 thông báo; nếu một người giữ nhiều vai thì cũng chỉ nhận 1, không nhận trùng
+- Nhu cầu CHƯA bàn giao lần nào thì người phụ trách hiểu là người chủ trì</t>
         </is>
       </c>
       <c r="J76" s="15" t="inlineStr"/>
@@ -5154,7 +5157,7 @@
       <c r="P81" s="4" t="n"/>
       <c r="Q81" s="5" t="n"/>
     </row>
-    <row r="82" ht="50" customHeight="1">
+    <row r="82" ht="56" customHeight="1">
       <c r="A82" s="15" t="inlineStr">
         <is>
           <t>Hạn xử lý nhu cầu KH</t>
@@ -5182,7 +5185,7 @@
       </c>
       <c r="F82" s="15" t="inlineStr">
         <is>
-          <t>M = 3, N = 30, cuộc họp Hoàn thành 16/08/2026 → nhu cầu #301 hết hạn 15/09/2026. Hôm nay 15/09/2026.</t>
+          <t>M = 3, N = 30, cuộc họp Hoàn thành 16/08/2026 -&gt; nhu cầu #301 hết hạn 15/09/2026. Hôm nay 15/09/2026.</t>
         </is>
       </c>
       <c r="G82" s="15" t="inlineStr">
@@ -5200,7 +5203,7 @@
         <is>
           <t>- Kết quả in ra có dòng ĐÓNG cho #301 — hết hạn 15/09/2026
 - Trạng thái #301 chuyển sang 'Đóng', badge màu xám
-- Cột hạn chuyển thành 'Không thời hạn'</t>
+- Cột hạn chuyển thành 'Không giới hạn thời gian hiệu lực'</t>
         </is>
       </c>
       <c r="J82" s="15" t="inlineStr"/>
@@ -5269,7 +5272,7 @@
       <c r="I83" s="15" t="inlineStr">
         <is>
           <t>- Nhu cầu chuyển sang Đóng
-- ⚠️ Ngày đóng ghi 10/09/2026 (ngày hết hạn thật), KHÔNG phải 15/09/2026</t>
+- LƯU Ý: Ngày đóng ghi 10/09/2026 (ngày hết hạn thật), KHÔNG phải 15/09/2026</t>
         </is>
       </c>
       <c r="J83" s="15" t="inlineStr"/>
@@ -5634,7 +5637,7 @@
       <c r="P88" s="16" t="inlineStr"/>
       <c r="Q88" s="16" t="inlineStr"/>
     </row>
-    <row r="89" ht="60" customHeight="1">
+    <row r="89" ht="61" customHeight="1">
       <c r="A89" s="15" t="inlineStr">
         <is>
           <t>Hạn xử lý nhu cầu KH</t>
@@ -5680,7 +5683,7 @@
       <c r="I89" s="15" t="inlineStr">
         <is>
           <t>- Kết quả liệt kê toàn bộ nhu cầu cũ sẽ bị đóng, mỗi dòng kèm đúng ngày hết hạn riêng
-- ⚠️ Kiểm kỹ trước khi chạy thật: đặt N nhỏ là đóng hàng loạt nhu cầu cũ ngay lần quét kế tiếp</t>
+- LƯU Ý: Kiểm kỹ trước khi chạy thật: đặt N nhỏ là đóng hàng loạt nhu cầu cũ ngay lần quét kế tiếp</t>
         </is>
       </c>
       <c r="J89" s="15" t="inlineStr"/>
@@ -5796,7 +5799,7 @@
       <c r="P91" s="4" t="n"/>
       <c r="Q91" s="5" t="n"/>
     </row>
-    <row r="92" ht="50" customHeight="1">
+    <row r="92" ht="51" customHeight="1">
       <c r="A92" s="15" t="inlineStr">
         <is>
           <t>Hạn xử lý nhu cầu KH</t>
@@ -5841,7 +5844,7 @@
       <c r="I92" s="15" t="inlineStr">
         <is>
           <t>- Ô chỉ hiện dấu '—', KHÔNG còn nút Tạo Dự án TKT
-- ⚠️ Yêu cầu gốc ghi 'làm mờ kèm tooltip' nhưng quy ước dự án là ẩn hẳn — ghi nhận, không tính là lỗi</t>
+- LƯU Ý: Yêu cầu gốc ghi 'làm mờ kèm tooltip' nhưng quy ước dự án là ẩn hẳn — ghi nhận, không tính là lỗi</t>
         </is>
       </c>
       <c r="J92" s="15" t="inlineStr"/>
@@ -6272,7 +6275,7 @@
       <c r="I99" s="15" t="inlineStr">
         <is>
           <t>- Cả 3 nơi đều hiện cùng một nhãn trạng thái màu xám
-- ⚠️ Hệ thống đang ghi 'Đóng' trong khi yêu cầu gốc ghi 'Đã đóng' — ghi nhận để chốt lại, không tự sửa</t>
+- LƯU Ý: Hệ thống đang ghi 'Đóng' trong khi yêu cầu gốc ghi 'Đã đóng' — ghi nhận để chốt lại, không tự sửa</t>
         </is>
       </c>
       <c r="J99" s="15" t="inlineStr"/>
@@ -6365,7 +6368,7 @@
       <c r="P100" s="16" t="inlineStr"/>
       <c r="Q100" s="16" t="inlineStr"/>
     </row>
-    <row r="101" ht="35" customHeight="1">
+    <row r="101" ht="37" customHeight="1">
       <c r="A101" s="15" t="inlineStr">
         <is>
           <t>Hạn xử lý nhu cầu KH</t>
@@ -6409,7 +6412,7 @@
       <c r="I101" s="15" t="inlineStr">
         <is>
           <t>- Bị từ chối với thông báo bắt buộc phải nhập
-- ⚠️ Không được ngầm hiểu thành 0 rồi tắt hạn của cả lĩnh vực</t>
+- LƯU Ý: Không được ngầm hiểu thành 0 rồi tắt hạn của cả lĩnh vực</t>
         </is>
       </c>
       <c r="J101" s="15" t="inlineStr"/>
@@ -6501,7 +6504,7 @@
       <c r="P102" s="16" t="inlineStr"/>
       <c r="Q102" s="16" t="inlineStr"/>
     </row>
-    <row r="103" ht="57" customHeight="1">
+    <row r="103" ht="63" customHeight="1">
       <c r="A103" s="15" t="inlineStr">
         <is>
           <t>Hạn xử lý nhu cầu KH</t>
@@ -6545,7 +6548,7 @@
       </c>
       <c r="I103" s="15" t="inlineStr">
         <is>
-          <t>- Nếu file có cột thời gian hiệu lực thì giá trị phải khớp bảng (30 và 'Không thời hạn'/0)
+          <t>- Nếu file có cột thời gian hiệu lực thì giá trị phải khớp bảng (30 và 'Không giới hạn thời gian hiệu lực'/0)
 - Nếu file không có cột này thì ghi nhận là điểm cần bổ sung, không phải lỗi chặn</t>
         </is>
       </c>
@@ -6570,30 +6573,75 @@
       <c r="P103" s="16" t="inlineStr"/>
       <c r="Q103" s="16" t="inlineStr"/>
     </row>
-    <row r="104" ht="26" customHeight="1">
-      <c r="A104" s="13" t="n"/>
-      <c r="B104" s="13" t="n"/>
-      <c r="C104" s="14" t="inlineStr">
-        <is>
-          <t>IX. CÔ LẬP DỮ LIỆU &amp; THAO TÁC ĐỒNG THỜI</t>
-        </is>
-      </c>
-      <c r="D104" s="4" t="n"/>
-      <c r="E104" s="4" t="n"/>
-      <c r="F104" s="4" t="n"/>
-      <c r="G104" s="4" t="n"/>
-      <c r="H104" s="4" t="n"/>
-      <c r="I104" s="4" t="n"/>
-      <c r="J104" s="4" t="n"/>
-      <c r="K104" s="4" t="n"/>
-      <c r="L104" s="4" t="n"/>
-      <c r="M104" s="4" t="n"/>
-      <c r="N104" s="4" t="n"/>
-      <c r="O104" s="4" t="n"/>
-      <c r="P104" s="4" t="n"/>
-      <c r="Q104" s="5" t="n"/>
-    </row>
-    <row r="105" ht="34" customHeight="1">
+    <row r="104" ht="39" customHeight="1">
+      <c r="A104" s="15" t="inlineStr">
+        <is>
+          <t>Hạn xử lý nhu cầu KH</t>
+        </is>
+      </c>
+      <c r="B104" s="15" t="inlineStr">
+        <is>
+          <t>RÀNG BUỘC NHẬP LIỆU &amp; HIỂN THỊ TRẠNG THÁI</t>
+        </is>
+      </c>
+      <c r="C104" s="16" t="inlineStr">
+        <is>
+          <t>TC_08.006</t>
+        </is>
+      </c>
+      <c r="D104" s="15" t="inlineStr">
+        <is>
+          <t>Bỏ trống cả Mã, Tên và N thì cả 3 ô đều báo lỗi</t>
+        </is>
+      </c>
+      <c r="E104" s="16" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="F104" s="15" t="inlineStr">
+        <is>
+          <t>Đang mở form Thêm mới lĩnh vực, chưa nhập gì.</t>
+        </is>
+      </c>
+      <c r="G104" s="15" t="inlineStr">
+        <is>
+          <t>1. Bấm Lưu ngay khi form còn trống</t>
+        </is>
+      </c>
+      <c r="H104" s="15" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I104" s="15" t="inlineStr">
+        <is>
+          <t>- CẢ 3 ô Mã, Tên, Thời gian hiệu lực đều viền đỏ kèm text lỗi
+- LƯU Ý: Không được chỉ mỗi ô Thời gian hiệu lực báo đỏ</t>
+        </is>
+      </c>
+      <c r="J104" s="15" t="inlineStr"/>
+      <c r="K104" s="16" t="inlineStr">
+        <is>
+          <t>Not Executed</t>
+        </is>
+      </c>
+      <c r="L104" s="16" t="inlineStr">
+        <is>
+          <t>Not Executed</t>
+        </is>
+      </c>
+      <c r="M104" s="16" t="inlineStr">
+        <is>
+          <t>Not Executed</t>
+        </is>
+      </c>
+      <c r="N104" s="15" t="inlineStr"/>
+      <c r="O104" s="16" t="inlineStr"/>
+      <c r="P104" s="16" t="inlineStr"/>
+      <c r="Q104" s="16" t="inlineStr"/>
+    </row>
+    <row r="105" ht="38" customHeight="1">
       <c r="A105" s="15" t="inlineStr">
         <is>
           <t>Hạn xử lý nhu cầu KH</t>
@@ -6601,17 +6649,17 @@
       </c>
       <c r="B105" s="15" t="inlineStr">
         <is>
-          <t>CÔ LẬP DỮ LIỆU &amp; THAO TÁC ĐỒNG THỜI</t>
+          <t>RÀNG BUỘC NHẬP LIỆU &amp; HIỂN THỊ TRẠNG THÁI</t>
         </is>
       </c>
       <c r="C105" s="16" t="inlineStr">
         <is>
-          <t>TC_09.001</t>
+          <t>TC_08.007</t>
         </is>
       </c>
       <c r="D105" s="15" t="inlineStr">
         <is>
-          <t>Đổi N trong lúc nhu cầu đang chờ đóng</t>
+          <t>Câu báo lỗi khi bỏ trống N và M</t>
         </is>
       </c>
       <c r="E105" s="16" t="inlineStr">
@@ -6621,24 +6669,24 @@
       </c>
       <c r="F105" s="15" t="inlineStr">
         <is>
-          <t>Nhu cầu #431 hết hạn hôm nay theo N = 30.</t>
+          <t>Form lĩnh vực và màn Cấu hình chung › Cấu hình hạn.</t>
         </is>
       </c>
       <c r="G105" s="15" t="inlineStr">
         <is>
-          <t>1. Trước khi chạy quét, đổi N của lĩnh vực thành 60
-2. Chạy lệnh quét hạn nhu cầu</t>
+          <t>1. Xoá trắng ô Thời gian hiệu lực nhu cầu rồi bấm Lưu
+2. Xoá trắng ô Cảnh báo trước khi đóng nhu cầu rồi bấm Lưu</t>
         </is>
       </c>
       <c r="H105" s="15" t="inlineStr">
         <is>
-          <t>Thời gian hiệu lực nhu cầu: 30 → 60</t>
+          <t>—</t>
         </is>
       </c>
       <c r="I105" s="15" t="inlineStr">
         <is>
-          <t>- Nhu cầu #431 KHÔNG bị đóng
-- Cột hạn lùi thêm 30 ngày</t>
+          <t>- Cả 2 ô báo đúng câu: 'Bắt buộc nhập, kiểu số nguyên dương &gt;= 0'
+- Không báo tiếng Anh, không báo câu chung chung</t>
         </is>
       </c>
       <c r="J105" s="15" t="inlineStr"/>
@@ -6662,7 +6710,7 @@
       <c r="P105" s="16" t="inlineStr"/>
       <c r="Q105" s="16" t="inlineStr"/>
     </row>
-    <row r="106" ht="38" customHeight="1">
+    <row r="106" ht="46" customHeight="1">
       <c r="A106" s="15" t="inlineStr">
         <is>
           <t>Hạn xử lý nhu cầu KH</t>
@@ -6670,17 +6718,17 @@
       </c>
       <c r="B106" s="15" t="inlineStr">
         <is>
-          <t>CÔ LẬP DỮ LIỆU &amp; THAO TÁC ĐỒNG THỜI</t>
+          <t>RÀNG BUỘC NHẬP LIỆU &amp; HIỂN THỊ TRẠNG THÁI</t>
         </is>
       </c>
       <c r="C106" s="16" t="inlineStr">
         <is>
-          <t>TC_09.002</t>
+          <t>TC_08.008</t>
         </is>
       </c>
       <c r="D106" s="15" t="inlineStr">
         <is>
-          <t>Đổi N nhỏ hơn làm nhu cầu quá hạn ngay</t>
+          <t>Ô M không nhận số âm</t>
         </is>
       </c>
       <c r="E106" s="16" t="inlineStr">
@@ -6690,25 +6738,26 @@
       </c>
       <c r="F106" s="15" t="inlineStr">
         <is>
-          <t>Nhu cầu #432 có cuộc họp Hoàn thành cách đây 40 ngày, lĩnh vực đang N = 60.</t>
+          <t>Màn Cấu hình chung › thẻ Quản lý dự án › thẻ con Cấu hình hạn.</t>
         </is>
       </c>
       <c r="G106" s="15" t="inlineStr">
         <is>
-          <t>1. Đổi N của lĩnh vực xuống 30
-2. Xem cột hạn của #432
-3. Chạy lệnh quét hạn nhu cầu</t>
+          <t>1. Gõ dấu trừ vào ô Cảnh báo trước khi đóng nhu cầu
+2. Thử dán giá trị -5 vào ô đó
+3. Bấm Lưu</t>
         </is>
       </c>
       <c r="H106" s="15" t="inlineStr">
         <is>
-          <t>Thời gian hiệu lực nhu cầu: 60 → 30</t>
+          <t>Cảnh báo trước khi đóng nhu cầu: -5</t>
         </is>
       </c>
       <c r="I106" s="15" t="inlineStr">
         <is>
-          <t>- Cột hạn chuyển sang '(quá hạn 10 ngày)' tô cam
-- Lần quét kế tiếp đóng nhu cầu với ngày đóng là ngày hết hạn mới</t>
+          <t>- Bước 1: bàn phím KHÔNG gõ được dấu trừ
+- Bước 2: dán không vào
+- LƯU Ý: Hệ thống KHÔNG được tự kéo giá trị về 0, phải báo đỏ và chặn lưu</t>
         </is>
       </c>
       <c r="J106" s="15" t="inlineStr"/>
@@ -6740,17 +6789,17 @@
       </c>
       <c r="B107" s="15" t="inlineStr">
         <is>
-          <t>CÔ LẬP DỮ LIỆU &amp; THAO TÁC ĐỒNG THỜI</t>
+          <t>RÀNG BUỘC NHẬP LIỆU &amp; HIỂN THỊ TRẠNG THÁI</t>
         </is>
       </c>
       <c r="C107" s="16" t="inlineStr">
         <is>
-          <t>TC_09.003</t>
+          <t>TC_08.009</t>
         </is>
       </c>
       <c r="D107" s="15" t="inlineStr">
         <is>
-          <t>Đổi M khi nhu cầu đã được cảnh báo</t>
+          <t>Ô N và M không nhận ký tự e, E, dấu cộng</t>
         </is>
       </c>
       <c r="E107" s="16" t="inlineStr">
@@ -6760,24 +6809,24 @@
       </c>
       <c r="F107" s="15" t="inlineStr">
         <is>
-          <t>Nhu cầu #433 đã nhận cảnh báo khi M = 3.</t>
+          <t>Form lĩnh vực và màn Cấu hình hạn.</t>
         </is>
       </c>
       <c r="G107" s="15" t="inlineStr">
         <is>
-          <t>1. Đổi M thành 10
-2. Chạy lại lệnh quét hạn nhu cầu</t>
+          <t>1. Gõ 1e3333 vào ô Thời gian hiệu lực nhu cầu
+2. Làm tương tự với ô Cảnh báo trước khi đóng</t>
         </is>
       </c>
       <c r="H107" s="15" t="inlineStr">
         <is>
-          <t>Cảnh báo trước khi đóng nhu cầu: 3 → 10</t>
+          <t>—</t>
         </is>
       </c>
       <c r="I107" s="15" t="inlineStr">
         <is>
-          <t>- Không gửi lại thông báo cho #433 (mỗi nhu cầu chỉ cảnh báo một lần)
-- Trên bảng, dòng vẫn tô cam</t>
+          <t>- Không gõ được e, E, dấu cộng
+- Ô không bị rỗng trắng sau khi gõ, giá trị giữ đúng phần số đã nhập</t>
         </is>
       </c>
       <c r="J107" s="15" t="inlineStr"/>
@@ -6801,7 +6850,7 @@
       <c r="P107" s="16" t="inlineStr"/>
       <c r="Q107" s="16" t="inlineStr"/>
     </row>
-    <row r="108" ht="34" customHeight="1">
+    <row r="108" ht="46" customHeight="1">
       <c r="A108" s="15" t="inlineStr">
         <is>
           <t>Hạn xử lý nhu cầu KH</t>
@@ -6809,33 +6858,33 @@
       </c>
       <c r="B108" s="15" t="inlineStr">
         <is>
-          <t>CÔ LẬP DỮ LIỆU &amp; THAO TÁC ĐỒNG THỜI</t>
+          <t>RÀNG BUỘC NHẬP LIỆU &amp; HIỂN THỊ TRẠNG THÁI</t>
         </is>
       </c>
       <c r="C108" s="16" t="inlineStr">
         <is>
-          <t>TC_09.004</t>
+          <t>TC_08.010</t>
         </is>
       </c>
       <c r="D108" s="15" t="inlineStr">
         <is>
-          <t>Người dùng lập dự án ngay trước giờ quét</t>
+          <t>Cột hạn hiện đủ chữ, không bị cắt</t>
         </is>
       </c>
       <c r="E108" s="16" t="inlineStr">
         <is>
-          <t>P0</t>
+          <t>P1</t>
         </is>
       </c>
       <c r="F108" s="15" t="inlineStr">
         <is>
-          <t>Nhu cầu #434 hết hạn hôm nay; người dùng lập Dự án TKT từ nhu cầu này lúc 23:50.</t>
+          <t>Danh mục có lĩnh vực để N = 0; màn Nhu cầu khách hàng có nhu cầu thuộc lĩnh vực đó.</t>
         </is>
       </c>
       <c r="G108" s="15" t="inlineStr">
         <is>
-          <t>1. Chạy lệnh quét hạn nhu cầu sau đó
-2. Kiểm tra #434</t>
+          <t>1. Mở màn Danh mục › Lĩnh vực Công ty kinh doanh, xem cột Thời gian hiệu lực
+2. Mở màn Nhu cầu khách hàng, xem cột Thời gian hết hạn nhu cầu</t>
         </is>
       </c>
       <c r="H108" s="15" t="inlineStr">
@@ -6845,7 +6894,8 @@
       </c>
       <c r="I108" s="15" t="inlineStr">
         <is>
-          <t>- Không bị đóng, trạng thái là 'Đã lập dự án TKT'</t>
+          <t>- Cả 2 màn hiện ĐỦ cụm 'Không giới hạn thời gian hiệu lực'
+- LƯU Ý: Không bị cắt thành '...thời gian hiệu' kèm dấu ba chấm</t>
         </is>
       </c>
       <c r="J108" s="15" t="inlineStr"/>
@@ -6869,119 +6919,75 @@
       <c r="P108" s="16" t="inlineStr"/>
       <c r="Q108" s="16" t="inlineStr"/>
     </row>
-    <row r="109" ht="34" customHeight="1">
-      <c r="A109" s="15" t="inlineStr">
-        <is>
-          <t>Hạn xử lý nhu cầu KH</t>
-        </is>
-      </c>
-      <c r="B109" s="15" t="inlineStr">
+    <row r="109" ht="26" customHeight="1">
+      <c r="A109" s="13" t="n"/>
+      <c r="B109" s="13" t="n"/>
+      <c r="C109" s="14" t="inlineStr">
+        <is>
+          <t>IX. CÔ LẬP DỮ LIỆU &amp; THAO TÁC ĐỒNG THỜI</t>
+        </is>
+      </c>
+      <c r="D109" s="4" t="n"/>
+      <c r="E109" s="4" t="n"/>
+      <c r="F109" s="4" t="n"/>
+      <c r="G109" s="4" t="n"/>
+      <c r="H109" s="4" t="n"/>
+      <c r="I109" s="4" t="n"/>
+      <c r="J109" s="4" t="n"/>
+      <c r="K109" s="4" t="n"/>
+      <c r="L109" s="4" t="n"/>
+      <c r="M109" s="4" t="n"/>
+      <c r="N109" s="4" t="n"/>
+      <c r="O109" s="4" t="n"/>
+      <c r="P109" s="4" t="n"/>
+      <c r="Q109" s="5" t="n"/>
+    </row>
+    <row r="110" ht="48" customHeight="1">
+      <c r="A110" s="15" t="inlineStr">
+        <is>
+          <t>Hạn xử lý nhu cầu KH</t>
+        </is>
+      </c>
+      <c r="B110" s="15" t="inlineStr">
         <is>
           <t>CÔ LẬP DỮ LIỆU &amp; THAO TÁC ĐỒNG THỜI</t>
         </is>
       </c>
-      <c r="C109" s="16" t="inlineStr">
-        <is>
-          <t>TC_09.005</t>
-        </is>
-      </c>
-      <c r="D109" s="15" t="inlineStr">
-        <is>
-          <t>Hai người cùng thao tác trên một nhu cầu</t>
-        </is>
-      </c>
-      <c r="E109" s="16" t="inlineStr">
-        <is>
-          <t>P1</t>
-        </is>
-      </c>
-      <c r="F109" s="15" t="inlineStr">
-        <is>
-          <t>Người 1 đang mở form lập dự án từ nhu cầu #435; người 2 đóng tay nhu cầu đó.</t>
-        </is>
-      </c>
-      <c r="G109" s="15" t="inlineStr">
-        <is>
-          <t>1. Người 1 bấm Lưu form lập dự án</t>
-        </is>
-      </c>
-      <c r="H109" s="15" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="I109" s="15" t="inlineStr">
-        <is>
-          <t>- Bị chặn kèm thông báo nhu cầu đã đóng, không tạo dự án
-- Màn không treo</t>
-        </is>
-      </c>
-      <c r="J109" s="15" t="inlineStr"/>
-      <c r="K109" s="16" t="inlineStr">
-        <is>
-          <t>Not Executed</t>
-        </is>
-      </c>
-      <c r="L109" s="16" t="inlineStr">
-        <is>
-          <t>Not Executed</t>
-        </is>
-      </c>
-      <c r="M109" s="16" t="inlineStr">
-        <is>
-          <t>Not Executed</t>
-        </is>
-      </c>
-      <c r="N109" s="15" t="inlineStr"/>
-      <c r="O109" s="16" t="inlineStr"/>
-      <c r="P109" s="16" t="inlineStr"/>
-      <c r="Q109" s="16" t="inlineStr"/>
-    </row>
-    <row r="110" ht="34" customHeight="1">
-      <c r="A110" s="15" t="inlineStr">
-        <is>
-          <t>Hạn xử lý nhu cầu KH</t>
-        </is>
-      </c>
-      <c r="B110" s="15" t="inlineStr">
-        <is>
-          <t>CÔ LẬP DỮ LIỆU &amp; THAO TÁC ĐỒNG THỜI</t>
-        </is>
-      </c>
       <c r="C110" s="16" t="inlineStr">
         <is>
-          <t>TC_09.006</t>
+          <t>TC_09.001</t>
         </is>
       </c>
       <c r="D110" s="15" t="inlineStr">
         <is>
-          <t>Quét chạy khi hệ thống chưa có cấu hình M</t>
+          <t>Đổi N trong lúc nhu cầu đang chờ đóng</t>
         </is>
       </c>
       <c r="E110" s="16" t="inlineStr">
         <is>
-          <t>P1</t>
+          <t>P0</t>
         </is>
       </c>
       <c r="F110" s="15" t="inlineStr">
         <is>
-          <t>Công ty của cuộc họp chưa từng lưu cấu hình hạn.</t>
+          <t>Nhu cầu #431 hết hạn hôm nay, N chụp lúc tạo là 30.</t>
         </is>
       </c>
       <c r="G110" s="15" t="inlineStr">
         <is>
-          <t>1. Chạy lệnh quét hạn nhu cầu với 1 nhu cầu còn 2 ngày tới hạn (N = 30)</t>
+          <t>1. Trước khi chạy quét, đổi N của lĩnh vực thành 60
+2. Chạy lệnh quét hạn nhu cầu</t>
         </is>
       </c>
       <c r="H110" s="15" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Thời gian hiệu lực nhu cầu: 30 -&gt; 60</t>
         </is>
       </c>
       <c r="I110" s="15" t="inlineStr">
         <is>
-          <t>- Hệ thống dùng mặc định 3 ngày: nhu cầu vẫn được cảnh báo
-- Không văng lỗi vì thiếu cấu hình</t>
+          <t>- LƯU Ý: Nhu cầu #431 VẪN BỊ ĐÓNG hôm nay — sửa N ở danh mục KHÔNG gia hạn được nhu cầu đang chạy
+- Cột hạn không đổi, vẫn là hạn tính theo N = 30</t>
         </is>
       </c>
       <c r="J110" s="15" t="inlineStr"/>
@@ -7018,37 +7024,40 @@
       </c>
       <c r="C111" s="16" t="inlineStr">
         <is>
-          <t>TC_09.007</t>
+          <t>TC_09.002</t>
         </is>
       </c>
       <c r="D111" s="15" t="inlineStr">
         <is>
-          <t>Cuộc họp bị xoá hoặc thiếu người chủ trì</t>
+          <t>Đổi N nhỏ hơn KHÔNG làm nhu cầu quá hạn</t>
         </is>
       </c>
       <c r="E111" s="16" t="inlineStr">
         <is>
-          <t>P2</t>
+          <t>P0</t>
         </is>
       </c>
       <c r="F111" s="15" t="inlineStr">
         <is>
-          <t>Nhu cầu #436 tới vùng cảnh báo nhưng cuộc họp không xác định được người chủ trì lẫn người tạo.</t>
+          <t>Nhu cầu #432 có cuộc họp Hoàn thành cách đây 40 ngày, N chụp lúc tạo là 60.</t>
         </is>
       </c>
       <c r="G111" s="15" t="inlineStr">
         <is>
-          <t>1. Chạy lệnh quét hạn nhu cầu</t>
+          <t>1. Đổi N của lĩnh vực xuống 30
+2. Xem cột hạn của #432
+3. Chạy lệnh quét hạn nhu cầu</t>
         </is>
       </c>
       <c r="H111" s="15" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Thời gian hiệu lực nhu cầu: 60 -&gt; 30</t>
         </is>
       </c>
       <c r="I111" s="15" t="inlineStr">
         <is>
-          <t>- Không gửi được thông báo nhưng lệnh vẫn chạy hết, các nhu cầu khác vẫn được xử lý bình thường</t>
+          <t>- LƯU Ý: Cột hạn KHÔNG đổi, vẫn tính theo N = 60 nên còn 20 ngày
+- Nhu cầu KHÔNG bị đóng</t>
         </is>
       </c>
       <c r="J111" s="15" t="inlineStr"/>
@@ -7072,61 +7081,401 @@
       <c r="P111" s="16" t="inlineStr"/>
       <c r="Q111" s="16" t="inlineStr"/>
     </row>
-    <row r="112" ht="26" customHeight="1">
-      <c r="A112" s="13" t="n"/>
-      <c r="B112" s="13" t="n"/>
-      <c r="C112" s="14" t="inlineStr">
+    <row r="112" ht="34" customHeight="1">
+      <c r="A112" s="15" t="inlineStr">
+        <is>
+          <t>Hạn xử lý nhu cầu KH</t>
+        </is>
+      </c>
+      <c r="B112" s="15" t="inlineStr">
+        <is>
+          <t>CÔ LẬP DỮ LIỆU &amp; THAO TÁC ĐỒNG THỜI</t>
+        </is>
+      </c>
+      <c r="C112" s="16" t="inlineStr">
+        <is>
+          <t>TC_09.003</t>
+        </is>
+      </c>
+      <c r="D112" s="15" t="inlineStr">
+        <is>
+          <t>Đổi M khi nhu cầu đã được cảnh báo</t>
+        </is>
+      </c>
+      <c r="E112" s="16" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="F112" s="15" t="inlineStr">
+        <is>
+          <t>Nhu cầu #433 đã nhận cảnh báo khi M = 3.</t>
+        </is>
+      </c>
+      <c r="G112" s="15" t="inlineStr">
+        <is>
+          <t>1. Đổi M thành 10
+2. Chạy lại lệnh quét hạn nhu cầu</t>
+        </is>
+      </c>
+      <c r="H112" s="15" t="inlineStr">
+        <is>
+          <t>Cảnh báo trước khi đóng nhu cầu: 3 -&gt; 10</t>
+        </is>
+      </c>
+      <c r="I112" s="15" t="inlineStr">
+        <is>
+          <t>- Không gửi lại thông báo cho #433 (mỗi nhu cầu chỉ cảnh báo một lần)
+- Trên bảng, dòng vẫn tô cam</t>
+        </is>
+      </c>
+      <c r="J112" s="15" t="inlineStr"/>
+      <c r="K112" s="16" t="inlineStr">
+        <is>
+          <t>Not Executed</t>
+        </is>
+      </c>
+      <c r="L112" s="16" t="inlineStr">
+        <is>
+          <t>Not Executed</t>
+        </is>
+      </c>
+      <c r="M112" s="16" t="inlineStr">
+        <is>
+          <t>Not Executed</t>
+        </is>
+      </c>
+      <c r="N112" s="15" t="inlineStr"/>
+      <c r="O112" s="16" t="inlineStr"/>
+      <c r="P112" s="16" t="inlineStr"/>
+      <c r="Q112" s="16" t="inlineStr"/>
+    </row>
+    <row r="113" ht="34" customHeight="1">
+      <c r="A113" s="15" t="inlineStr">
+        <is>
+          <t>Hạn xử lý nhu cầu KH</t>
+        </is>
+      </c>
+      <c r="B113" s="15" t="inlineStr">
+        <is>
+          <t>CÔ LẬP DỮ LIỆU &amp; THAO TÁC ĐỒNG THỜI</t>
+        </is>
+      </c>
+      <c r="C113" s="16" t="inlineStr">
+        <is>
+          <t>TC_09.004</t>
+        </is>
+      </c>
+      <c r="D113" s="15" t="inlineStr">
+        <is>
+          <t>Người dùng lập dự án ngay trước giờ quét</t>
+        </is>
+      </c>
+      <c r="E113" s="16" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="F113" s="15" t="inlineStr">
+        <is>
+          <t>Nhu cầu #434 hết hạn hôm nay; người dùng lập Dự án TKT từ nhu cầu này lúc 23:50.</t>
+        </is>
+      </c>
+      <c r="G113" s="15" t="inlineStr">
+        <is>
+          <t>1. Chạy lệnh quét hạn nhu cầu sau đó
+2. Kiểm tra #434</t>
+        </is>
+      </c>
+      <c r="H113" s="15" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I113" s="15" t="inlineStr">
+        <is>
+          <t>- Không bị đóng, trạng thái là 'Đã lập dự án TKT'</t>
+        </is>
+      </c>
+      <c r="J113" s="15" t="inlineStr"/>
+      <c r="K113" s="16" t="inlineStr">
+        <is>
+          <t>Not Executed</t>
+        </is>
+      </c>
+      <c r="L113" s="16" t="inlineStr">
+        <is>
+          <t>Not Executed</t>
+        </is>
+      </c>
+      <c r="M113" s="16" t="inlineStr">
+        <is>
+          <t>Not Executed</t>
+        </is>
+      </c>
+      <c r="N113" s="15" t="inlineStr"/>
+      <c r="O113" s="16" t="inlineStr"/>
+      <c r="P113" s="16" t="inlineStr"/>
+      <c r="Q113" s="16" t="inlineStr"/>
+    </row>
+    <row r="114" ht="34" customHeight="1">
+      <c r="A114" s="15" t="inlineStr">
+        <is>
+          <t>Hạn xử lý nhu cầu KH</t>
+        </is>
+      </c>
+      <c r="B114" s="15" t="inlineStr">
+        <is>
+          <t>CÔ LẬP DỮ LIỆU &amp; THAO TÁC ĐỒNG THỜI</t>
+        </is>
+      </c>
+      <c r="C114" s="16" t="inlineStr">
+        <is>
+          <t>TC_09.005</t>
+        </is>
+      </c>
+      <c r="D114" s="15" t="inlineStr">
+        <is>
+          <t>Hai người cùng thao tác trên một nhu cầu</t>
+        </is>
+      </c>
+      <c r="E114" s="16" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="F114" s="15" t="inlineStr">
+        <is>
+          <t>Người 1 đang mở form lập dự án từ nhu cầu #435; người 2 đóng tay nhu cầu đó.</t>
+        </is>
+      </c>
+      <c r="G114" s="15" t="inlineStr">
+        <is>
+          <t>1. Người 1 bấm Lưu form lập dự án</t>
+        </is>
+      </c>
+      <c r="H114" s="15" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I114" s="15" t="inlineStr">
+        <is>
+          <t>- Bị chặn kèm thông báo nhu cầu đã đóng, không tạo dự án
+- Màn không treo</t>
+        </is>
+      </c>
+      <c r="J114" s="15" t="inlineStr"/>
+      <c r="K114" s="16" t="inlineStr">
+        <is>
+          <t>Not Executed</t>
+        </is>
+      </c>
+      <c r="L114" s="16" t="inlineStr">
+        <is>
+          <t>Not Executed</t>
+        </is>
+      </c>
+      <c r="M114" s="16" t="inlineStr">
+        <is>
+          <t>Not Executed</t>
+        </is>
+      </c>
+      <c r="N114" s="15" t="inlineStr"/>
+      <c r="O114" s="16" t="inlineStr"/>
+      <c r="P114" s="16" t="inlineStr"/>
+      <c r="Q114" s="16" t="inlineStr"/>
+    </row>
+    <row r="115" ht="34" customHeight="1">
+      <c r="A115" s="15" t="inlineStr">
+        <is>
+          <t>Hạn xử lý nhu cầu KH</t>
+        </is>
+      </c>
+      <c r="B115" s="15" t="inlineStr">
+        <is>
+          <t>CÔ LẬP DỮ LIỆU &amp; THAO TÁC ĐỒNG THỜI</t>
+        </is>
+      </c>
+      <c r="C115" s="16" t="inlineStr">
+        <is>
+          <t>TC_09.006</t>
+        </is>
+      </c>
+      <c r="D115" s="15" t="inlineStr">
+        <is>
+          <t>Quét chạy khi hệ thống chưa có cấu hình M</t>
+        </is>
+      </c>
+      <c r="E115" s="16" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="F115" s="15" t="inlineStr">
+        <is>
+          <t>Công ty của cuộc họp chưa từng lưu cấu hình hạn.</t>
+        </is>
+      </c>
+      <c r="G115" s="15" t="inlineStr">
+        <is>
+          <t>1. Chạy lệnh quét hạn nhu cầu với 1 nhu cầu còn 2 ngày tới hạn (N = 30)</t>
+        </is>
+      </c>
+      <c r="H115" s="15" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I115" s="15" t="inlineStr">
+        <is>
+          <t>- Hệ thống dùng mặc định 3 ngày: nhu cầu vẫn được cảnh báo
+- Không văng lỗi vì thiếu cấu hình</t>
+        </is>
+      </c>
+      <c r="J115" s="15" t="inlineStr"/>
+      <c r="K115" s="16" t="inlineStr">
+        <is>
+          <t>Not Executed</t>
+        </is>
+      </c>
+      <c r="L115" s="16" t="inlineStr">
+        <is>
+          <t>Not Executed</t>
+        </is>
+      </c>
+      <c r="M115" s="16" t="inlineStr">
+        <is>
+          <t>Not Executed</t>
+        </is>
+      </c>
+      <c r="N115" s="15" t="inlineStr"/>
+      <c r="O115" s="16" t="inlineStr"/>
+      <c r="P115" s="16" t="inlineStr"/>
+      <c r="Q115" s="16" t="inlineStr"/>
+    </row>
+    <row r="116" ht="34" customHeight="1">
+      <c r="A116" s="15" t="inlineStr">
+        <is>
+          <t>Hạn xử lý nhu cầu KH</t>
+        </is>
+      </c>
+      <c r="B116" s="15" t="inlineStr">
+        <is>
+          <t>CÔ LẬP DỮ LIỆU &amp; THAO TÁC ĐỒNG THỜI</t>
+        </is>
+      </c>
+      <c r="C116" s="16" t="inlineStr">
+        <is>
+          <t>TC_09.007</t>
+        </is>
+      </c>
+      <c r="D116" s="15" t="inlineStr">
+        <is>
+          <t>Cuộc họp bị xoá hoặc thiếu người chủ trì</t>
+        </is>
+      </c>
+      <c r="E116" s="16" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="F116" s="15" t="inlineStr">
+        <is>
+          <t>Nhu cầu #436 tới vùng cảnh báo nhưng cuộc họp không xác định được người chủ trì lẫn người tạo.</t>
+        </is>
+      </c>
+      <c r="G116" s="15" t="inlineStr">
+        <is>
+          <t>1. Chạy lệnh quét hạn nhu cầu</t>
+        </is>
+      </c>
+      <c r="H116" s="15" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I116" s="15" t="inlineStr">
+        <is>
+          <t>- Không gửi được thông báo nhưng lệnh vẫn chạy hết, các nhu cầu khác vẫn được xử lý bình thường</t>
+        </is>
+      </c>
+      <c r="J116" s="15" t="inlineStr"/>
+      <c r="K116" s="16" t="inlineStr">
+        <is>
+          <t>Not Executed</t>
+        </is>
+      </c>
+      <c r="L116" s="16" t="inlineStr">
+        <is>
+          <t>Not Executed</t>
+        </is>
+      </c>
+      <c r="M116" s="16" t="inlineStr">
+        <is>
+          <t>Not Executed</t>
+        </is>
+      </c>
+      <c r="N116" s="15" t="inlineStr"/>
+      <c r="O116" s="16" t="inlineStr"/>
+      <c r="P116" s="16" t="inlineStr"/>
+      <c r="Q116" s="16" t="inlineStr"/>
+    </row>
+    <row r="117" ht="26" customHeight="1">
+      <c r="A117" s="13" t="n"/>
+      <c r="B117" s="13" t="n"/>
+      <c r="C117" s="14" t="inlineStr">
         <is>
           <t>X. E2E FLOW</t>
         </is>
       </c>
-      <c r="D112" s="4" t="n"/>
-      <c r="E112" s="4" t="n"/>
-      <c r="F112" s="4" t="n"/>
-      <c r="G112" s="4" t="n"/>
-      <c r="H112" s="4" t="n"/>
-      <c r="I112" s="4" t="n"/>
-      <c r="J112" s="4" t="n"/>
-      <c r="K112" s="4" t="n"/>
-      <c r="L112" s="4" t="n"/>
-      <c r="M112" s="4" t="n"/>
-      <c r="N112" s="4" t="n"/>
-      <c r="O112" s="4" t="n"/>
-      <c r="P112" s="4" t="n"/>
-      <c r="Q112" s="5" t="n"/>
-    </row>
-    <row r="113" ht="87" customHeight="1">
-      <c r="A113" s="15" t="inlineStr">
-        <is>
-          <t>Hạn xử lý nhu cầu KH</t>
-        </is>
-      </c>
-      <c r="B113" s="15" t="inlineStr">
+      <c r="D117" s="4" t="n"/>
+      <c r="E117" s="4" t="n"/>
+      <c r="F117" s="4" t="n"/>
+      <c r="G117" s="4" t="n"/>
+      <c r="H117" s="4" t="n"/>
+      <c r="I117" s="4" t="n"/>
+      <c r="J117" s="4" t="n"/>
+      <c r="K117" s="4" t="n"/>
+      <c r="L117" s="4" t="n"/>
+      <c r="M117" s="4" t="n"/>
+      <c r="N117" s="4" t="n"/>
+      <c r="O117" s="4" t="n"/>
+      <c r="P117" s="4" t="n"/>
+      <c r="Q117" s="5" t="n"/>
+    </row>
+    <row r="118" ht="87" customHeight="1">
+      <c r="A118" s="15" t="inlineStr">
+        <is>
+          <t>Hạn xử lý nhu cầu KH</t>
+        </is>
+      </c>
+      <c r="B118" s="15" t="inlineStr">
         <is>
           <t>E2E FLOW</t>
         </is>
       </c>
-      <c r="C113" s="16" t="inlineStr">
+      <c r="C118" s="16" t="inlineStr">
         <is>
           <t>TC_10.001</t>
         </is>
       </c>
-      <c r="D113" s="15" t="inlineStr">
-        <is>
-          <t>Luồng đầy đủ: khai N và M → cảnh báo → tự đóng → chặn lập dự án</t>
-        </is>
-      </c>
-      <c r="E113" s="16" t="inlineStr">
+      <c r="D118" s="15" t="inlineStr">
+        <is>
+          <t>Luồng đầy đủ: khai N và M -&gt; cảnh báo -&gt; tự đóng -&gt; chặn lập dự án</t>
+        </is>
+      </c>
+      <c r="E118" s="16" t="inlineStr">
         <is>
           <t>P0</t>
         </is>
       </c>
-      <c r="F113" s="15" t="inlineStr">
+      <c r="F118" s="15" t="inlineStr">
         <is>
           <t>Lĩnh vực LVCTKD.E2E đang N = 0; cuộc họp M-E2E có 1 nhu cầu, chưa Hoàn thành; M = 3.</t>
         </is>
       </c>
-      <c r="G113" s="15" t="inlineStr">
+      <c r="G118" s="15" t="inlineStr">
         <is>
           <t>1. Khai N = 5 cho lĩnh vực LVCTKD.E2E
 2. Chuyển cuộc họp M-E2E sang Hoàn thành
@@ -7136,12 +7485,12 @@
 6. Thử lập Dự án TKT từ nhu cầu đó</t>
         </is>
       </c>
-      <c r="H113" s="15" t="inlineStr">
+      <c r="H118" s="15" t="inlineStr">
         <is>
           <t>Thời gian hiệu lực nhu cầu: 5 · Cảnh báo trước khi đóng: 3</t>
         </is>
       </c>
-      <c r="I113" s="15" t="inlineStr">
+      <c r="I118" s="15" t="inlineStr">
         <is>
           <t>- Bước 3: cột hạn = ngày Hoàn thành + 5 ngày
 - Bước 4: người chủ trì nhận 1 thông báo, dòng tô cam '(còn 3 ngày)'
@@ -7149,59 +7498,59 @@
 - Bước 6: không còn nút Tạo Dự án TKT; gọi thẳng chức năng thì bị chặn đúng câu thông báo</t>
         </is>
       </c>
-      <c r="J113" s="15" t="inlineStr"/>
-      <c r="K113" s="16" t="inlineStr">
-        <is>
-          <t>Not Executed</t>
-        </is>
-      </c>
-      <c r="L113" s="16" t="inlineStr">
-        <is>
-          <t>Not Executed</t>
-        </is>
-      </c>
-      <c r="M113" s="16" t="inlineStr">
-        <is>
-          <t>Not Executed</t>
-        </is>
-      </c>
-      <c r="N113" s="15" t="inlineStr"/>
-      <c r="O113" s="16" t="inlineStr"/>
-      <c r="P113" s="16" t="inlineStr"/>
-      <c r="Q113" s="16" t="inlineStr"/>
-    </row>
-    <row r="114" ht="47" customHeight="1">
-      <c r="A114" s="15" t="inlineStr">
-        <is>
-          <t>Hạn xử lý nhu cầu KH</t>
-        </is>
-      </c>
-      <c r="B114" s="15" t="inlineStr">
+      <c r="J118" s="15" t="inlineStr"/>
+      <c r="K118" s="16" t="inlineStr">
+        <is>
+          <t>Not Executed</t>
+        </is>
+      </c>
+      <c r="L118" s="16" t="inlineStr">
+        <is>
+          <t>Not Executed</t>
+        </is>
+      </c>
+      <c r="M118" s="16" t="inlineStr">
+        <is>
+          <t>Not Executed</t>
+        </is>
+      </c>
+      <c r="N118" s="15" t="inlineStr"/>
+      <c r="O118" s="16" t="inlineStr"/>
+      <c r="P118" s="16" t="inlineStr"/>
+      <c r="Q118" s="16" t="inlineStr"/>
+    </row>
+    <row r="119" ht="47" customHeight="1">
+      <c r="A119" s="15" t="inlineStr">
+        <is>
+          <t>Hạn xử lý nhu cầu KH</t>
+        </is>
+      </c>
+      <c r="B119" s="15" t="inlineStr">
         <is>
           <t>E2E FLOW</t>
         </is>
       </c>
-      <c r="C114" s="16" t="inlineStr">
+      <c r="C119" s="16" t="inlineStr">
         <is>
           <t>TC_10.002</t>
         </is>
       </c>
-      <c r="D114" s="15" t="inlineStr">
+      <c r="D119" s="15" t="inlineStr">
         <is>
           <t>Luồng lập dự án kịp hạn</t>
         </is>
       </c>
-      <c r="E114" s="16" t="inlineStr">
+      <c r="E119" s="16" t="inlineStr">
         <is>
           <t>P0</t>
         </is>
       </c>
-      <c r="F114" s="15" t="inlineStr">
+      <c r="F119" s="15" t="inlineStr">
         <is>
           <t>Nhu cầu #501 còn 2 ngày tới hạn, đã nhận cảnh báo.</t>
         </is>
       </c>
-      <c r="G114" s="15" t="inlineStr">
+      <c r="G119" s="15" t="inlineStr">
         <is>
           <t>1. Bấm nút Tạo Dự án TKT từ nhu cầu #501
 2. Lập dự án và lưu
@@ -7209,184 +7558,185 @@
 4. Chạy lệnh quét hạn nhu cầu sau ngày hết hạn</t>
         </is>
       </c>
-      <c r="H114" s="15" t="inlineStr">
+      <c r="H119" s="15" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="I114" s="15" t="inlineStr">
-        <is>
-          <t>- Sau bước 2: nhu cầu chuyển 'Đã lập dự án TKT', cột hạn thành 'Không thời hạn'
+      <c r="I119" s="15" t="inlineStr">
+        <is>
+          <t>- Sau bước 2: nhu cầu chuyển 'Đã lập dự án TKT', cột hạn thành 'Không giới hạn thời gian hiệu lực'
 - Sau bước 4: nhu cầu KHÔNG bị đóng</t>
         </is>
       </c>
-      <c r="J114" s="15" t="inlineStr"/>
-      <c r="K114" s="16" t="inlineStr">
-        <is>
-          <t>Not Executed</t>
-        </is>
-      </c>
-      <c r="L114" s="16" t="inlineStr">
-        <is>
-          <t>Not Executed</t>
-        </is>
-      </c>
-      <c r="M114" s="16" t="inlineStr">
-        <is>
-          <t>Not Executed</t>
-        </is>
-      </c>
-      <c r="N114" s="15" t="inlineStr"/>
-      <c r="O114" s="16" t="inlineStr"/>
-      <c r="P114" s="16" t="inlineStr"/>
-      <c r="Q114" s="16" t="inlineStr"/>
-    </row>
-    <row r="115" ht="34" customHeight="1">
-      <c r="A115" s="15" t="inlineStr">
-        <is>
-          <t>Hạn xử lý nhu cầu KH</t>
-        </is>
-      </c>
-      <c r="B115" s="15" t="inlineStr">
+      <c r="J119" s="15" t="inlineStr"/>
+      <c r="K119" s="16" t="inlineStr">
+        <is>
+          <t>Not Executed</t>
+        </is>
+      </c>
+      <c r="L119" s="16" t="inlineStr">
+        <is>
+          <t>Not Executed</t>
+        </is>
+      </c>
+      <c r="M119" s="16" t="inlineStr">
+        <is>
+          <t>Not Executed</t>
+        </is>
+      </c>
+      <c r="N119" s="15" t="inlineStr"/>
+      <c r="O119" s="16" t="inlineStr"/>
+      <c r="P119" s="16" t="inlineStr"/>
+      <c r="Q119" s="16" t="inlineStr"/>
+    </row>
+    <row r="120" ht="38" customHeight="1">
+      <c r="A120" s="15" t="inlineStr">
+        <is>
+          <t>Hạn xử lý nhu cầu KH</t>
+        </is>
+      </c>
+      <c r="B120" s="15" t="inlineStr">
         <is>
           <t>E2E FLOW</t>
         </is>
       </c>
-      <c r="C115" s="16" t="inlineStr">
+      <c r="C120" s="16" t="inlineStr">
         <is>
           <t>TC_10.003</t>
         </is>
       </c>
-      <c r="D115" s="15" t="inlineStr">
+      <c r="D120" s="15" t="inlineStr">
         <is>
           <t>Luồng lĩnh vực không đặt thời hạn</t>
         </is>
       </c>
-      <c r="E115" s="16" t="inlineStr">
+      <c r="E120" s="16" t="inlineStr">
         <is>
           <t>P1</t>
         </is>
       </c>
-      <c r="F115" s="15" t="inlineStr">
+      <c r="F120" s="15" t="inlineStr">
         <is>
           <t>Lĩnh vực LVCTKD.KHAC để N = 0, có 10 nhu cầu cũ từ nhiều tháng trước.</t>
         </is>
       </c>
-      <c r="G115" s="15" t="inlineStr">
+      <c r="G120" s="15" t="inlineStr">
         <is>
           <t>1. Chạy lệnh quét hạn nhu cầu
 2. Xem 10 nhu cầu đó trên màn danh sách</t>
         </is>
       </c>
-      <c r="H115" s="15" t="inlineStr">
+      <c r="H120" s="15" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="I115" s="15" t="inlineStr">
+      <c r="I120" s="15" t="inlineStr">
         <is>
           <t>- Không nhu cầu nào bị đóng, không thông báo nào được gửi
-- Cả 10 dòng đều ghi 'Không thời hạn'</t>
-        </is>
-      </c>
-      <c r="J115" s="15" t="inlineStr"/>
-      <c r="K115" s="16" t="inlineStr">
-        <is>
-          <t>Not Executed</t>
-        </is>
-      </c>
-      <c r="L115" s="16" t="inlineStr">
-        <is>
-          <t>Not Executed</t>
-        </is>
-      </c>
-      <c r="M115" s="16" t="inlineStr">
-        <is>
-          <t>Not Executed</t>
-        </is>
-      </c>
-      <c r="N115" s="15" t="inlineStr"/>
-      <c r="O115" s="16" t="inlineStr"/>
-      <c r="P115" s="16" t="inlineStr"/>
-      <c r="Q115" s="16" t="inlineStr"/>
-    </row>
-    <row r="116" ht="49" customHeight="1">
-      <c r="A116" s="15" t="inlineStr">
-        <is>
-          <t>Hạn xử lý nhu cầu KH</t>
-        </is>
-      </c>
-      <c r="B116" s="15" t="inlineStr">
+- Cả 10 dòng đều ghi 'Không giới hạn thời gian hiệu lực'</t>
+        </is>
+      </c>
+      <c r="J120" s="15" t="inlineStr"/>
+      <c r="K120" s="16" t="inlineStr">
+        <is>
+          <t>Not Executed</t>
+        </is>
+      </c>
+      <c r="L120" s="16" t="inlineStr">
+        <is>
+          <t>Not Executed</t>
+        </is>
+      </c>
+      <c r="M120" s="16" t="inlineStr">
+        <is>
+          <t>Not Executed</t>
+        </is>
+      </c>
+      <c r="N120" s="15" t="inlineStr"/>
+      <c r="O120" s="16" t="inlineStr"/>
+      <c r="P120" s="16" t="inlineStr"/>
+      <c r="Q120" s="16" t="inlineStr"/>
+    </row>
+    <row r="121" ht="49" customHeight="1">
+      <c r="A121" s="15" t="inlineStr">
+        <is>
+          <t>Hạn xử lý nhu cầu KH</t>
+        </is>
+      </c>
+      <c r="B121" s="15" t="inlineStr">
         <is>
           <t>E2E FLOW</t>
         </is>
       </c>
-      <c r="C116" s="16" t="inlineStr">
+      <c r="C121" s="16" t="inlineStr">
         <is>
           <t>TC_10.004</t>
         </is>
       </c>
-      <c r="D116" s="15" t="inlineStr">
+      <c r="D121" s="15" t="inlineStr">
         <is>
           <t>Luồng hai lĩnh vực hạn khác nhau trong cùng cuộc họp</t>
         </is>
       </c>
-      <c r="E116" s="16" t="inlineStr">
+      <c r="E121" s="16" t="inlineStr">
         <is>
           <t>P1</t>
         </is>
       </c>
-      <c r="F116" s="15" t="inlineStr">
+      <c r="F121" s="15" t="inlineStr">
         <is>
           <t>Cuộc họp M-E2E2 Hoàn thành 01/09/2026, phát sinh 2 nhu cầu: một thuộc lĩnh vực N = 10, một thuộc lĩnh vực N = 40.</t>
         </is>
       </c>
-      <c r="G116" s="15" t="inlineStr">
+      <c r="G121" s="15" t="inlineStr">
         <is>
           <t>1. Xem cột hạn của 2 nhu cầu
 2. Chạy lệnh quét hạn nhu cầu vào ngày 11/09/2026</t>
         </is>
       </c>
-      <c r="H116" s="15" t="inlineStr">
+      <c r="H121" s="15" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="I116" s="15" t="inlineStr">
+      <c r="I121" s="15" t="inlineStr">
         <is>
           <t>- Nhu cầu thứ nhất hạn 11/09/2026, nhu cầu thứ hai hạn 11/10/2026
 - Lần quét ngày 11/09 chỉ đóng nhu cầu thứ nhất, nhu cầu thứ hai vẫn Đang theo dõi</t>
         </is>
       </c>
-      <c r="J116" s="15" t="inlineStr"/>
-      <c r="K116" s="16" t="inlineStr">
-        <is>
-          <t>Not Executed</t>
-        </is>
-      </c>
-      <c r="L116" s="16" t="inlineStr">
-        <is>
-          <t>Not Executed</t>
-        </is>
-      </c>
-      <c r="M116" s="16" t="inlineStr">
-        <is>
-          <t>Not Executed</t>
-        </is>
-      </c>
-      <c r="N116" s="15" t="inlineStr"/>
-      <c r="O116" s="16" t="inlineStr"/>
-      <c r="P116" s="16" t="inlineStr"/>
-      <c r="Q116" s="16" t="inlineStr"/>
+      <c r="J121" s="15" t="inlineStr"/>
+      <c r="K121" s="16" t="inlineStr">
+        <is>
+          <t>Not Executed</t>
+        </is>
+      </c>
+      <c r="L121" s="16" t="inlineStr">
+        <is>
+          <t>Not Executed</t>
+        </is>
+      </c>
+      <c r="M121" s="16" t="inlineStr">
+        <is>
+          <t>Not Executed</t>
+        </is>
+      </c>
+      <c r="N121" s="15" t="inlineStr"/>
+      <c r="O121" s="16" t="inlineStr"/>
+      <c r="P121" s="16" t="inlineStr"/>
+      <c r="Q121" s="16" t="inlineStr"/>
     </row>
   </sheetData>
   <mergeCells count="43">
+    <mergeCell ref="C109:Q109"/>
     <mergeCell ref="B9:N9"/>
     <mergeCell ref="I15:J15"/>
-    <mergeCell ref="C112:Q112"/>
     <mergeCell ref="K15:L15"/>
     <mergeCell ref="A11:E11"/>
     <mergeCell ref="I11:J11"/>
+    <mergeCell ref="C117:Q117"/>
     <mergeCell ref="B6:N6"/>
     <mergeCell ref="A1:N1"/>
     <mergeCell ref="B5:N5"/>
@@ -7419,17 +7769,16 @@
     <mergeCell ref="C58:Q58"/>
     <mergeCell ref="M14:N14"/>
     <mergeCell ref="C98:Q98"/>
-    <mergeCell ref="C104:Q104"/>
     <mergeCell ref="I13:J13"/>
     <mergeCell ref="F11:H15"/>
     <mergeCell ref="K13:L13"/>
     <mergeCell ref="B10:N10"/>
   </mergeCells>
   <dataValidations count="2">
-    <dataValidation sqref="K18:M166" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="K18:M171" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Passed,Failed,Pending,Not Executed"</formula1>
     </dataValidation>
-    <dataValidation sqref="O18:Q166" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="O18:Q171" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"P,F,PE"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>

<commit_message>
docs(11377): sinh lai testcase.xlsx (94 TC / 122 dong)
Ban .xlsx tuong ung voi gen_testcase.py o commit b264cd3 (truoc do chua ghi
duoc vi file dang bi Excel khoa).

Refs #11377

Co-Authored-By: Claude Opus 5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/hrm/.plans/canh-bao-tu-dong-dong-nhu-cau/testcase.xlsx
+++ b/hrm/.plans/canh-bao-tu-dong-dong-nhu-cau/testcase.xlsx
@@ -567,7 +567,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q121"/>
+  <dimension ref="A1:Q122"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26.9" customWidth="1" min="1" max="1"/>
@@ -817,7 +817,7 @@
       <c r="M9" s="4" t="n"/>
       <c r="N9" s="5" t="n"/>
     </row>
-    <row r="10" ht="151" customHeight="1">
+    <row r="10" ht="185" customHeight="1">
       <c r="A10" s="2" t="inlineStr">
         <is>
           <t>9. Ghi chú đọc bảng</t>
@@ -828,6 +828,8 @@
           <t>Bẫy dễ sai nhất của đợt này:
 - N = 0 nghĩa là KHÔNG đặt thời hạn, không phải 'hết hạn ngay'. Mặc định sau khi lên bản mới, mọi lĩnh vực đều là 0, tức chưa nhu cầu nào bị đóng cho tới khi người quản trị khai N.
 - N &lt;= M thì KHÔNG có bước cảnh báo, nhu cầu vẫn bị đóng đúng hạn. Đừng báo lỗi 'thiếu thông báo'.
+- MỌI testcase kỳ vọng CÓ cảnh báo đều đã chốt sẵn N &gt; M trong cột Điều kiện. Khi test trên dữ liệu thật, phải kiểm N của lĩnh vực trước: N &lt;= M mà không thấy cảnh báo là ĐÚNG, không phải lỗi.
+- Nâng M lên KHÔNG phải lúc nào cũng làm nhiều nhu cầu được cảnh báo hơn: M vượt quá N của lĩnh vực nào thì nhu cầu của lĩnh vực đó MẤT cảnh báo.
 - Nhu cầu quá hạn vẫn nằm trong danh sách cho tới lần quét kế tiếp (01:20 hôm sau) mới chuyển sang Đóng — trong khoảng đó cột hạn hiện '(quá hạn X ngày)' là đúng.
 - Ngày đóng là ngày HẾT HẠN chứ không phải ngày chạy quét.
 - Sửa N ở danh mục làm hạn của mọi nhu cầu thuộc lĩnh vực đó đổi ngay, kể cả nhu cầu cũ.
@@ -2964,7 +2966,7 @@
       </c>
       <c r="F47" s="15" t="inlineStr">
         <is>
-          <t>M đang là 3. Có nhu cầu #101 hết hạn sau 2 ngày nữa.</t>
+          <t>M đang là 3. Có nhu cầu #101 thuộc lĩnh vực N = 30, hết hạn sau 2 ngày nữa.</t>
         </is>
       </c>
       <c r="G47" s="15" t="inlineStr">
@@ -3836,7 +3838,7 @@
       </c>
       <c r="F61" s="15" t="inlineStr">
         <is>
-          <t>M = 3. Nhu cầu #102 hết hạn 17/09/2026, hôm nay 15/09/2026.</t>
+          <t>M = 3, lĩnh vực của nhu cầu #102 có N = 30. Nhu cầu #102 hết hạn 17/09/2026, hôm nay 15/09/2026.</t>
         </is>
       </c>
       <c r="G61" s="15" t="inlineStr">
@@ -3904,7 +3906,7 @@
       </c>
       <c r="F62" s="15" t="inlineStr">
         <is>
-          <t>M = 3. Nhu cầu #103 hết hạn đúng hôm nay.</t>
+          <t>M = 3, lĩnh vực của nhu cầu #103 có N = 30. Nhu cầu #103 hết hạn đúng hôm nay.</t>
         </is>
       </c>
       <c r="G62" s="15" t="inlineStr">
@@ -3943,7 +3945,7 @@
       <c r="P62" s="16" t="inlineStr"/>
       <c r="Q62" s="16" t="inlineStr"/>
     </row>
-    <row r="63" ht="34" customHeight="1">
+    <row r="63" ht="41" customHeight="1">
       <c r="A63" s="15" t="inlineStr">
         <is>
           <t>Hạn xử lý nhu cầu KH</t>
@@ -3971,7 +3973,7 @@
       </c>
       <c r="F63" s="15" t="inlineStr">
         <is>
-          <t>Nhu cầu #104 hết hạn 12/09/2026, hôm nay 15/09/2026, lần quét gần nhất chưa chạy.</t>
+          <t>M = 3, lĩnh vực của nhu cầu #104 có N = 30. Nhu cầu #104 hết hạn 12/09/2026, hôm nay 15/09/2026, lần quét gần nhất chưa chạy.</t>
         </is>
       </c>
       <c r="G63" s="15" t="inlineStr">
@@ -4242,7 +4244,7 @@
       </c>
       <c r="F67" s="15" t="inlineStr">
         <is>
-          <t>Tài khoản đang phụ trách ít nhất 1 nhu cầu sắp hết hạn.</t>
+          <t>Tài khoản đang phụ trách ít nhất 1 nhu cầu sắp hết hạn, thuộc lĩnh vực có N = 30 (M = 3).</t>
         </is>
       </c>
       <c r="G67" s="15" t="inlineStr">
@@ -4352,7 +4354,7 @@
       <c r="P68" s="16" t="inlineStr"/>
       <c r="Q68" s="16" t="inlineStr"/>
     </row>
-    <row r="69" ht="34" customHeight="1">
+    <row r="69" ht="61" customHeight="1">
       <c r="A69" s="15" t="inlineStr">
         <is>
           <t>Hạn xử lý nhu cầu KH</t>
@@ -4380,7 +4382,7 @@
       </c>
       <c r="F69" s="15" t="inlineStr">
         <is>
-          <t>M = 3, nhu cầu #108 hết hạn sau 5 ngày nữa (chưa tô cam).</t>
+          <t>M = 3, nhu cầu #108 thuộc lĩnh vực có N = 30, hết hạn sau 5 ngày nữa (chưa tô cam).</t>
         </is>
       </c>
       <c r="G69" s="15" t="inlineStr">
@@ -4396,7 +4398,8 @@
       </c>
       <c r="I69" s="15" t="inlineStr">
         <is>
-          <t>- Dòng #108 chuyển sang tô cam kèm '(còn 5 ngày)'</t>
+          <t>- Dòng #108 chuyển sang tô cam kèm '(còn 5 ngày)'
+- LƯU Ý: kết quả này chỉ đúng vì N = 30 vẫn LỚN HƠN M = 7. Nâng M vượt quá N thì cảnh báo TẮT đi chứ không bật thêm — xem TC ngay dưới</t>
         </is>
       </c>
       <c r="J69" s="15" t="inlineStr"/>
@@ -4420,146 +4423,147 @@
       <c r="P69" s="16" t="inlineStr"/>
       <c r="Q69" s="16" t="inlineStr"/>
     </row>
-    <row r="70" ht="26" customHeight="1">
-      <c r="A70" s="13" t="n"/>
-      <c r="B70" s="13" t="n"/>
-      <c r="C70" s="14" t="inlineStr">
+    <row r="70" ht="75" customHeight="1">
+      <c r="A70" s="15" t="inlineStr">
+        <is>
+          <t>Hạn xử lý nhu cầu KH</t>
+        </is>
+      </c>
+      <c r="B70" s="15" t="inlineStr">
+        <is>
+          <t>HIỂN THỊ HẠN Ở MÀN NHU CẦU KHÁCH HÀNG</t>
+        </is>
+      </c>
+      <c r="C70" s="16" t="inlineStr">
+        <is>
+          <t>TC_04.012</t>
+        </is>
+      </c>
+      <c r="D70" s="15" t="inlineStr">
+        <is>
+          <t>Nâng M vượt quá N thì cảnh báo TẮT đi</t>
+        </is>
+      </c>
+      <c r="E70" s="16" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="F70" s="15" t="inlineStr">
+        <is>
+          <t>M = 3, nhu cầu #109 thuộc lĩnh vực có N = 5, đang tô cam vì còn 2 ngày.</t>
+        </is>
+      </c>
+      <c r="G70" s="15" t="inlineStr">
+        <is>
+          <t>1. Đổi M thành 7 ở Cấu hình chung, lưu
+2. Quay lại màn Nhu cầu khách hàng, tải lại</t>
+        </is>
+      </c>
+      <c r="H70" s="15" t="inlineStr">
+        <is>
+          <t>Cảnh báo trước khi đóng nhu cầu: 3 -&gt; 7</t>
+        </is>
+      </c>
+      <c r="I70" s="15" t="inlineStr">
+        <is>
+          <t>- Dòng #109 HẾT tô cam, hết ghi chú số ngày, chỉ còn ngày hết hạn
+- LƯU Ý: đây là ĐÚNG yêu cầu, không phải lỗi. N = 5 nay nhỏ hơn M = 7 nên rơi vào ngoại lệ 'N &lt;= M thì bỏ qua cảnh báo'
+- Nhu cầu vẫn bị đóng đúng hạn như thường</t>
+        </is>
+      </c>
+      <c r="J70" s="15" t="inlineStr"/>
+      <c r="K70" s="16" t="inlineStr">
+        <is>
+          <t>Not Executed</t>
+        </is>
+      </c>
+      <c r="L70" s="16" t="inlineStr">
+        <is>
+          <t>Not Executed</t>
+        </is>
+      </c>
+      <c r="M70" s="16" t="inlineStr">
+        <is>
+          <t>Not Executed</t>
+        </is>
+      </c>
+      <c r="N70" s="15" t="inlineStr"/>
+      <c r="O70" s="16" t="inlineStr"/>
+      <c r="P70" s="16" t="inlineStr"/>
+      <c r="Q70" s="16" t="inlineStr"/>
+    </row>
+    <row r="71" ht="26" customHeight="1">
+      <c r="A71" s="13" t="n"/>
+      <c r="B71" s="13" t="n"/>
+      <c r="C71" s="14" t="inlineStr">
         <is>
           <t>V. CẢNH BÁO TRƯỚC HẠN</t>
         </is>
       </c>
-      <c r="D70" s="4" t="n"/>
-      <c r="E70" s="4" t="n"/>
-      <c r="F70" s="4" t="n"/>
-      <c r="G70" s="4" t="n"/>
-      <c r="H70" s="4" t="n"/>
-      <c r="I70" s="4" t="n"/>
-      <c r="J70" s="4" t="n"/>
-      <c r="K70" s="4" t="n"/>
-      <c r="L70" s="4" t="n"/>
-      <c r="M70" s="4" t="n"/>
-      <c r="N70" s="4" t="n"/>
-      <c r="O70" s="4" t="n"/>
-      <c r="P70" s="4" t="n"/>
-      <c r="Q70" s="5" t="n"/>
-    </row>
-    <row r="71" ht="87" customHeight="1">
-      <c r="A71" s="15" t="inlineStr">
-        <is>
-          <t>Hạn xử lý nhu cầu KH</t>
-        </is>
-      </c>
-      <c r="B71" s="15" t="inlineStr">
+      <c r="D71" s="4" t="n"/>
+      <c r="E71" s="4" t="n"/>
+      <c r="F71" s="4" t="n"/>
+      <c r="G71" s="4" t="n"/>
+      <c r="H71" s="4" t="n"/>
+      <c r="I71" s="4" t="n"/>
+      <c r="J71" s="4" t="n"/>
+      <c r="K71" s="4" t="n"/>
+      <c r="L71" s="4" t="n"/>
+      <c r="M71" s="4" t="n"/>
+      <c r="N71" s="4" t="n"/>
+      <c r="O71" s="4" t="n"/>
+      <c r="P71" s="4" t="n"/>
+      <c r="Q71" s="5" t="n"/>
+    </row>
+    <row r="72" ht="87" customHeight="1">
+      <c r="A72" s="15" t="inlineStr">
+        <is>
+          <t>Hạn xử lý nhu cầu KH</t>
+        </is>
+      </c>
+      <c r="B72" s="15" t="inlineStr">
         <is>
           <t>CẢNH BÁO TRƯỚC HẠN</t>
         </is>
       </c>
-      <c r="C71" s="16" t="inlineStr">
+      <c r="C72" s="16" t="inlineStr">
         <is>
           <t>TC_05.001</t>
         </is>
       </c>
-      <c r="D71" s="15" t="inlineStr">
+      <c r="D72" s="15" t="inlineStr">
         <is>
           <t>Cảnh báo đúng mốc T + N - M</t>
         </is>
       </c>
-      <c r="E71" s="16" t="inlineStr">
+      <c r="E72" s="16" t="inlineStr">
         <is>
           <t>P0</t>
         </is>
       </c>
-      <c r="F71" s="15" t="inlineStr">
+      <c r="F72" s="15" t="inlineStr">
         <is>
           <t>M = 3, lĩnh vực N = 30. Cuộc họp Hoàn thành 16/08/2026 -&gt; nhu cầu #201 hết hạn 15/09/2026. Hôm nay 12/09/2026. Nhu cầu chưa từng được cảnh báo, chưa lập dự án.</t>
         </is>
       </c>
-      <c r="G71" s="15" t="inlineStr">
+      <c r="G72" s="15" t="inlineStr">
         <is>
           <t>1. Nhờ kỹ thuật chạy lệnh quét hạn nhu cầu (assign:close-expired-customer-demands)
 2. Đọc kết quả in ra
 3. Đăng nhập tài khoản chủ trì cuộc họp, mở chuông thông báo</t>
         </is>
       </c>
-      <c r="H71" s="15" t="inlineStr">
+      <c r="H72" s="15" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="I71" s="15" t="inlineStr">
+      <c r="I72" s="15" t="inlineStr">
         <is>
           <t>- Kết quả in ra có dòng CẢNH BÁO cho nhu cầu #201 — còn 3 ngày, hết hạn 15/09/2026
 - Người chủ trì nhận được 1 thông báo trong ứng dụng, nội dung nêu tên khách hàng - nhu cầu và số ngày còn lại trước khi tự đóng
 - Bấm vào thông báo mở đúng màn Nhu cầu khách hàng</t>
-        </is>
-      </c>
-      <c r="J71" s="15" t="inlineStr"/>
-      <c r="K71" s="16" t="inlineStr">
-        <is>
-          <t>Not Executed</t>
-        </is>
-      </c>
-      <c r="L71" s="16" t="inlineStr">
-        <is>
-          <t>Not Executed</t>
-        </is>
-      </c>
-      <c r="M71" s="16" t="inlineStr">
-        <is>
-          <t>Not Executed</t>
-        </is>
-      </c>
-      <c r="N71" s="15" t="inlineStr"/>
-      <c r="O71" s="16" t="inlineStr"/>
-      <c r="P71" s="16" t="inlineStr"/>
-      <c r="Q71" s="16" t="inlineStr"/>
-    </row>
-    <row r="72" ht="34" customHeight="1">
-      <c r="A72" s="15" t="inlineStr">
-        <is>
-          <t>Hạn xử lý nhu cầu KH</t>
-        </is>
-      </c>
-      <c r="B72" s="15" t="inlineStr">
-        <is>
-          <t>CẢNH BÁO TRƯỚC HẠN</t>
-        </is>
-      </c>
-      <c r="C72" s="16" t="inlineStr">
-        <is>
-          <t>TC_05.002</t>
-        </is>
-      </c>
-      <c r="D72" s="15" t="inlineStr">
-        <is>
-          <t>Chưa tới mốc cảnh báo thì im lặng</t>
-        </is>
-      </c>
-      <c r="E72" s="16" t="inlineStr">
-        <is>
-          <t>P0</t>
-        </is>
-      </c>
-      <c r="F72" s="15" t="inlineStr">
-        <is>
-          <t>Như trên nhưng hôm nay là 10/09/2026 (còn 5 ngày, vùng cảnh báo là 3 ngày).</t>
-        </is>
-      </c>
-      <c r="G72" s="15" t="inlineStr">
-        <is>
-          <t>1. Chạy lệnh quét hạn nhu cầu
-2. Đọc kết quả</t>
-        </is>
-      </c>
-      <c r="H72" s="15" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="I72" s="15" t="inlineStr">
-        <is>
-          <t>- Không có dòng cảnh báo nào cho nhu cầu #201
-- Không ai nhận được thông báo</t>
         </is>
       </c>
       <c r="J72" s="15" t="inlineStr"/>
@@ -4596,12 +4600,12 @@
       </c>
       <c r="C73" s="16" t="inlineStr">
         <is>
-          <t>TC_05.003</t>
+          <t>TC_05.002</t>
         </is>
       </c>
       <c r="D73" s="15" t="inlineStr">
         <is>
-          <t>Không cảnh báo lại mỗi ngày</t>
+          <t>Chưa tới mốc cảnh báo thì im lặng</t>
         </is>
       </c>
       <c r="E73" s="16" t="inlineStr">
@@ -4611,13 +4615,13 @@
       </c>
       <c r="F73" s="15" t="inlineStr">
         <is>
-          <t>Nhu cầu #201 đã được cảnh báo hôm 12/09/2026.</t>
+          <t>Như trên (M = 3, lĩnh vực N = 30) nhưng hôm nay là 10/09/2026 — còn 5 ngày, vùng cảnh báo là 3 ngày.</t>
         </is>
       </c>
       <c r="G73" s="15" t="inlineStr">
         <is>
-          <t>1. Ngày 13/09/2026 chạy lại lệnh quét hạn nhu cầu
-2. Đọc kết quả và kiểm tra chuông thông báo</t>
+          <t>1. Chạy lệnh quét hạn nhu cầu
+2. Đọc kết quả</t>
         </is>
       </c>
       <c r="H73" s="15" t="inlineStr">
@@ -4627,8 +4631,8 @@
       </c>
       <c r="I73" s="15" t="inlineStr">
         <is>
-          <t>- Không có dòng cảnh báo lặp lại cho #201
-- Người chủ trì không nhận thêm thông báo thứ hai</t>
+          <t>- Không có dòng cảnh báo nào cho nhu cầu #201
+- Không ai nhận được thông báo</t>
         </is>
       </c>
       <c r="J73" s="15" t="inlineStr"/>
@@ -4652,7 +4656,7 @@
       <c r="P73" s="16" t="inlineStr"/>
       <c r="Q73" s="16" t="inlineStr"/>
     </row>
-    <row r="74" ht="67" customHeight="1">
+    <row r="74" ht="34" customHeight="1">
       <c r="A74" s="15" t="inlineStr">
         <is>
           <t>Hạn xử lý nhu cầu KH</t>
@@ -4665,12 +4669,12 @@
       </c>
       <c r="C74" s="16" t="inlineStr">
         <is>
-          <t>TC_05.004</t>
+          <t>TC_05.003</t>
         </is>
       </c>
       <c r="D74" s="15" t="inlineStr">
         <is>
-          <t>N &lt;= M thì bỏ qua cảnh báo</t>
+          <t>Không cảnh báo lại mỗi ngày</t>
         </is>
       </c>
       <c r="E74" s="16" t="inlineStr">
@@ -4680,25 +4684,24 @@
       </c>
       <c r="F74" s="15" t="inlineStr">
         <is>
-          <t>M = 3, lĩnh vực đặt N = 2. Cuộc họp Hoàn thành hôm qua -&gt; nhu cầu #202 hết hạn ngày mai.</t>
+          <t>Nhu cầu #201 (lĩnh vực N = 30, M = 3) đã được cảnh báo hôm 12/09/2026.</t>
         </is>
       </c>
       <c r="G74" s="15" t="inlineStr">
         <is>
-          <t>1. Chạy lệnh quét hạn nhu cầu
-2. Đọc kết quả</t>
+          <t>1. Ngày 13/09/2026 chạy lại lệnh quét hạn nhu cầu
+2. Đọc kết quả và kiểm tra chuông thông báo</t>
         </is>
       </c>
       <c r="H74" s="15" t="inlineStr">
         <is>
-          <t>Thời gian hiệu lực nhu cầu: 2 · Cảnh báo trước khi đóng: 3</t>
+          <t>—</t>
         </is>
       </c>
       <c r="I74" s="15" t="inlineStr">
         <is>
-          <t>- Không có dòng cảnh báo cho #202
-- LƯU Ý: Đây là đúng yêu cầu (thời gian hiệu lực ngắn hơn thời gian cảnh báo thì bỏ cảnh báo), không phải lỗi thiếu thông báo
-- Nhu cầu vẫn sẽ bị đóng đúng ngày hết hạn</t>
+          <t>- Không có dòng cảnh báo lặp lại cho #201
+- Người chủ trì không nhận thêm thông báo thứ hai</t>
         </is>
       </c>
       <c r="J74" s="15" t="inlineStr"/>
@@ -4722,7 +4725,7 @@
       <c r="P74" s="16" t="inlineStr"/>
       <c r="Q74" s="16" t="inlineStr"/>
     </row>
-    <row r="75" ht="34" customHeight="1">
+    <row r="75" ht="67" customHeight="1">
       <c r="A75" s="15" t="inlineStr">
         <is>
           <t>Hạn xử lý nhu cầu KH</t>
@@ -4735,38 +4738,40 @@
       </c>
       <c r="C75" s="16" t="inlineStr">
         <is>
-          <t>TC_05.005</t>
+          <t>TC_05.004</t>
         </is>
       </c>
       <c r="D75" s="15" t="inlineStr">
         <is>
-          <t>N bằng đúng M</t>
+          <t>N &lt;= M thì bỏ qua cảnh báo</t>
         </is>
       </c>
       <c r="E75" s="16" t="inlineStr">
         <is>
-          <t>P1</t>
+          <t>P0</t>
         </is>
       </c>
       <c r="F75" s="15" t="inlineStr">
         <is>
-          <t>M = 3, lĩnh vực N = 3.</t>
+          <t>M = 3, lĩnh vực đặt N = 2. Cuộc họp Hoàn thành hôm qua -&gt; nhu cầu #202 hết hạn ngày mai.</t>
         </is>
       </c>
       <c r="G75" s="15" t="inlineStr">
         <is>
-          <t>1. Chạy lệnh quét hạn nhu cầu với nhu cầu đang trong 3 ngày cuối
+          <t>1. Chạy lệnh quét hạn nhu cầu
 2. Đọc kết quả</t>
         </is>
       </c>
       <c r="H75" s="15" t="inlineStr">
         <is>
-          <t>Thời gian hiệu lực: 3 · Cảnh báo trước: 3</t>
+          <t>Thời gian hiệu lực nhu cầu: 2 · Cảnh báo trước khi đóng: 3</t>
         </is>
       </c>
       <c r="I75" s="15" t="inlineStr">
         <is>
-          <t>- Không cảnh báo (điều kiện là thời gian hiệu lực phải LỚN HƠN thời gian cảnh báo)</t>
+          <t>- Không có dòng cảnh báo cho #202
+- LƯU Ý: Đây là đúng yêu cầu (thời gian hiệu lực ngắn hơn thời gian cảnh báo thì bỏ cảnh báo), không phải lỗi thiếu thông báo
+- Nhu cầu vẫn sẽ bị đóng đúng ngày hết hạn</t>
         </is>
       </c>
       <c r="J75" s="15" t="inlineStr"/>
@@ -4790,7 +4795,7 @@
       <c r="P75" s="16" t="inlineStr"/>
       <c r="Q75" s="16" t="inlineStr"/>
     </row>
-    <row r="76" ht="101" customHeight="1">
+    <row r="76" ht="34" customHeight="1">
       <c r="A76" s="15" t="inlineStr">
         <is>
           <t>Hạn xử lý nhu cầu KH</t>
@@ -4803,40 +4808,38 @@
       </c>
       <c r="C76" s="16" t="inlineStr">
         <is>
-          <t>TC_05.006</t>
+          <t>TC_05.005</t>
         </is>
       </c>
       <c r="D76" s="15" t="inlineStr">
         <is>
-          <t>Người nhận cảnh báo gồm cả 3 vai</t>
+          <t>N bằng đúng M</t>
         </is>
       </c>
       <c r="E76" s="16" t="inlineStr">
         <is>
-          <t>P0</t>
+          <t>P1</t>
         </is>
       </c>
       <c r="F76" s="15" t="inlineStr">
         <is>
-          <t>Cuộc họp M-01 do Nguyễn Thị Cần chủ trì, do Trần Văn B tạo hộ. Nhu cầu #201 đã bàn giao cho Lê Thị C phụ trách, đang trong vùng cảnh báo.</t>
+          <t>M = 3, lĩnh vực N = 3.</t>
         </is>
       </c>
       <c r="G76" s="15" t="inlineStr">
         <is>
-          <t>1. Chạy lệnh quét hạn nhu cầu
-2. Kiểm tra chuông thông báo của cả 3 tài khoản</t>
+          <t>1. Chạy lệnh quét hạn nhu cầu với nhu cầu đang trong 3 ngày cuối
+2. Đọc kết quả</t>
         </is>
       </c>
       <c r="H76" s="15" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Thời gian hiệu lực: 3 · Cảnh báo trước: 3</t>
         </is>
       </c>
       <c r="I76" s="15" t="inlineStr">
         <is>
-          <t>- CẢ 3 đều nhận thông báo: Lê Thị C (nhân sự phụ trách nhu cầu), Trần Văn B (người tạo cuộc họp), Nguyễn Thị Cần (người chủ trì)
-- Mỗi người nhận ĐÚNG 1 thông báo; nếu một người giữ nhiều vai thì cũng chỉ nhận 1, không nhận trùng
-- Nhu cầu CHƯA bàn giao lần nào thì người phụ trách hiểu là người chủ trì</t>
+          <t>- Không cảnh báo (điều kiện là thời gian hiệu lực phải LỚN HƠN thời gian cảnh báo)</t>
         </is>
       </c>
       <c r="J76" s="15" t="inlineStr"/>
@@ -4860,7 +4863,7 @@
       <c r="P76" s="16" t="inlineStr"/>
       <c r="Q76" s="16" t="inlineStr"/>
     </row>
-    <row r="77" ht="55" customHeight="1">
+    <row r="77" ht="101" customHeight="1">
       <c r="A77" s="15" t="inlineStr">
         <is>
           <t>Hạn xử lý nhu cầu KH</t>
@@ -4873,28 +4876,28 @@
       </c>
       <c r="C77" s="16" t="inlineStr">
         <is>
-          <t>TC_05.007</t>
+          <t>TC_05.006</t>
         </is>
       </c>
       <c r="D77" s="15" t="inlineStr">
         <is>
-          <t>Nội dung thông báo đúng khuôn</t>
+          <t>Người nhận cảnh báo gồm cả 3 vai</t>
         </is>
       </c>
       <c r="E77" s="16" t="inlineStr">
         <is>
-          <t>P1</t>
+          <t>P0</t>
         </is>
       </c>
       <c r="F77" s="15" t="inlineStr">
         <is>
-          <t>Nhu cầu #201 của khách 'Công ty ABC', nhu cầu 'Dây chuyền sơn', còn 3 ngày.</t>
+          <t>Cuộc họp M-01 do Nguyễn Thị Cần chủ trì, do Trần Văn B tạo hộ. Nhu cầu #201 đã bàn giao cho Lê Thị C phụ trách, đang trong vùng cảnh báo.</t>
         </is>
       </c>
       <c r="G77" s="15" t="inlineStr">
         <is>
           <t>1. Chạy lệnh quét hạn nhu cầu
-2. Mở chuông thông báo đọc nội dung</t>
+2. Kiểm tra chuông thông báo của cả 3 tài khoản</t>
         </is>
       </c>
       <c r="H77" s="15" t="inlineStr">
@@ -4904,8 +4907,9 @@
       </c>
       <c r="I77" s="15" t="inlineStr">
         <is>
-          <t>- Nội dung nêu rõ: tên khách hàng - tên nhu cầu, cụm 'Sắp đến hạn', và câu 'Tự đóng sau 3 ngày, lập Dự án TKT nếu cần.'
-- Tên nhu cầu in đậm, toàn bộ câu không quá dài</t>
+          <t>- CẢ 3 đều nhận thông báo: Lê Thị C (nhân sự phụ trách nhu cầu), Trần Văn B (người tạo cuộc họp), Nguyễn Thị Cần (người chủ trì)
+- Mỗi người nhận ĐÚNG 1 thông báo; nếu một người giữ nhiều vai thì cũng chỉ nhận 1, không nhận trùng
+- Nhu cầu CHƯA bàn giao lần nào thì người phụ trách hiểu là người chủ trì</t>
         </is>
       </c>
       <c r="J77" s="15" t="inlineStr"/>
@@ -4929,7 +4933,7 @@
       <c r="P77" s="16" t="inlineStr"/>
       <c r="Q77" s="16" t="inlineStr"/>
     </row>
-    <row r="78" ht="34" customHeight="1">
+    <row r="78" ht="55" customHeight="1">
       <c r="A78" s="15" t="inlineStr">
         <is>
           <t>Hạn xử lý nhu cầu KH</t>
@@ -4942,28 +4946,28 @@
       </c>
       <c r="C78" s="16" t="inlineStr">
         <is>
-          <t>TC_05.008</t>
+          <t>TC_05.007</t>
         </is>
       </c>
       <c r="D78" s="15" t="inlineStr">
         <is>
-          <t>Không cảnh báo nhu cầu đã lập dự án</t>
+          <t>Nội dung thông báo đúng khuôn</t>
         </is>
       </c>
       <c r="E78" s="16" t="inlineStr">
         <is>
-          <t>P0</t>
+          <t>P1</t>
         </is>
       </c>
       <c r="F78" s="15" t="inlineStr">
         <is>
-          <t>Nhu cầu #203 đã gắn Dự án TKT, lĩnh vực N = 30, đang trong vùng 3 ngày cuối.</t>
+          <t>Nhu cầu #201 của khách 'Công ty ABC', nhu cầu 'Dây chuyền sơn', còn 3 ngày.</t>
         </is>
       </c>
       <c r="G78" s="15" t="inlineStr">
         <is>
           <t>1. Chạy lệnh quét hạn nhu cầu
-2. Đọc kết quả</t>
+2. Mở chuông thông báo đọc nội dung</t>
         </is>
       </c>
       <c r="H78" s="15" t="inlineStr">
@@ -4973,7 +4977,8 @@
       </c>
       <c r="I78" s="15" t="inlineStr">
         <is>
-          <t>- Không có dòng cảnh báo cho #203</t>
+          <t>- Nội dung nêu rõ: tên khách hàng - tên nhu cầu, cụm 'Sắp đến hạn', và câu 'Tự đóng sau 3 ngày, lập Dự án TKT nếu cần.'
+- Tên nhu cầu in đậm, toàn bộ câu không quá dài</t>
         </is>
       </c>
       <c r="J78" s="15" t="inlineStr"/>
@@ -5010,12 +5015,12 @@
       </c>
       <c r="C79" s="16" t="inlineStr">
         <is>
-          <t>TC_05.009</t>
+          <t>TC_05.008</t>
         </is>
       </c>
       <c r="D79" s="15" t="inlineStr">
         <is>
-          <t>Không cảnh báo nhu cầu lĩnh vực N = 0</t>
+          <t>Không cảnh báo nhu cầu đã lập dự án</t>
         </is>
       </c>
       <c r="E79" s="16" t="inlineStr">
@@ -5025,7 +5030,7 @@
       </c>
       <c r="F79" s="15" t="inlineStr">
         <is>
-          <t>Nhu cầu #204 thuộc lĩnh vực N = 0.</t>
+          <t>Nhu cầu #203 đã gắn Dự án TKT, lĩnh vực N = 30, đang trong vùng 3 ngày cuối.</t>
         </is>
       </c>
       <c r="G79" s="15" t="inlineStr">
@@ -5041,7 +5046,7 @@
       </c>
       <c r="I79" s="15" t="inlineStr">
         <is>
-          <t>- #204 nằm trong nhóm 'bỏ qua vì không đặt thời hạn', không cảnh báo, không đóng</t>
+          <t>- Không có dòng cảnh báo cho #203</t>
         </is>
       </c>
       <c r="J79" s="15" t="inlineStr"/>
@@ -5065,7 +5070,7 @@
       <c r="P79" s="16" t="inlineStr"/>
       <c r="Q79" s="16" t="inlineStr"/>
     </row>
-    <row r="80" ht="37" customHeight="1">
+    <row r="80" ht="34" customHeight="1">
       <c r="A80" s="15" t="inlineStr">
         <is>
           <t>Hạn xử lý nhu cầu KH</t>
@@ -5078,28 +5083,28 @@
       </c>
       <c r="C80" s="16" t="inlineStr">
         <is>
-          <t>TC_05.010</t>
+          <t>TC_05.009</t>
         </is>
       </c>
       <c r="D80" s="15" t="inlineStr">
         <is>
-          <t>Chế độ chạy thử không ghi dữ liệu</t>
+          <t>Không cảnh báo nhu cầu lĩnh vực N = 0</t>
         </is>
       </c>
       <c r="E80" s="16" t="inlineStr">
         <is>
-          <t>P1</t>
+          <t>P0</t>
         </is>
       </c>
       <c r="F80" s="15" t="inlineStr">
         <is>
-          <t>Có 2 nhu cầu trong vùng cảnh báo và 1 nhu cầu quá hạn.</t>
+          <t>Nhu cầu #204 thuộc lĩnh vực N = 0.</t>
         </is>
       </c>
       <c r="G80" s="15" t="inlineStr">
         <is>
-          <t>1. Chạy lệnh quét hạn nhu cầu ở chế độ liệt kê (dry-run)
-2. Kiểm tra chuông thông báo và trạng thái nhu cầu</t>
+          <t>1. Chạy lệnh quét hạn nhu cầu
+2. Đọc kết quả</t>
         </is>
       </c>
       <c r="H80" s="15" t="inlineStr">
@@ -5109,8 +5114,7 @@
       </c>
       <c r="I80" s="15" t="inlineStr">
         <is>
-          <t>- Kết quả in ra đủ 2 dòng cảnh báo và 1 dòng đóng
-- Nhưng KHÔNG ai nhận thông báo, trạng thái nhu cầu không đổi</t>
+          <t>- #204 nằm trong nhóm 'bỏ qua vì không đặt thời hạn', không cảnh báo, không đóng</t>
         </is>
       </c>
       <c r="J80" s="15" t="inlineStr"/>
@@ -5134,145 +5138,145 @@
       <c r="P80" s="16" t="inlineStr"/>
       <c r="Q80" s="16" t="inlineStr"/>
     </row>
-    <row r="81" ht="26" customHeight="1">
-      <c r="A81" s="13" t="n"/>
-      <c r="B81" s="13" t="n"/>
-      <c r="C81" s="14" t="inlineStr">
+    <row r="81" ht="37" customHeight="1">
+      <c r="A81" s="15" t="inlineStr">
+        <is>
+          <t>Hạn xử lý nhu cầu KH</t>
+        </is>
+      </c>
+      <c r="B81" s="15" t="inlineStr">
+        <is>
+          <t>CẢNH BÁO TRƯỚC HẠN</t>
+        </is>
+      </c>
+      <c r="C81" s="16" t="inlineStr">
+        <is>
+          <t>TC_05.010</t>
+        </is>
+      </c>
+      <c r="D81" s="15" t="inlineStr">
+        <is>
+          <t>Chế độ chạy thử không ghi dữ liệu</t>
+        </is>
+      </c>
+      <c r="E81" s="16" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="F81" s="15" t="inlineStr">
+        <is>
+          <t>Có 2 nhu cầu trong vùng cảnh báo và 1 nhu cầu quá hạn.</t>
+        </is>
+      </c>
+      <c r="G81" s="15" t="inlineStr">
+        <is>
+          <t>1. Chạy lệnh quét hạn nhu cầu ở chế độ liệt kê (dry-run)
+2. Kiểm tra chuông thông báo và trạng thái nhu cầu</t>
+        </is>
+      </c>
+      <c r="H81" s="15" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I81" s="15" t="inlineStr">
+        <is>
+          <t>- Kết quả in ra đủ 2 dòng cảnh báo và 1 dòng đóng
+- Nhưng KHÔNG ai nhận thông báo, trạng thái nhu cầu không đổi</t>
+        </is>
+      </c>
+      <c r="J81" s="15" t="inlineStr"/>
+      <c r="K81" s="16" t="inlineStr">
+        <is>
+          <t>Not Executed</t>
+        </is>
+      </c>
+      <c r="L81" s="16" t="inlineStr">
+        <is>
+          <t>Not Executed</t>
+        </is>
+      </c>
+      <c r="M81" s="16" t="inlineStr">
+        <is>
+          <t>Not Executed</t>
+        </is>
+      </c>
+      <c r="N81" s="15" t="inlineStr"/>
+      <c r="O81" s="16" t="inlineStr"/>
+      <c r="P81" s="16" t="inlineStr"/>
+      <c r="Q81" s="16" t="inlineStr"/>
+    </row>
+    <row r="82" ht="26" customHeight="1">
+      <c r="A82" s="13" t="n"/>
+      <c r="B82" s="13" t="n"/>
+      <c r="C82" s="14" t="inlineStr">
         <is>
           <t>VI. TỰ ĐỘNG ĐÓNG NHU CẦU QUÁ HẠN</t>
         </is>
       </c>
-      <c r="D81" s="4" t="n"/>
-      <c r="E81" s="4" t="n"/>
-      <c r="F81" s="4" t="n"/>
-      <c r="G81" s="4" t="n"/>
-      <c r="H81" s="4" t="n"/>
-      <c r="I81" s="4" t="n"/>
-      <c r="J81" s="4" t="n"/>
-      <c r="K81" s="4" t="n"/>
-      <c r="L81" s="4" t="n"/>
-      <c r="M81" s="4" t="n"/>
-      <c r="N81" s="4" t="n"/>
-      <c r="O81" s="4" t="n"/>
-      <c r="P81" s="4" t="n"/>
-      <c r="Q81" s="5" t="n"/>
-    </row>
-    <row r="82" ht="56" customHeight="1">
-      <c r="A82" s="15" t="inlineStr">
-        <is>
-          <t>Hạn xử lý nhu cầu KH</t>
-        </is>
-      </c>
-      <c r="B82" s="15" t="inlineStr">
+      <c r="D82" s="4" t="n"/>
+      <c r="E82" s="4" t="n"/>
+      <c r="F82" s="4" t="n"/>
+      <c r="G82" s="4" t="n"/>
+      <c r="H82" s="4" t="n"/>
+      <c r="I82" s="4" t="n"/>
+      <c r="J82" s="4" t="n"/>
+      <c r="K82" s="4" t="n"/>
+      <c r="L82" s="4" t="n"/>
+      <c r="M82" s="4" t="n"/>
+      <c r="N82" s="4" t="n"/>
+      <c r="O82" s="4" t="n"/>
+      <c r="P82" s="4" t="n"/>
+      <c r="Q82" s="5" t="n"/>
+    </row>
+    <row r="83" ht="56" customHeight="1">
+      <c r="A83" s="15" t="inlineStr">
+        <is>
+          <t>Hạn xử lý nhu cầu KH</t>
+        </is>
+      </c>
+      <c r="B83" s="15" t="inlineStr">
         <is>
           <t>TỰ ĐỘNG ĐÓNG NHU CẦU QUÁ HẠN</t>
         </is>
       </c>
-      <c r="C82" s="16" t="inlineStr">
+      <c r="C83" s="16" t="inlineStr">
         <is>
           <t>TC_06.001</t>
         </is>
       </c>
-      <c r="D82" s="15" t="inlineStr">
+      <c r="D83" s="15" t="inlineStr">
         <is>
           <t>Tự đóng đúng ngày hết hạn</t>
         </is>
       </c>
-      <c r="E82" s="16" t="inlineStr">
+      <c r="E83" s="16" t="inlineStr">
         <is>
           <t>P0</t>
         </is>
       </c>
-      <c r="F82" s="15" t="inlineStr">
+      <c r="F83" s="15" t="inlineStr">
         <is>
           <t>M = 3, N = 30, cuộc họp Hoàn thành 16/08/2026 -&gt; nhu cầu #301 hết hạn 15/09/2026. Hôm nay 15/09/2026.</t>
         </is>
       </c>
-      <c r="G82" s="15" t="inlineStr">
+      <c r="G83" s="15" t="inlineStr">
         <is>
           <t>1. Chạy lệnh quét hạn nhu cầu
 2. Mở màn Nhu cầu khách hàng xem #301</t>
         </is>
       </c>
-      <c r="H82" s="15" t="inlineStr">
+      <c r="H83" s="15" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="I82" s="15" t="inlineStr">
+      <c r="I83" s="15" t="inlineStr">
         <is>
           <t>- Kết quả in ra có dòng ĐÓNG cho #301 — hết hạn 15/09/2026
 - Trạng thái #301 chuyển sang 'Đóng', badge màu xám
 - Cột hạn chuyển thành 'Không giới hạn thời gian hiệu lực'</t>
-        </is>
-      </c>
-      <c r="J82" s="15" t="inlineStr"/>
-      <c r="K82" s="16" t="inlineStr">
-        <is>
-          <t>Not Executed</t>
-        </is>
-      </c>
-      <c r="L82" s="16" t="inlineStr">
-        <is>
-          <t>Not Executed</t>
-        </is>
-      </c>
-      <c r="M82" s="16" t="inlineStr">
-        <is>
-          <t>Not Executed</t>
-        </is>
-      </c>
-      <c r="N82" s="15" t="inlineStr"/>
-      <c r="O82" s="16" t="inlineStr"/>
-      <c r="P82" s="16" t="inlineStr"/>
-      <c r="Q82" s="16" t="inlineStr"/>
-    </row>
-    <row r="83" ht="34" customHeight="1">
-      <c r="A83" s="15" t="inlineStr">
-        <is>
-          <t>Hạn xử lý nhu cầu KH</t>
-        </is>
-      </c>
-      <c r="B83" s="15" t="inlineStr">
-        <is>
-          <t>TỰ ĐỘNG ĐÓNG NHU CẦU QUÁ HẠN</t>
-        </is>
-      </c>
-      <c r="C83" s="16" t="inlineStr">
-        <is>
-          <t>TC_06.002</t>
-        </is>
-      </c>
-      <c r="D83" s="15" t="inlineStr">
-        <is>
-          <t>Ngày đóng ghi đúng ngày hết hạn dù chạy muộn</t>
-        </is>
-      </c>
-      <c r="E83" s="16" t="inlineStr">
-        <is>
-          <t>P0</t>
-        </is>
-      </c>
-      <c r="F83" s="15" t="inlineStr">
-        <is>
-          <t>Nhu cầu #302 hết hạn 10/09/2026 nhưng việc quét không chạy mấy ngày; hôm nay 15/09/2026.</t>
-        </is>
-      </c>
-      <c r="G83" s="15" t="inlineStr">
-        <is>
-          <t>1. Chạy lệnh quét hạn nhu cầu
-2. Mở chi tiết / lịch sử của nhu cầu #302 xem ngày đóng</t>
-        </is>
-      </c>
-      <c r="H83" s="15" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="I83" s="15" t="inlineStr">
-        <is>
-          <t>- Nhu cầu chuyển sang Đóng
-- LƯU Ý: Ngày đóng ghi 10/09/2026 (ngày hết hạn thật), KHÔNG phải 15/09/2026</t>
         </is>
       </c>
       <c r="J83" s="15" t="inlineStr"/>
@@ -5309,12 +5313,12 @@
       </c>
       <c r="C84" s="16" t="inlineStr">
         <is>
-          <t>TC_06.003</t>
+          <t>TC_06.002</t>
         </is>
       </c>
       <c r="D84" s="15" t="inlineStr">
         <is>
-          <t>Chưa tới hạn thì chưa đóng</t>
+          <t>Ngày đóng ghi đúng ngày hết hạn dù chạy muộn</t>
         </is>
       </c>
       <c r="E84" s="16" t="inlineStr">
@@ -5324,13 +5328,13 @@
       </c>
       <c r="F84" s="15" t="inlineStr">
         <is>
-          <t>Nhu cầu #303 hết hạn 20/09/2026, hôm nay 15/09/2026.</t>
+          <t>Nhu cầu #302 hết hạn 10/09/2026 nhưng việc quét không chạy mấy ngày; hôm nay 15/09/2026.</t>
         </is>
       </c>
       <c r="G84" s="15" t="inlineStr">
         <is>
           <t>1. Chạy lệnh quét hạn nhu cầu
-2. Kiểm tra trạng thái #303</t>
+2. Mở chi tiết / lịch sử của nhu cầu #302 xem ngày đóng</t>
         </is>
       </c>
       <c r="H84" s="15" t="inlineStr">
@@ -5340,7 +5344,8 @@
       </c>
       <c r="I84" s="15" t="inlineStr">
         <is>
-          <t>- Vẫn 'Đang theo dõi', không bị đóng</t>
+          <t>- Nhu cầu chuyển sang Đóng
+- LƯU Ý: Ngày đóng ghi 10/09/2026 (ngày hết hạn thật), KHÔNG phải 15/09/2026</t>
         </is>
       </c>
       <c r="J84" s="15" t="inlineStr"/>
@@ -5377,12 +5382,12 @@
       </c>
       <c r="C85" s="16" t="inlineStr">
         <is>
-          <t>TC_06.004</t>
+          <t>TC_06.003</t>
         </is>
       </c>
       <c r="D85" s="15" t="inlineStr">
         <is>
-          <t>Không đóng nhu cầu đã lập Dự án TKT</t>
+          <t>Chưa tới hạn thì chưa đóng</t>
         </is>
       </c>
       <c r="E85" s="16" t="inlineStr">
@@ -5392,13 +5397,13 @@
       </c>
       <c r="F85" s="15" t="inlineStr">
         <is>
-          <t>Nhu cầu #304 quá hạn 5 ngày nhưng đã gắn Dự án TKT.</t>
+          <t>Nhu cầu #303 hết hạn 20/09/2026, hôm nay 15/09/2026.</t>
         </is>
       </c>
       <c r="G85" s="15" t="inlineStr">
         <is>
           <t>1. Chạy lệnh quét hạn nhu cầu
-2. Kiểm tra #304</t>
+2. Kiểm tra trạng thái #303</t>
         </is>
       </c>
       <c r="H85" s="15" t="inlineStr">
@@ -5408,7 +5413,7 @@
       </c>
       <c r="I85" s="15" t="inlineStr">
         <is>
-          <t>- Không bị đóng, trạng thái vẫn là 'Đã lập dự án TKT'</t>
+          <t>- Vẫn 'Đang theo dõi', không bị đóng</t>
         </is>
       </c>
       <c r="J85" s="15" t="inlineStr"/>
@@ -5445,12 +5450,12 @@
       </c>
       <c r="C86" s="16" t="inlineStr">
         <is>
-          <t>TC_06.005</t>
+          <t>TC_06.004</t>
         </is>
       </c>
       <c r="D86" s="15" t="inlineStr">
         <is>
-          <t>Không đụng nhu cầu đã đóng tay trước đó</t>
+          <t>Không đóng nhu cầu đã lập Dự án TKT</t>
         </is>
       </c>
       <c r="E86" s="16" t="inlineStr">
@@ -5460,13 +5465,13 @@
       </c>
       <c r="F86" s="15" t="inlineStr">
         <is>
-          <t>Nhu cầu #305 đã được người dùng đóng tay kèm ghi chú 'Khách dừng đầu tư'.</t>
+          <t>Nhu cầu #304 quá hạn 5 ngày nhưng đã gắn Dự án TKT.</t>
         </is>
       </c>
       <c r="G86" s="15" t="inlineStr">
         <is>
           <t>1. Chạy lệnh quét hạn nhu cầu
-2. Mở #305 xem ghi chú đóng</t>
+2. Kiểm tra #304</t>
         </is>
       </c>
       <c r="H86" s="15" t="inlineStr">
@@ -5476,7 +5481,7 @@
       </c>
       <c r="I86" s="15" t="inlineStr">
         <is>
-          <t>- Ghi chú và người đóng giữ nguyên, không bị ghi đè thành đóng tự động</t>
+          <t>- Không bị đóng, trạng thái vẫn là 'Đã lập dự án TKT'</t>
         </is>
       </c>
       <c r="J86" s="15" t="inlineStr"/>
@@ -5500,7 +5505,7 @@
       <c r="P86" s="16" t="inlineStr"/>
       <c r="Q86" s="16" t="inlineStr"/>
     </row>
-    <row r="87" ht="37" customHeight="1">
+    <row r="87" ht="34" customHeight="1">
       <c r="A87" s="15" t="inlineStr">
         <is>
           <t>Hạn xử lý nhu cầu KH</t>
@@ -5513,12 +5518,12 @@
       </c>
       <c r="C87" s="16" t="inlineStr">
         <is>
-          <t>TC_06.006</t>
+          <t>TC_06.005</t>
         </is>
       </c>
       <c r="D87" s="15" t="inlineStr">
         <is>
-          <t>Chạy lại nhiều lần cho cùng kết quả</t>
+          <t>Không đụng nhu cầu đã đóng tay trước đó</t>
         </is>
       </c>
       <c r="E87" s="16" t="inlineStr">
@@ -5528,13 +5533,13 @@
       </c>
       <c r="F87" s="15" t="inlineStr">
         <is>
-          <t>Vừa chạy quét xong, đã đóng 3 nhu cầu.</t>
+          <t>Nhu cầu #305 đã được người dùng đóng tay kèm ghi chú 'Khách dừng đầu tư'.</t>
         </is>
       </c>
       <c r="G87" s="15" t="inlineStr">
         <is>
-          <t>1. Chạy lại lệnh quét hạn nhu cầu ngay lập tức
-2. Đọc kết quả</t>
+          <t>1. Chạy lệnh quét hạn nhu cầu
+2. Mở #305 xem ghi chú đóng</t>
         </is>
       </c>
       <c r="H87" s="15" t="inlineStr">
@@ -5544,8 +5549,7 @@
       </c>
       <c r="I87" s="15" t="inlineStr">
         <is>
-          <t>- Lần 2 báo đóng 0 nhu cầu, cảnh báo 0 nhu cầu
-- Không nhu cầu nào bị đóng hai lần, không ai nhận thông báo lặp</t>
+          <t>- Ghi chú và người đóng giữ nguyên, không bị ghi đè thành đóng tự động</t>
         </is>
       </c>
       <c r="J87" s="15" t="inlineStr"/>
@@ -5569,7 +5573,7 @@
       <c r="P87" s="16" t="inlineStr"/>
       <c r="Q87" s="16" t="inlineStr"/>
     </row>
-    <row r="88" ht="34" customHeight="1">
+    <row r="88" ht="37" customHeight="1">
       <c r="A88" s="15" t="inlineStr">
         <is>
           <t>Hạn xử lý nhu cầu KH</t>
@@ -5582,28 +5586,28 @@
       </c>
       <c r="C88" s="16" t="inlineStr">
         <is>
-          <t>TC_06.007</t>
+          <t>TC_06.006</t>
         </is>
       </c>
       <c r="D88" s="15" t="inlineStr">
         <is>
-          <t>Dòng tổng kết sau khi chạy</t>
+          <t>Chạy lại nhiều lần cho cùng kết quả</t>
         </is>
       </c>
       <c r="E88" s="16" t="inlineStr">
         <is>
-          <t>P1</t>
+          <t>P0</t>
         </is>
       </c>
       <c r="F88" s="15" t="inlineStr">
         <is>
-          <t>Có 2 nhu cầu tới hạn, 1 nhu cầu trong vùng cảnh báo, 30 nhu cầu thuộc lĩnh vực N = 0.</t>
+          <t>Vừa chạy quét xong, đã đóng 3 nhu cầu.</t>
         </is>
       </c>
       <c r="G88" s="15" t="inlineStr">
         <is>
-          <t>1. Chạy lệnh quét hạn nhu cầu
-2. Đọc dòng tổng kết cuối cùng</t>
+          <t>1. Chạy lại lệnh quét hạn nhu cầu ngay lập tức
+2. Đọc kết quả</t>
         </is>
       </c>
       <c r="H88" s="15" t="inlineStr">
@@ -5613,7 +5617,8 @@
       </c>
       <c r="I88" s="15" t="inlineStr">
         <is>
-          <t>- Ghi 'Đã đóng 2 nhu cầu, cảnh báo 1 nhu cầu (bỏ qua 30 nhu cầu không đặt thời hạn).'</t>
+          <t>- Lần 2 báo đóng 0 nhu cầu, cảnh báo 0 nhu cầu
+- Không nhu cầu nào bị đóng hai lần, không ai nhận thông báo lặp</t>
         </is>
       </c>
       <c r="J88" s="15" t="inlineStr"/>
@@ -5637,7 +5642,7 @@
       <c r="P88" s="16" t="inlineStr"/>
       <c r="Q88" s="16" t="inlineStr"/>
     </row>
-    <row r="89" ht="61" customHeight="1">
+    <row r="89" ht="34" customHeight="1">
       <c r="A89" s="15" t="inlineStr">
         <is>
           <t>Hạn xử lý nhu cầu KH</t>
@@ -5650,12 +5655,12 @@
       </c>
       <c r="C89" s="16" t="inlineStr">
         <is>
-          <t>TC_06.008</t>
+          <t>TC_06.007</t>
         </is>
       </c>
       <c r="D89" s="15" t="inlineStr">
         <is>
-          <t>Đặt N nhỏ làm nhu cầu cũ tới hạn ngay</t>
+          <t>Dòng tổng kết sau khi chạy</t>
         </is>
       </c>
       <c r="E89" s="16" t="inlineStr">
@@ -5665,25 +5670,23 @@
       </c>
       <c r="F89" s="15" t="inlineStr">
         <is>
-          <t>Nhiều nhu cầu cũ của lĩnh vực LVCTKD.0001, cuộc họp Hoàn thành từ 3 tháng trước; lĩnh vực đang N = 0.</t>
+          <t>Có 2 nhu cầu tới hạn, 1 nhu cầu trong vùng cảnh báo, 30 nhu cầu thuộc lĩnh vực N = 0.</t>
         </is>
       </c>
       <c r="G89" s="15" t="inlineStr">
         <is>
-          <t>1. Sửa lĩnh vực đặt N = 30
-2. Chạy lệnh quét hạn nhu cầu ở chế độ liệt kê
-3. Đọc kết quả</t>
+          <t>1. Chạy lệnh quét hạn nhu cầu
+2. Đọc dòng tổng kết cuối cùng</t>
         </is>
       </c>
       <c r="H89" s="15" t="inlineStr">
         <is>
-          <t>Thời gian hiệu lực nhu cầu: 30</t>
+          <t>—</t>
         </is>
       </c>
       <c r="I89" s="15" t="inlineStr">
         <is>
-          <t>- Kết quả liệt kê toàn bộ nhu cầu cũ sẽ bị đóng, mỗi dòng kèm đúng ngày hết hạn riêng
-- LƯU Ý: Kiểm kỹ trước khi chạy thật: đặt N nhỏ là đóng hàng loạt nhu cầu cũ ngay lần quét kế tiếp</t>
+          <t>- Ghi 'Đã đóng 2 nhu cầu, cảnh báo 1 nhu cầu (bỏ qua 30 nhu cầu không đặt thời hạn).'</t>
         </is>
       </c>
       <c r="J89" s="15" t="inlineStr"/>
@@ -5707,7 +5710,7 @@
       <c r="P89" s="16" t="inlineStr"/>
       <c r="Q89" s="16" t="inlineStr"/>
     </row>
-    <row r="90" ht="47" customHeight="1">
+    <row r="90" ht="61" customHeight="1">
       <c r="A90" s="15" t="inlineStr">
         <is>
           <t>Hạn xử lý nhu cầu KH</t>
@@ -5720,12 +5723,12 @@
       </c>
       <c r="C90" s="16" t="inlineStr">
         <is>
-          <t>TC_06.009</t>
+          <t>TC_06.008</t>
         </is>
       </c>
       <c r="D90" s="15" t="inlineStr">
         <is>
-          <t>Nhu cầu bị đóng vẫn xem được trong danh sách</t>
+          <t>Đặt N nhỏ làm nhu cầu cũ tới hạn ngay</t>
         </is>
       </c>
       <c r="E90" s="16" t="inlineStr">
@@ -5735,24 +5738,25 @@
       </c>
       <c r="F90" s="15" t="inlineStr">
         <is>
-          <t>Nhu cầu #301 vừa bị hệ thống đóng.</t>
+          <t>Nhiều nhu cầu cũ của lĩnh vực LVCTKD.0001, cuộc họp Hoàn thành từ 3 tháng trước; lĩnh vực đang N = 0.</t>
         </is>
       </c>
       <c r="G90" s="15" t="inlineStr">
         <is>
-          <t>1. Vào màn Nhu cầu khách hàng, lọc trạng thái Đóng
-2. Mở lịch sử cập nhật của #301</t>
+          <t>1. Sửa lĩnh vực đặt N = 30
+2. Chạy lệnh quét hạn nhu cầu ở chế độ liệt kê
+3. Đọc kết quả</t>
         </is>
       </c>
       <c r="H90" s="15" t="inlineStr">
         <is>
-          <t>Trạng thái: Đóng</t>
+          <t>Thời gian hiệu lực nhu cầu: 30</t>
         </is>
       </c>
       <c r="I90" s="15" t="inlineStr">
         <is>
-          <t>- Dòng #301 vẫn nằm trong danh sách khi lọc trạng thái Đóng
-- Lịch sử cho thấy nhu cầu bị đóng, người đóng để trống nghĩa là hệ thống tự đóng</t>
+          <t>- Kết quả liệt kê toàn bộ nhu cầu cũ sẽ bị đóng, mỗi dòng kèm đúng ngày hết hạn riêng
+- LƯU Ý: Kiểm kỹ trước khi chạy thật: đặt N nhỏ là đóng hàng loạt nhu cầu cũ ngay lần quét kế tiếp</t>
         </is>
       </c>
       <c r="J90" s="15" t="inlineStr"/>
@@ -5776,142 +5780,144 @@
       <c r="P90" s="16" t="inlineStr"/>
       <c r="Q90" s="16" t="inlineStr"/>
     </row>
-    <row r="91" ht="26" customHeight="1">
-      <c r="A91" s="13" t="n"/>
-      <c r="B91" s="13" t="n"/>
-      <c r="C91" s="14" t="inlineStr">
+    <row r="91" ht="47" customHeight="1">
+      <c r="A91" s="15" t="inlineStr">
+        <is>
+          <t>Hạn xử lý nhu cầu KH</t>
+        </is>
+      </c>
+      <c r="B91" s="15" t="inlineStr">
+        <is>
+          <t>TỰ ĐỘNG ĐÓNG NHU CẦU QUÁ HẠN</t>
+        </is>
+      </c>
+      <c r="C91" s="16" t="inlineStr">
+        <is>
+          <t>TC_06.009</t>
+        </is>
+      </c>
+      <c r="D91" s="15" t="inlineStr">
+        <is>
+          <t>Nhu cầu bị đóng vẫn xem được trong danh sách</t>
+        </is>
+      </c>
+      <c r="E91" s="16" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="F91" s="15" t="inlineStr">
+        <is>
+          <t>Nhu cầu #301 vừa bị hệ thống đóng.</t>
+        </is>
+      </c>
+      <c r="G91" s="15" t="inlineStr">
+        <is>
+          <t>1. Vào màn Nhu cầu khách hàng, lọc trạng thái Đóng
+2. Mở lịch sử cập nhật của #301</t>
+        </is>
+      </c>
+      <c r="H91" s="15" t="inlineStr">
+        <is>
+          <t>Trạng thái: Đóng</t>
+        </is>
+      </c>
+      <c r="I91" s="15" t="inlineStr">
+        <is>
+          <t>- Dòng #301 vẫn nằm trong danh sách khi lọc trạng thái Đóng
+- Lịch sử cho thấy nhu cầu bị đóng, người đóng để trống nghĩa là hệ thống tự đóng</t>
+        </is>
+      </c>
+      <c r="J91" s="15" t="inlineStr"/>
+      <c r="K91" s="16" t="inlineStr">
+        <is>
+          <t>Not Executed</t>
+        </is>
+      </c>
+      <c r="L91" s="16" t="inlineStr">
+        <is>
+          <t>Not Executed</t>
+        </is>
+      </c>
+      <c r="M91" s="16" t="inlineStr">
+        <is>
+          <t>Not Executed</t>
+        </is>
+      </c>
+      <c r="N91" s="15" t="inlineStr"/>
+      <c r="O91" s="16" t="inlineStr"/>
+      <c r="P91" s="16" t="inlineStr"/>
+      <c r="Q91" s="16" t="inlineStr"/>
+    </row>
+    <row r="92" ht="26" customHeight="1">
+      <c r="A92" s="13" t="n"/>
+      <c r="B92" s="13" t="n"/>
+      <c r="C92" s="14" t="inlineStr">
         <is>
           <t>VII. CHẶN TẠO DỰ ÁN TKT TỪ NHU CẦU ĐÃ ĐÓNG</t>
         </is>
       </c>
-      <c r="D91" s="4" t="n"/>
-      <c r="E91" s="4" t="n"/>
-      <c r="F91" s="4" t="n"/>
-      <c r="G91" s="4" t="n"/>
-      <c r="H91" s="4" t="n"/>
-      <c r="I91" s="4" t="n"/>
-      <c r="J91" s="4" t="n"/>
-      <c r="K91" s="4" t="n"/>
-      <c r="L91" s="4" t="n"/>
-      <c r="M91" s="4" t="n"/>
-      <c r="N91" s="4" t="n"/>
-      <c r="O91" s="4" t="n"/>
-      <c r="P91" s="4" t="n"/>
-      <c r="Q91" s="5" t="n"/>
-    </row>
-    <row r="92" ht="51" customHeight="1">
-      <c r="A92" s="15" t="inlineStr">
-        <is>
-          <t>Hạn xử lý nhu cầu KH</t>
-        </is>
-      </c>
-      <c r="B92" s="15" t="inlineStr">
+      <c r="D92" s="4" t="n"/>
+      <c r="E92" s="4" t="n"/>
+      <c r="F92" s="4" t="n"/>
+      <c r="G92" s="4" t="n"/>
+      <c r="H92" s="4" t="n"/>
+      <c r="I92" s="4" t="n"/>
+      <c r="J92" s="4" t="n"/>
+      <c r="K92" s="4" t="n"/>
+      <c r="L92" s="4" t="n"/>
+      <c r="M92" s="4" t="n"/>
+      <c r="N92" s="4" t="n"/>
+      <c r="O92" s="4" t="n"/>
+      <c r="P92" s="4" t="n"/>
+      <c r="Q92" s="5" t="n"/>
+    </row>
+    <row r="93" ht="51" customHeight="1">
+      <c r="A93" s="15" t="inlineStr">
+        <is>
+          <t>Hạn xử lý nhu cầu KH</t>
+        </is>
+      </c>
+      <c r="B93" s="15" t="inlineStr">
         <is>
           <t>CHẶN TẠO DỰ ÁN TKT TỪ NHU CẦU ĐÃ ĐÓNG</t>
         </is>
       </c>
-      <c r="C92" s="16" t="inlineStr">
+      <c r="C93" s="16" t="inlineStr">
         <is>
           <t>TC_07.001</t>
         </is>
       </c>
-      <c r="D92" s="15" t="inlineStr">
+      <c r="D93" s="15" t="inlineStr">
         <is>
           <t>Ẩn nút Tạo Dự án TKT khi nhu cầu đã đóng</t>
         </is>
       </c>
-      <c r="E92" s="16" t="inlineStr">
+      <c r="E93" s="16" t="inlineStr">
         <is>
           <t>P0</t>
         </is>
       </c>
-      <c r="F92" s="15" t="inlineStr">
+      <c r="F93" s="15" t="inlineStr">
         <is>
           <t>Nhu cầu #301 đang Đóng, chưa có dự án.</t>
         </is>
       </c>
-      <c r="G92" s="15" t="inlineStr">
+      <c r="G93" s="15" t="inlineStr">
         <is>
           <t>1. Vào màn Nhu cầu khách hàng, tìm dòng #301
 2. Quan sát cột Dự án TKT</t>
         </is>
       </c>
-      <c r="H92" s="15" t="inlineStr">
+      <c r="H93" s="15" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="I92" s="15" t="inlineStr">
+      <c r="I93" s="15" t="inlineStr">
         <is>
           <t>- Ô chỉ hiện dấu '—', KHÔNG còn nút Tạo Dự án TKT
 - LƯU Ý: Yêu cầu gốc ghi 'làm mờ kèm tooltip' nhưng quy ước dự án là ẩn hẳn — ghi nhận, không tính là lỗi</t>
-        </is>
-      </c>
-      <c r="J92" s="15" t="inlineStr"/>
-      <c r="K92" s="16" t="inlineStr">
-        <is>
-          <t>Not Executed</t>
-        </is>
-      </c>
-      <c r="L92" s="16" t="inlineStr">
-        <is>
-          <t>Not Executed</t>
-        </is>
-      </c>
-      <c r="M92" s="16" t="inlineStr">
-        <is>
-          <t>Not Executed</t>
-        </is>
-      </c>
-      <c r="N92" s="15" t="inlineStr"/>
-      <c r="O92" s="16" t="inlineStr"/>
-      <c r="P92" s="16" t="inlineStr"/>
-      <c r="Q92" s="16" t="inlineStr"/>
-    </row>
-    <row r="93" ht="34" customHeight="1">
-      <c r="A93" s="15" t="inlineStr">
-        <is>
-          <t>Hạn xử lý nhu cầu KH</t>
-        </is>
-      </c>
-      <c r="B93" s="15" t="inlineStr">
-        <is>
-          <t>CHẶN TẠO DỰ ÁN TKT TỪ NHU CẦU ĐÃ ĐÓNG</t>
-        </is>
-      </c>
-      <c r="C93" s="16" t="inlineStr">
-        <is>
-          <t>TC_07.002</t>
-        </is>
-      </c>
-      <c r="D93" s="15" t="inlineStr">
-        <is>
-          <t>Nút Tạo Dự án TKT còn nguyên với nhu cầu đang theo dõi</t>
-        </is>
-      </c>
-      <c r="E93" s="16" t="inlineStr">
-        <is>
-          <t>P0</t>
-        </is>
-      </c>
-      <c r="F93" s="15" t="inlineStr">
-        <is>
-          <t>Nhu cầu #303 đang theo dõi, chưa có dự án.</t>
-        </is>
-      </c>
-      <c r="G93" s="15" t="inlineStr">
-        <is>
-          <t>1. Tìm dòng #303, quan sát cột Dự án TKT</t>
-        </is>
-      </c>
-      <c r="H93" s="15" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="I93" s="15" t="inlineStr">
-        <is>
-          <t>- Hiện nút 'Tạo Dự án TKT', bấm được và mở màn lập dự án</t>
         </is>
       </c>
       <c r="J93" s="15" t="inlineStr"/>
@@ -5935,7 +5941,7 @@
       <c r="P93" s="16" t="inlineStr"/>
       <c r="Q93" s="16" t="inlineStr"/>
     </row>
-    <row r="94" ht="45" customHeight="1">
+    <row r="94" ht="34" customHeight="1">
       <c r="A94" s="15" t="inlineStr">
         <is>
           <t>Hạn xử lý nhu cầu KH</t>
@@ -5948,12 +5954,12 @@
       </c>
       <c r="C94" s="16" t="inlineStr">
         <is>
-          <t>TC_07.003</t>
+          <t>TC_07.002</t>
         </is>
       </c>
       <c r="D94" s="15" t="inlineStr">
         <is>
-          <t>Chặn lập dự án khi nhu cầu bị đóng ngay lúc đang mở form</t>
+          <t>Nút Tạo Dự án TKT còn nguyên với nhu cầu đang theo dõi</t>
         </is>
       </c>
       <c r="E94" s="16" t="inlineStr">
@@ -5963,13 +5969,12 @@
       </c>
       <c r="F94" s="15" t="inlineStr">
         <is>
-          <t>Người dùng đã mở form lập Dự án TKT từ nhu cầu #306; trong lúc đó việc quét chạy và đóng #306.</t>
+          <t>Nhu cầu #303 đang theo dõi, chưa có dự án.</t>
         </is>
       </c>
       <c r="G94" s="15" t="inlineStr">
         <is>
-          <t>1. Quay lại form đang mở, điền đủ thông tin
-2. Bấm Lưu</t>
+          <t>1. Tìm dòng #303, quan sát cột Dự án TKT</t>
         </is>
       </c>
       <c r="H94" s="15" t="inlineStr">
@@ -5979,8 +5984,7 @@
       </c>
       <c r="I94" s="15" t="inlineStr">
         <is>
-          <t>- Hệ thống từ chối kèm câu: 'Nhu cầu này đã quá hạn xử lý và bị đóng tự động. Không thể tạo Dự án tiền khả thi.'
-- Không tạo ra dự án nào</t>
+          <t>- Hiện nút 'Tạo Dự án TKT', bấm được và mở màn lập dự án</t>
         </is>
       </c>
       <c r="J94" s="15" t="inlineStr"/>
@@ -6004,7 +6008,7 @@
       <c r="P94" s="16" t="inlineStr"/>
       <c r="Q94" s="16" t="inlineStr"/>
     </row>
-    <row r="95" ht="34" customHeight="1">
+    <row r="95" ht="45" customHeight="1">
       <c r="A95" s="15" t="inlineStr">
         <is>
           <t>Hạn xử lý nhu cầu KH</t>
@@ -6017,12 +6021,12 @@
       </c>
       <c r="C95" s="16" t="inlineStr">
         <is>
-          <t>TC_07.004</t>
+          <t>TC_07.003</t>
         </is>
       </c>
       <c r="D95" s="15" t="inlineStr">
         <is>
-          <t>Gắn thêm nhu cầu đã đóng vào dự án đang sửa</t>
+          <t>Chặn lập dự án khi nhu cầu bị đóng ngay lúc đang mở form</t>
         </is>
       </c>
       <c r="E95" s="16" t="inlineStr">
@@ -6032,25 +6036,24 @@
       </c>
       <c r="F95" s="15" t="inlineStr">
         <is>
-          <t>Dự án TKT DA-01 đang sửa; nhu cầu #301 đã Đóng.</t>
+          <t>Người dùng đã mở form lập Dự án TKT từ nhu cầu #306; trong lúc đó việc quét chạy và đóng #306.</t>
         </is>
       </c>
       <c r="G95" s="15" t="inlineStr">
         <is>
-          <t>1. Mở màn Sửa dự án DA-01
-2. Chọn nhu cầu #301 vào dự án
-3. Bấm Lưu</t>
+          <t>1. Quay lại form đang mở, điền đủ thông tin
+2. Bấm Lưu</t>
         </is>
       </c>
       <c r="H95" s="15" t="inlineStr">
         <is>
-          <t>Nhu cầu: #301</t>
+          <t>—</t>
         </is>
       </c>
       <c r="I95" s="15" t="inlineStr">
         <is>
-          <t>- Bị chặn với đúng câu thông báo như mục 3
-- Dự án không lưu được liên kết đó</t>
+          <t>- Hệ thống từ chối kèm câu: 'Nhu cầu này đã quá hạn xử lý và bị đóng tự động. Không thể tạo Dự án tiền khả thi.'
+- Không tạo ra dự án nào</t>
         </is>
       </c>
       <c r="J95" s="15" t="inlineStr"/>
@@ -6087,37 +6090,40 @@
       </c>
       <c r="C96" s="16" t="inlineStr">
         <is>
-          <t>TC_07.005</t>
+          <t>TC_07.004</t>
         </is>
       </c>
       <c r="D96" s="15" t="inlineStr">
         <is>
-          <t>Nhu cầu đóng tay cũng bị chặn lập dự án</t>
+          <t>Gắn thêm nhu cầu đã đóng vào dự án đang sửa</t>
         </is>
       </c>
       <c r="E96" s="16" t="inlineStr">
         <is>
-          <t>P1</t>
+          <t>P0</t>
         </is>
       </c>
       <c r="F96" s="15" t="inlineStr">
         <is>
-          <t>Nhu cầu #305 do người dùng đóng tay.</t>
+          <t>Dự án TKT DA-01 đang sửa; nhu cầu #301 đã Đóng.</t>
         </is>
       </c>
       <c r="G96" s="15" t="inlineStr">
         <is>
-          <t>1. Thử lập Dự án TKT từ #305</t>
+          <t>1. Mở màn Sửa dự án DA-01
+2. Chọn nhu cầu #301 vào dự án
+3. Bấm Lưu</t>
         </is>
       </c>
       <c r="H96" s="15" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Nhu cầu: #301</t>
         </is>
       </c>
       <c r="I96" s="15" t="inlineStr">
         <is>
-          <t>- Không có nút Tạo Dự án TKT; gọi thẳng chức năng cũng bị chặn</t>
+          <t>- Bị chặn với đúng câu thông báo như mục 3
+- Dự án không lưu được liên kết đó</t>
         </is>
       </c>
       <c r="J96" s="15" t="inlineStr"/>
@@ -6154,27 +6160,27 @@
       </c>
       <c r="C97" s="16" t="inlineStr">
         <is>
-          <t>TC_07.006</t>
+          <t>TC_07.005</t>
         </is>
       </c>
       <c r="D97" s="15" t="inlineStr">
         <is>
-          <t>Nhu cầu đã có dự án thì hiện liên kết thay vì nút</t>
+          <t>Nhu cầu đóng tay cũng bị chặn lập dự án</t>
         </is>
       </c>
       <c r="E97" s="16" t="inlineStr">
         <is>
-          <t>P2</t>
+          <t>P1</t>
         </is>
       </c>
       <c r="F97" s="15" t="inlineStr">
         <is>
-          <t>Nhu cầu #106 đã gắn dự án DA-02.</t>
+          <t>Nhu cầu #305 do người dùng đóng tay.</t>
         </is>
       </c>
       <c r="G97" s="15" t="inlineStr">
         <is>
-          <t>1. Xem cột Dự án TKT của dòng #106</t>
+          <t>1. Thử lập Dự án TKT từ #305</t>
         </is>
       </c>
       <c r="H97" s="15" t="inlineStr">
@@ -6184,7 +6190,7 @@
       </c>
       <c r="I97" s="15" t="inlineStr">
         <is>
-          <t>- Hiện mã dự án bấm được, dẫn sang màn chi tiết dự án, không còn nút tạo mới</t>
+          <t>- Không có nút Tạo Dự án TKT; gọi thẳng chức năng cũng bị chặn</t>
         </is>
       </c>
       <c r="J97" s="15" t="inlineStr"/>
@@ -6208,143 +6214,141 @@
       <c r="P97" s="16" t="inlineStr"/>
       <c r="Q97" s="16" t="inlineStr"/>
     </row>
-    <row r="98" ht="26" customHeight="1">
-      <c r="A98" s="13" t="n"/>
-      <c r="B98" s="13" t="n"/>
-      <c r="C98" s="14" t="inlineStr">
+    <row r="98" ht="34" customHeight="1">
+      <c r="A98" s="15" t="inlineStr">
+        <is>
+          <t>Hạn xử lý nhu cầu KH</t>
+        </is>
+      </c>
+      <c r="B98" s="15" t="inlineStr">
+        <is>
+          <t>CHẶN TẠO DỰ ÁN TKT TỪ NHU CẦU ĐÃ ĐÓNG</t>
+        </is>
+      </c>
+      <c r="C98" s="16" t="inlineStr">
+        <is>
+          <t>TC_07.006</t>
+        </is>
+      </c>
+      <c r="D98" s="15" t="inlineStr">
+        <is>
+          <t>Nhu cầu đã có dự án thì hiện liên kết thay vì nút</t>
+        </is>
+      </c>
+      <c r="E98" s="16" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="F98" s="15" t="inlineStr">
+        <is>
+          <t>Nhu cầu #106 đã gắn dự án DA-02.</t>
+        </is>
+      </c>
+      <c r="G98" s="15" t="inlineStr">
+        <is>
+          <t>1. Xem cột Dự án TKT của dòng #106</t>
+        </is>
+      </c>
+      <c r="H98" s="15" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I98" s="15" t="inlineStr">
+        <is>
+          <t>- Hiện mã dự án bấm được, dẫn sang màn chi tiết dự án, không còn nút tạo mới</t>
+        </is>
+      </c>
+      <c r="J98" s="15" t="inlineStr"/>
+      <c r="K98" s="16" t="inlineStr">
+        <is>
+          <t>Not Executed</t>
+        </is>
+      </c>
+      <c r="L98" s="16" t="inlineStr">
+        <is>
+          <t>Not Executed</t>
+        </is>
+      </c>
+      <c r="M98" s="16" t="inlineStr">
+        <is>
+          <t>Not Executed</t>
+        </is>
+      </c>
+      <c r="N98" s="15" t="inlineStr"/>
+      <c r="O98" s="16" t="inlineStr"/>
+      <c r="P98" s="16" t="inlineStr"/>
+      <c r="Q98" s="16" t="inlineStr"/>
+    </row>
+    <row r="99" ht="26" customHeight="1">
+      <c r="A99" s="13" t="n"/>
+      <c r="B99" s="13" t="n"/>
+      <c r="C99" s="14" t="inlineStr">
         <is>
           <t>VIII. RÀNG BUỘC NHẬP LIỆU &amp; HIỂN THỊ TRẠNG THÁI</t>
         </is>
       </c>
-      <c r="D98" s="4" t="n"/>
-      <c r="E98" s="4" t="n"/>
-      <c r="F98" s="4" t="n"/>
-      <c r="G98" s="4" t="n"/>
-      <c r="H98" s="4" t="n"/>
-      <c r="I98" s="4" t="n"/>
-      <c r="J98" s="4" t="n"/>
-      <c r="K98" s="4" t="n"/>
-      <c r="L98" s="4" t="n"/>
-      <c r="M98" s="4" t="n"/>
-      <c r="N98" s="4" t="n"/>
-      <c r="O98" s="4" t="n"/>
-      <c r="P98" s="4" t="n"/>
-      <c r="Q98" s="5" t="n"/>
-    </row>
-    <row r="99" ht="53" customHeight="1">
-      <c r="A99" s="15" t="inlineStr">
-        <is>
-          <t>Hạn xử lý nhu cầu KH</t>
-        </is>
-      </c>
-      <c r="B99" s="15" t="inlineStr">
+      <c r="D99" s="4" t="n"/>
+      <c r="E99" s="4" t="n"/>
+      <c r="F99" s="4" t="n"/>
+      <c r="G99" s="4" t="n"/>
+      <c r="H99" s="4" t="n"/>
+      <c r="I99" s="4" t="n"/>
+      <c r="J99" s="4" t="n"/>
+      <c r="K99" s="4" t="n"/>
+      <c r="L99" s="4" t="n"/>
+      <c r="M99" s="4" t="n"/>
+      <c r="N99" s="4" t="n"/>
+      <c r="O99" s="4" t="n"/>
+      <c r="P99" s="4" t="n"/>
+      <c r="Q99" s="5" t="n"/>
+    </row>
+    <row r="100" ht="53" customHeight="1">
+      <c r="A100" s="15" t="inlineStr">
+        <is>
+          <t>Hạn xử lý nhu cầu KH</t>
+        </is>
+      </c>
+      <c r="B100" s="15" t="inlineStr">
         <is>
           <t>RÀNG BUỘC NHẬP LIỆU &amp; HIỂN THỊ TRẠNG THÁI</t>
         </is>
       </c>
-      <c r="C99" s="16" t="inlineStr">
+      <c r="C100" s="16" t="inlineStr">
         <is>
           <t>TC_08.001</t>
         </is>
       </c>
-      <c r="D99" s="15" t="inlineStr">
+      <c r="D100" s="15" t="inlineStr">
         <is>
           <t>Badge trạng thái của nhu cầu bị đóng</t>
         </is>
       </c>
-      <c r="E99" s="16" t="inlineStr">
+      <c r="E100" s="16" t="inlineStr">
         <is>
           <t>P0</t>
         </is>
       </c>
-      <c r="F99" s="15" t="inlineStr">
+      <c r="F100" s="15" t="inlineStr">
         <is>
           <t>Nhu cầu #301 vừa bị hệ thống đóng.</t>
         </is>
       </c>
-      <c r="G99" s="15" t="inlineStr">
+      <c r="G100" s="15" t="inlineStr">
         <is>
           <t>1. Xem cột Trạng thái của dòng #301 ở màn Nhu cầu khách hàng, ở thẻ Nhu cầu của khách hàng trong Công việc của tôi, và trong biên bản cuộc họp phát sinh nhu cầu</t>
         </is>
       </c>
-      <c r="H99" s="15" t="inlineStr">
+      <c r="H100" s="15" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="I99" s="15" t="inlineStr">
+      <c r="I100" s="15" t="inlineStr">
         <is>
           <t>- Cả 3 nơi đều hiện cùng một nhãn trạng thái màu xám
 - LƯU Ý: Hệ thống đang ghi 'Đóng' trong khi yêu cầu gốc ghi 'Đã đóng' — ghi nhận để chốt lại, không tự sửa</t>
-        </is>
-      </c>
-      <c r="J99" s="15" t="inlineStr"/>
-      <c r="K99" s="16" t="inlineStr">
-        <is>
-          <t>Not Executed</t>
-        </is>
-      </c>
-      <c r="L99" s="16" t="inlineStr">
-        <is>
-          <t>Not Executed</t>
-        </is>
-      </c>
-      <c r="M99" s="16" t="inlineStr">
-        <is>
-          <t>Not Executed</t>
-        </is>
-      </c>
-      <c r="N99" s="15" t="inlineStr"/>
-      <c r="O99" s="16" t="inlineStr"/>
-      <c r="P99" s="16" t="inlineStr"/>
-      <c r="Q99" s="16" t="inlineStr"/>
-    </row>
-    <row r="100" ht="45" customHeight="1">
-      <c r="A100" s="15" t="inlineStr">
-        <is>
-          <t>Hạn xử lý nhu cầu KH</t>
-        </is>
-      </c>
-      <c r="B100" s="15" t="inlineStr">
-        <is>
-          <t>RÀNG BUỘC NHẬP LIỆU &amp; HIỂN THỊ TRẠNG THÁI</t>
-        </is>
-      </c>
-      <c r="C100" s="16" t="inlineStr">
-        <is>
-          <t>TC_08.002</t>
-        </is>
-      </c>
-      <c r="D100" s="15" t="inlineStr">
-        <is>
-          <t>Ô N chỉ nhận số nguyên không âm ở mọi đường ghi</t>
-        </is>
-      </c>
-      <c r="E100" s="16" t="inlineStr">
-        <is>
-          <t>P0</t>
-        </is>
-      </c>
-      <c r="F100" s="15" t="inlineStr">
-        <is>
-          <t>Tài khoản có quyền quản lý danh mục.</t>
-        </is>
-      </c>
-      <c r="G100" s="15" t="inlineStr">
-        <is>
-          <t>1. Gọi thẳng chức năng Sửa lĩnh vực với số ngày hiệu lực = -1, bỏ qua giao diện
-2. Lặp lại với giá trị 'abc' và 5000</t>
-        </is>
-      </c>
-      <c r="H100" s="15" t="inlineStr">
-        <is>
-          <t>Thời gian hiệu lực nhu cầu: -1 / abc / 5000</t>
-        </is>
-      </c>
-      <c r="I100" s="15" t="inlineStr">
-        <is>
-          <t>- Cả 3 lần đều bị từ chối kèm thông báo tương ứng (không âm, phải là số nguyên, tối đa 3650 ngày)
-- Giá trị cũ trong danh mục không đổi</t>
         </is>
       </c>
       <c r="J100" s="15" t="inlineStr"/>
@@ -6368,7 +6372,7 @@
       <c r="P100" s="16" t="inlineStr"/>
       <c r="Q100" s="16" t="inlineStr"/>
     </row>
-    <row r="101" ht="37" customHeight="1">
+    <row r="101" ht="45" customHeight="1">
       <c r="A101" s="15" t="inlineStr">
         <is>
           <t>Hạn xử lý nhu cầu KH</t>
@@ -6381,12 +6385,12 @@
       </c>
       <c r="C101" s="16" t="inlineStr">
         <is>
-          <t>TC_08.003</t>
+          <t>TC_08.002</t>
         </is>
       </c>
       <c r="D101" s="15" t="inlineStr">
         <is>
-          <t>Bỏ trống N khi gọi thẳng chức năng</t>
+          <t>Ô N chỉ nhận số nguyên không âm ở mọi đường ghi</t>
         </is>
       </c>
       <c r="E101" s="16" t="inlineStr">
@@ -6396,23 +6400,24 @@
       </c>
       <c r="F101" s="15" t="inlineStr">
         <is>
-          <t>Lĩnh vực LVCTKD.0001 đang N = 30.</t>
+          <t>Tài khoản có quyền quản lý danh mục.</t>
         </is>
       </c>
       <c r="G101" s="15" t="inlineStr">
         <is>
-          <t>1. Gọi thẳng chức năng Sửa lĩnh vực, không gửi số ngày hiệu lực</t>
+          <t>1. Gọi thẳng chức năng Sửa lĩnh vực với số ngày hiệu lực = -1, bỏ qua giao diện
+2. Lặp lại với giá trị 'abc' và 5000</t>
         </is>
       </c>
       <c r="H101" s="15" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Thời gian hiệu lực nhu cầu: -1 / abc / 5000</t>
         </is>
       </c>
       <c r="I101" s="15" t="inlineStr">
         <is>
-          <t>- Bị từ chối với thông báo bắt buộc phải nhập
-- LƯU Ý: Không được ngầm hiểu thành 0 rồi tắt hạn của cả lĩnh vực</t>
+          <t>- Cả 3 lần đều bị từ chối kèm thông báo tương ứng (không âm, phải là số nguyên, tối đa 3650 ngày)
+- Giá trị cũ trong danh mục không đổi</t>
         </is>
       </c>
       <c r="J101" s="15" t="inlineStr"/>
@@ -6436,7 +6441,7 @@
       <c r="P101" s="16" t="inlineStr"/>
       <c r="Q101" s="16" t="inlineStr"/>
     </row>
-    <row r="102" ht="34" customHeight="1">
+    <row r="102" ht="37" customHeight="1">
       <c r="A102" s="15" t="inlineStr">
         <is>
           <t>Hạn xử lý nhu cầu KH</t>
@@ -6449,27 +6454,27 @@
       </c>
       <c r="C102" s="16" t="inlineStr">
         <is>
-          <t>TC_08.004</t>
+          <t>TC_08.003</t>
         </is>
       </c>
       <c r="D102" s="15" t="inlineStr">
         <is>
-          <t>Lĩnh vực đang khoá không sửa được N</t>
+          <t>Bỏ trống N khi gọi thẳng chức năng</t>
         </is>
       </c>
       <c r="E102" s="16" t="inlineStr">
         <is>
-          <t>P1</t>
+          <t>P0</t>
         </is>
       </c>
       <c r="F102" s="15" t="inlineStr">
         <is>
-          <t>Lĩnh vực LVCTKD.T1 đang Khoá, N = 30.</t>
+          <t>Lĩnh vực LVCTKD.0001 đang N = 30.</t>
         </is>
       </c>
       <c r="G102" s="15" t="inlineStr">
         <is>
-          <t>1. Gọi thẳng chức năng Sửa lĩnh vực đó với N = 10</t>
+          <t>1. Gọi thẳng chức năng Sửa lĩnh vực, không gửi số ngày hiệu lực</t>
         </is>
       </c>
       <c r="H102" s="15" t="inlineStr">
@@ -6479,8 +6484,8 @@
       </c>
       <c r="I102" s="15" t="inlineStr">
         <is>
-          <t>- Bị từ chối vì bản ghi đang khoá, phải mở khoá trước
-- N vẫn là 30</t>
+          <t>- Bị từ chối với thông báo bắt buộc phải nhập
+- LƯU Ý: Không được ngầm hiểu thành 0 rồi tắt hạn của cả lĩnh vực</t>
         </is>
       </c>
       <c r="J102" s="15" t="inlineStr"/>
@@ -6504,7 +6509,7 @@
       <c r="P102" s="16" t="inlineStr"/>
       <c r="Q102" s="16" t="inlineStr"/>
     </row>
-    <row r="103" ht="63" customHeight="1">
+    <row r="103" ht="34" customHeight="1">
       <c r="A103" s="15" t="inlineStr">
         <is>
           <t>Hạn xử lý nhu cầu KH</t>
@@ -6517,28 +6522,27 @@
       </c>
       <c r="C103" s="16" t="inlineStr">
         <is>
-          <t>TC_08.005</t>
+          <t>TC_08.004</t>
         </is>
       </c>
       <c r="D103" s="15" t="inlineStr">
         <is>
-          <t>Xuất Excel danh mục có cột thời gian hiệu lực</t>
+          <t>Lĩnh vực đang khoá không sửa được N</t>
         </is>
       </c>
       <c r="E103" s="16" t="inlineStr">
         <is>
-          <t>P2</t>
+          <t>P1</t>
         </is>
       </c>
       <c r="F103" s="15" t="inlineStr">
         <is>
-          <t>Danh mục có lĩnh vực N = 30 và lĩnh vực N = 0.</t>
+          <t>Lĩnh vực LVCTKD.T1 đang Khoá, N = 30.</t>
         </is>
       </c>
       <c r="G103" s="15" t="inlineStr">
         <is>
-          <t>1. Bấm Xuất Excel ở màn danh mục
-2. Mở file</t>
+          <t>1. Gọi thẳng chức năng Sửa lĩnh vực đó với N = 10</t>
         </is>
       </c>
       <c r="H103" s="15" t="inlineStr">
@@ -6548,8 +6552,8 @@
       </c>
       <c r="I103" s="15" t="inlineStr">
         <is>
-          <t>- Nếu file có cột thời gian hiệu lực thì giá trị phải khớp bảng (30 và 'Không giới hạn thời gian hiệu lực'/0)
-- Nếu file không có cột này thì ghi nhận là điểm cần bổ sung, không phải lỗi chặn</t>
+          <t>- Bị từ chối vì bản ghi đang khoá, phải mở khoá trước
+- N vẫn là 30</t>
         </is>
       </c>
       <c r="J103" s="15" t="inlineStr"/>
@@ -6573,7 +6577,7 @@
       <c r="P103" s="16" t="inlineStr"/>
       <c r="Q103" s="16" t="inlineStr"/>
     </row>
-    <row r="104" ht="39" customHeight="1">
+    <row r="104" ht="63" customHeight="1">
       <c r="A104" s="15" t="inlineStr">
         <is>
           <t>Hạn xử lý nhu cầu KH</t>
@@ -6586,27 +6590,28 @@
       </c>
       <c r="C104" s="16" t="inlineStr">
         <is>
-          <t>TC_08.006</t>
+          <t>TC_08.005</t>
         </is>
       </c>
       <c r="D104" s="15" t="inlineStr">
         <is>
-          <t>Bỏ trống cả Mã, Tên và N thì cả 3 ô đều báo lỗi</t>
+          <t>Xuất Excel danh mục có cột thời gian hiệu lực</t>
         </is>
       </c>
       <c r="E104" s="16" t="inlineStr">
         <is>
-          <t>P0</t>
+          <t>P2</t>
         </is>
       </c>
       <c r="F104" s="15" t="inlineStr">
         <is>
-          <t>Đang mở form Thêm mới lĩnh vực, chưa nhập gì.</t>
+          <t>Danh mục có lĩnh vực N = 30 và lĩnh vực N = 0.</t>
         </is>
       </c>
       <c r="G104" s="15" t="inlineStr">
         <is>
-          <t>1. Bấm Lưu ngay khi form còn trống</t>
+          <t>1. Bấm Xuất Excel ở màn danh mục
+2. Mở file</t>
         </is>
       </c>
       <c r="H104" s="15" t="inlineStr">
@@ -6616,8 +6621,8 @@
       </c>
       <c r="I104" s="15" t="inlineStr">
         <is>
-          <t>- CẢ 3 ô Mã, Tên, Thời gian hiệu lực đều viền đỏ kèm text lỗi
-- LƯU Ý: Không được chỉ mỗi ô Thời gian hiệu lực báo đỏ</t>
+          <t>- Nếu file có cột thời gian hiệu lực thì giá trị phải khớp bảng (30 và 'Không giới hạn thời gian hiệu lực'/0)
+- Nếu file không có cột này thì ghi nhận là điểm cần bổ sung, không phải lỗi chặn</t>
         </is>
       </c>
       <c r="J104" s="15" t="inlineStr"/>
@@ -6641,7 +6646,7 @@
       <c r="P104" s="16" t="inlineStr"/>
       <c r="Q104" s="16" t="inlineStr"/>
     </row>
-    <row r="105" ht="38" customHeight="1">
+    <row r="105" ht="39" customHeight="1">
       <c r="A105" s="15" t="inlineStr">
         <is>
           <t>Hạn xử lý nhu cầu KH</t>
@@ -6654,12 +6659,12 @@
       </c>
       <c r="C105" s="16" t="inlineStr">
         <is>
-          <t>TC_08.007</t>
+          <t>TC_08.006</t>
         </is>
       </c>
       <c r="D105" s="15" t="inlineStr">
         <is>
-          <t>Câu báo lỗi khi bỏ trống N và M</t>
+          <t>Bỏ trống cả Mã, Tên và N thì cả 3 ô đều báo lỗi</t>
         </is>
       </c>
       <c r="E105" s="16" t="inlineStr">
@@ -6669,13 +6674,12 @@
       </c>
       <c r="F105" s="15" t="inlineStr">
         <is>
-          <t>Form lĩnh vực và màn Cấu hình chung › Cấu hình hạn.</t>
+          <t>Đang mở form Thêm mới lĩnh vực, chưa nhập gì.</t>
         </is>
       </c>
       <c r="G105" s="15" t="inlineStr">
         <is>
-          <t>1. Xoá trắng ô Thời gian hiệu lực nhu cầu rồi bấm Lưu
-2. Xoá trắng ô Cảnh báo trước khi đóng nhu cầu rồi bấm Lưu</t>
+          <t>1. Bấm Lưu ngay khi form còn trống</t>
         </is>
       </c>
       <c r="H105" s="15" t="inlineStr">
@@ -6685,8 +6689,8 @@
       </c>
       <c r="I105" s="15" t="inlineStr">
         <is>
-          <t>- Cả 2 ô báo đúng câu: 'Bắt buộc nhập, kiểu số nguyên dương &gt;= 0'
-- Không báo tiếng Anh, không báo câu chung chung</t>
+          <t>- CẢ 3 ô Mã, Tên, Thời gian hiệu lực đều viền đỏ kèm text lỗi
+- LƯU Ý: Không được chỉ mỗi ô Thời gian hiệu lực báo đỏ</t>
         </is>
       </c>
       <c r="J105" s="15" t="inlineStr"/>
@@ -6710,7 +6714,7 @@
       <c r="P105" s="16" t="inlineStr"/>
       <c r="Q105" s="16" t="inlineStr"/>
     </row>
-    <row r="106" ht="46" customHeight="1">
+    <row r="106" ht="38" customHeight="1">
       <c r="A106" s="15" t="inlineStr">
         <is>
           <t>Hạn xử lý nhu cầu KH</t>
@@ -6723,12 +6727,12 @@
       </c>
       <c r="C106" s="16" t="inlineStr">
         <is>
-          <t>TC_08.008</t>
+          <t>TC_08.007</t>
         </is>
       </c>
       <c r="D106" s="15" t="inlineStr">
         <is>
-          <t>Ô M không nhận số âm</t>
+          <t>Câu báo lỗi khi bỏ trống N và M</t>
         </is>
       </c>
       <c r="E106" s="16" t="inlineStr">
@@ -6738,26 +6742,24 @@
       </c>
       <c r="F106" s="15" t="inlineStr">
         <is>
-          <t>Màn Cấu hình chung › thẻ Quản lý dự án › thẻ con Cấu hình hạn.</t>
+          <t>Form lĩnh vực và màn Cấu hình chung › Cấu hình hạn.</t>
         </is>
       </c>
       <c r="G106" s="15" t="inlineStr">
         <is>
-          <t>1. Gõ dấu trừ vào ô Cảnh báo trước khi đóng nhu cầu
-2. Thử dán giá trị -5 vào ô đó
-3. Bấm Lưu</t>
+          <t>1. Xoá trắng ô Thời gian hiệu lực nhu cầu rồi bấm Lưu
+2. Xoá trắng ô Cảnh báo trước khi đóng nhu cầu rồi bấm Lưu</t>
         </is>
       </c>
       <c r="H106" s="15" t="inlineStr">
         <is>
-          <t>Cảnh báo trước khi đóng nhu cầu: -5</t>
+          <t>—</t>
         </is>
       </c>
       <c r="I106" s="15" t="inlineStr">
         <is>
-          <t>- Bước 1: bàn phím KHÔNG gõ được dấu trừ
-- Bước 2: dán không vào
-- LƯU Ý: Hệ thống KHÔNG được tự kéo giá trị về 0, phải báo đỏ và chặn lưu</t>
+          <t>- Cả 2 ô báo đúng câu: 'Bắt buộc nhập, kiểu số nguyên dương &gt;= 0'
+- Không báo tiếng Anh, không báo câu chung chung</t>
         </is>
       </c>
       <c r="J106" s="15" t="inlineStr"/>
@@ -6781,7 +6783,7 @@
       <c r="P106" s="16" t="inlineStr"/>
       <c r="Q106" s="16" t="inlineStr"/>
     </row>
-    <row r="107" ht="34" customHeight="1">
+    <row r="107" ht="46" customHeight="1">
       <c r="A107" s="15" t="inlineStr">
         <is>
           <t>Hạn xử lý nhu cầu KH</t>
@@ -6794,39 +6796,41 @@
       </c>
       <c r="C107" s="16" t="inlineStr">
         <is>
-          <t>TC_08.009</t>
+          <t>TC_08.008</t>
         </is>
       </c>
       <c r="D107" s="15" t="inlineStr">
         <is>
-          <t>Ô N và M không nhận ký tự e, E, dấu cộng</t>
+          <t>Ô M không nhận số âm</t>
         </is>
       </c>
       <c r="E107" s="16" t="inlineStr">
         <is>
-          <t>P1</t>
+          <t>P0</t>
         </is>
       </c>
       <c r="F107" s="15" t="inlineStr">
         <is>
-          <t>Form lĩnh vực và màn Cấu hình hạn.</t>
+          <t>Màn Cấu hình chung › thẻ Quản lý dự án › thẻ con Cấu hình hạn.</t>
         </is>
       </c>
       <c r="G107" s="15" t="inlineStr">
         <is>
-          <t>1. Gõ 1e3333 vào ô Thời gian hiệu lực nhu cầu
-2. Làm tương tự với ô Cảnh báo trước khi đóng</t>
+          <t>1. Gõ dấu trừ vào ô Cảnh báo trước khi đóng nhu cầu
+2. Thử dán giá trị -5 vào ô đó
+3. Bấm Lưu</t>
         </is>
       </c>
       <c r="H107" s="15" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Cảnh báo trước khi đóng nhu cầu: -5</t>
         </is>
       </c>
       <c r="I107" s="15" t="inlineStr">
         <is>
-          <t>- Không gõ được e, E, dấu cộng
-- Ô không bị rỗng trắng sau khi gõ, giá trị giữ đúng phần số đã nhập</t>
+          <t>- Bước 1: bàn phím KHÔNG gõ được dấu trừ
+- Bước 2: dán không vào
+- LƯU Ý: Hệ thống KHÔNG được tự kéo giá trị về 0, phải báo đỏ và chặn lưu</t>
         </is>
       </c>
       <c r="J107" s="15" t="inlineStr"/>
@@ -6850,7 +6854,7 @@
       <c r="P107" s="16" t="inlineStr"/>
       <c r="Q107" s="16" t="inlineStr"/>
     </row>
-    <row r="108" ht="46" customHeight="1">
+    <row r="108" ht="34" customHeight="1">
       <c r="A108" s="15" t="inlineStr">
         <is>
           <t>Hạn xử lý nhu cầu KH</t>
@@ -6863,12 +6867,12 @@
       </c>
       <c r="C108" s="16" t="inlineStr">
         <is>
-          <t>TC_08.010</t>
+          <t>TC_08.009</t>
         </is>
       </c>
       <c r="D108" s="15" t="inlineStr">
         <is>
-          <t>Cột hạn hiện đủ chữ, không bị cắt</t>
+          <t>Ô N và M không nhận ký tự e, E, dấu cộng</t>
         </is>
       </c>
       <c r="E108" s="16" t="inlineStr">
@@ -6878,13 +6882,13 @@
       </c>
       <c r="F108" s="15" t="inlineStr">
         <is>
-          <t>Danh mục có lĩnh vực để N = 0; màn Nhu cầu khách hàng có nhu cầu thuộc lĩnh vực đó.</t>
+          <t>Form lĩnh vực và màn Cấu hình hạn.</t>
         </is>
       </c>
       <c r="G108" s="15" t="inlineStr">
         <is>
-          <t>1. Mở màn Danh mục › Lĩnh vực Công ty kinh doanh, xem cột Thời gian hiệu lực
-2. Mở màn Nhu cầu khách hàng, xem cột Thời gian hết hạn nhu cầu</t>
+          <t>1. Gõ 1e3333 vào ô Thời gian hiệu lực nhu cầu
+2. Làm tương tự với ô Cảnh báo trước khi đóng</t>
         </is>
       </c>
       <c r="H108" s="15" t="inlineStr">
@@ -6894,8 +6898,8 @@
       </c>
       <c r="I108" s="15" t="inlineStr">
         <is>
-          <t>- Cả 2 màn hiện ĐỦ cụm 'Không giới hạn thời gian hiệu lực'
-- LƯU Ý: Không bị cắt thành '...thời gian hiệu' kèm dấu ba chấm</t>
+          <t>- Không gõ được e, E, dấu cộng
+- Ô không bị rỗng trắng sau khi gõ, giá trị giữ đúng phần số đã nhập</t>
         </is>
       </c>
       <c r="J108" s="15" t="inlineStr"/>
@@ -6919,145 +6923,144 @@
       <c r="P108" s="16" t="inlineStr"/>
       <c r="Q108" s="16" t="inlineStr"/>
     </row>
-    <row r="109" ht="26" customHeight="1">
-      <c r="A109" s="13" t="n"/>
-      <c r="B109" s="13" t="n"/>
-      <c r="C109" s="14" t="inlineStr">
+    <row r="109" ht="46" customHeight="1">
+      <c r="A109" s="15" t="inlineStr">
+        <is>
+          <t>Hạn xử lý nhu cầu KH</t>
+        </is>
+      </c>
+      <c r="B109" s="15" t="inlineStr">
+        <is>
+          <t>RÀNG BUỘC NHẬP LIỆU &amp; HIỂN THỊ TRẠNG THÁI</t>
+        </is>
+      </c>
+      <c r="C109" s="16" t="inlineStr">
+        <is>
+          <t>TC_08.010</t>
+        </is>
+      </c>
+      <c r="D109" s="15" t="inlineStr">
+        <is>
+          <t>Cột hạn hiện đủ chữ, không bị cắt</t>
+        </is>
+      </c>
+      <c r="E109" s="16" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="F109" s="15" t="inlineStr">
+        <is>
+          <t>Danh mục có lĩnh vực để N = 0; màn Nhu cầu khách hàng có nhu cầu thuộc lĩnh vực đó.</t>
+        </is>
+      </c>
+      <c r="G109" s="15" t="inlineStr">
+        <is>
+          <t>1. Mở màn Danh mục › Lĩnh vực Công ty kinh doanh, xem cột Thời gian hiệu lực
+2. Mở màn Nhu cầu khách hàng, xem cột Thời gian hết hạn nhu cầu</t>
+        </is>
+      </c>
+      <c r="H109" s="15" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I109" s="15" t="inlineStr">
+        <is>
+          <t>- Cả 2 màn hiện ĐỦ cụm 'Không giới hạn thời gian hiệu lực'
+- LƯU Ý: Không bị cắt thành '...thời gian hiệu' kèm dấu ba chấm</t>
+        </is>
+      </c>
+      <c r="J109" s="15" t="inlineStr"/>
+      <c r="K109" s="16" t="inlineStr">
+        <is>
+          <t>Not Executed</t>
+        </is>
+      </c>
+      <c r="L109" s="16" t="inlineStr">
+        <is>
+          <t>Not Executed</t>
+        </is>
+      </c>
+      <c r="M109" s="16" t="inlineStr">
+        <is>
+          <t>Not Executed</t>
+        </is>
+      </c>
+      <c r="N109" s="15" t="inlineStr"/>
+      <c r="O109" s="16" t="inlineStr"/>
+      <c r="P109" s="16" t="inlineStr"/>
+      <c r="Q109" s="16" t="inlineStr"/>
+    </row>
+    <row r="110" ht="26" customHeight="1">
+      <c r="A110" s="13" t="n"/>
+      <c r="B110" s="13" t="n"/>
+      <c r="C110" s="14" t="inlineStr">
         <is>
           <t>IX. CÔ LẬP DỮ LIỆU &amp; THAO TÁC ĐỒNG THỜI</t>
         </is>
       </c>
-      <c r="D109" s="4" t="n"/>
-      <c r="E109" s="4" t="n"/>
-      <c r="F109" s="4" t="n"/>
-      <c r="G109" s="4" t="n"/>
-      <c r="H109" s="4" t="n"/>
-      <c r="I109" s="4" t="n"/>
-      <c r="J109" s="4" t="n"/>
-      <c r="K109" s="4" t="n"/>
-      <c r="L109" s="4" t="n"/>
-      <c r="M109" s="4" t="n"/>
-      <c r="N109" s="4" t="n"/>
-      <c r="O109" s="4" t="n"/>
-      <c r="P109" s="4" t="n"/>
-      <c r="Q109" s="5" t="n"/>
-    </row>
-    <row r="110" ht="48" customHeight="1">
-      <c r="A110" s="15" t="inlineStr">
-        <is>
-          <t>Hạn xử lý nhu cầu KH</t>
-        </is>
-      </c>
-      <c r="B110" s="15" t="inlineStr">
+      <c r="D110" s="4" t="n"/>
+      <c r="E110" s="4" t="n"/>
+      <c r="F110" s="4" t="n"/>
+      <c r="G110" s="4" t="n"/>
+      <c r="H110" s="4" t="n"/>
+      <c r="I110" s="4" t="n"/>
+      <c r="J110" s="4" t="n"/>
+      <c r="K110" s="4" t="n"/>
+      <c r="L110" s="4" t="n"/>
+      <c r="M110" s="4" t="n"/>
+      <c r="N110" s="4" t="n"/>
+      <c r="O110" s="4" t="n"/>
+      <c r="P110" s="4" t="n"/>
+      <c r="Q110" s="5" t="n"/>
+    </row>
+    <row r="111" ht="48" customHeight="1">
+      <c r="A111" s="15" t="inlineStr">
+        <is>
+          <t>Hạn xử lý nhu cầu KH</t>
+        </is>
+      </c>
+      <c r="B111" s="15" t="inlineStr">
         <is>
           <t>CÔ LẬP DỮ LIỆU &amp; THAO TÁC ĐỒNG THỜI</t>
         </is>
       </c>
-      <c r="C110" s="16" t="inlineStr">
+      <c r="C111" s="16" t="inlineStr">
         <is>
           <t>TC_09.001</t>
         </is>
       </c>
-      <c r="D110" s="15" t="inlineStr">
+      <c r="D111" s="15" t="inlineStr">
         <is>
           <t>Đổi N trong lúc nhu cầu đang chờ đóng</t>
         </is>
       </c>
-      <c r="E110" s="16" t="inlineStr">
+      <c r="E111" s="16" t="inlineStr">
         <is>
           <t>P0</t>
         </is>
       </c>
-      <c r="F110" s="15" t="inlineStr">
+      <c r="F111" s="15" t="inlineStr">
         <is>
           <t>Nhu cầu #431 hết hạn hôm nay, N chụp lúc tạo là 30.</t>
         </is>
       </c>
-      <c r="G110" s="15" t="inlineStr">
+      <c r="G111" s="15" t="inlineStr">
         <is>
           <t>1. Trước khi chạy quét, đổi N của lĩnh vực thành 60
 2. Chạy lệnh quét hạn nhu cầu</t>
         </is>
       </c>
-      <c r="H110" s="15" t="inlineStr">
+      <c r="H111" s="15" t="inlineStr">
         <is>
           <t>Thời gian hiệu lực nhu cầu: 30 -&gt; 60</t>
         </is>
       </c>
-      <c r="I110" s="15" t="inlineStr">
+      <c r="I111" s="15" t="inlineStr">
         <is>
           <t>- LƯU Ý: Nhu cầu #431 VẪN BỊ ĐÓNG hôm nay — sửa N ở danh mục KHÔNG gia hạn được nhu cầu đang chạy
 - Cột hạn không đổi, vẫn là hạn tính theo N = 30</t>
-        </is>
-      </c>
-      <c r="J110" s="15" t="inlineStr"/>
-      <c r="K110" s="16" t="inlineStr">
-        <is>
-          <t>Not Executed</t>
-        </is>
-      </c>
-      <c r="L110" s="16" t="inlineStr">
-        <is>
-          <t>Not Executed</t>
-        </is>
-      </c>
-      <c r="M110" s="16" t="inlineStr">
-        <is>
-          <t>Not Executed</t>
-        </is>
-      </c>
-      <c r="N110" s="15" t="inlineStr"/>
-      <c r="O110" s="16" t="inlineStr"/>
-      <c r="P110" s="16" t="inlineStr"/>
-      <c r="Q110" s="16" t="inlineStr"/>
-    </row>
-    <row r="111" ht="34" customHeight="1">
-      <c r="A111" s="15" t="inlineStr">
-        <is>
-          <t>Hạn xử lý nhu cầu KH</t>
-        </is>
-      </c>
-      <c r="B111" s="15" t="inlineStr">
-        <is>
-          <t>CÔ LẬP DỮ LIỆU &amp; THAO TÁC ĐỒNG THỜI</t>
-        </is>
-      </c>
-      <c r="C111" s="16" t="inlineStr">
-        <is>
-          <t>TC_09.002</t>
-        </is>
-      </c>
-      <c r="D111" s="15" t="inlineStr">
-        <is>
-          <t>Đổi N nhỏ hơn KHÔNG làm nhu cầu quá hạn</t>
-        </is>
-      </c>
-      <c r="E111" s="16" t="inlineStr">
-        <is>
-          <t>P0</t>
-        </is>
-      </c>
-      <c r="F111" s="15" t="inlineStr">
-        <is>
-          <t>Nhu cầu #432 có cuộc họp Hoàn thành cách đây 40 ngày, N chụp lúc tạo là 60.</t>
-        </is>
-      </c>
-      <c r="G111" s="15" t="inlineStr">
-        <is>
-          <t>1. Đổi N của lĩnh vực xuống 30
-2. Xem cột hạn của #432
-3. Chạy lệnh quét hạn nhu cầu</t>
-        </is>
-      </c>
-      <c r="H111" s="15" t="inlineStr">
-        <is>
-          <t>Thời gian hiệu lực nhu cầu: 60 -&gt; 30</t>
-        </is>
-      </c>
-      <c r="I111" s="15" t="inlineStr">
-        <is>
-          <t>- LƯU Ý: Cột hạn KHÔNG đổi, vẫn tính theo N = 60 nên còn 20 ngày
-- Nhu cầu KHÔNG bị đóng</t>
         </is>
       </c>
       <c r="J111" s="15" t="inlineStr"/>
@@ -7094,39 +7097,40 @@
       </c>
       <c r="C112" s="16" t="inlineStr">
         <is>
-          <t>TC_09.003</t>
+          <t>TC_09.002</t>
         </is>
       </c>
       <c r="D112" s="15" t="inlineStr">
         <is>
-          <t>Đổi M khi nhu cầu đã được cảnh báo</t>
+          <t>Đổi N nhỏ hơn KHÔNG làm nhu cầu quá hạn</t>
         </is>
       </c>
       <c r="E112" s="16" t="inlineStr">
         <is>
-          <t>P1</t>
+          <t>P0</t>
         </is>
       </c>
       <c r="F112" s="15" t="inlineStr">
         <is>
-          <t>Nhu cầu #433 đã nhận cảnh báo khi M = 3.</t>
+          <t>Nhu cầu #432 có cuộc họp Hoàn thành cách đây 40 ngày, N chụp lúc tạo là 60.</t>
         </is>
       </c>
       <c r="G112" s="15" t="inlineStr">
         <is>
-          <t>1. Đổi M thành 10
-2. Chạy lại lệnh quét hạn nhu cầu</t>
+          <t>1. Đổi N của lĩnh vực xuống 30
+2. Xem cột hạn của #432
+3. Chạy lệnh quét hạn nhu cầu</t>
         </is>
       </c>
       <c r="H112" s="15" t="inlineStr">
         <is>
-          <t>Cảnh báo trước khi đóng nhu cầu: 3 -&gt; 10</t>
+          <t>Thời gian hiệu lực nhu cầu: 60 -&gt; 30</t>
         </is>
       </c>
       <c r="I112" s="15" t="inlineStr">
         <is>
-          <t>- Không gửi lại thông báo cho #433 (mỗi nhu cầu chỉ cảnh báo một lần)
-- Trên bảng, dòng vẫn tô cam</t>
+          <t>- LƯU Ý: Cột hạn KHÔNG đổi, vẫn tính theo N = 60 nên còn 20 ngày
+- Nhu cầu KHÔNG bị đóng</t>
         </is>
       </c>
       <c r="J112" s="15" t="inlineStr"/>
@@ -7163,38 +7167,39 @@
       </c>
       <c r="C113" s="16" t="inlineStr">
         <is>
-          <t>TC_09.004</t>
+          <t>TC_09.003</t>
         </is>
       </c>
       <c r="D113" s="15" t="inlineStr">
         <is>
-          <t>Người dùng lập dự án ngay trước giờ quét</t>
+          <t>Đổi M khi nhu cầu đã được cảnh báo</t>
         </is>
       </c>
       <c r="E113" s="16" t="inlineStr">
         <is>
-          <t>P0</t>
+          <t>P1</t>
         </is>
       </c>
       <c r="F113" s="15" t="inlineStr">
         <is>
-          <t>Nhu cầu #434 hết hạn hôm nay; người dùng lập Dự án TKT từ nhu cầu này lúc 23:50.</t>
+          <t>Nhu cầu #433 thuộc lĩnh vực có N = 30, đã nhận cảnh báo khi M = 3.</t>
         </is>
       </c>
       <c r="G113" s="15" t="inlineStr">
         <is>
-          <t>1. Chạy lệnh quét hạn nhu cầu sau đó
-2. Kiểm tra #434</t>
+          <t>1. Đổi M thành 10
+2. Chạy lại lệnh quét hạn nhu cầu</t>
         </is>
       </c>
       <c r="H113" s="15" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Cảnh báo trước khi đóng nhu cầu: 3 -&gt; 10</t>
         </is>
       </c>
       <c r="I113" s="15" t="inlineStr">
         <is>
-          <t>- Không bị đóng, trạng thái là 'Đã lập dự án TKT'</t>
+          <t>- Không gửi lại thông báo cho #433 (mỗi nhu cầu chỉ cảnh báo một lần)
+- Trên bảng, dòng vẫn tô cam</t>
         </is>
       </c>
       <c r="J113" s="15" t="inlineStr"/>
@@ -7231,27 +7236,28 @@
       </c>
       <c r="C114" s="16" t="inlineStr">
         <is>
-          <t>TC_09.005</t>
+          <t>TC_09.004</t>
         </is>
       </c>
       <c r="D114" s="15" t="inlineStr">
         <is>
-          <t>Hai người cùng thao tác trên một nhu cầu</t>
+          <t>Người dùng lập dự án ngay trước giờ quét</t>
         </is>
       </c>
       <c r="E114" s="16" t="inlineStr">
         <is>
-          <t>P1</t>
+          <t>P0</t>
         </is>
       </c>
       <c r="F114" s="15" t="inlineStr">
         <is>
-          <t>Người 1 đang mở form lập dự án từ nhu cầu #435; người 2 đóng tay nhu cầu đó.</t>
+          <t>Nhu cầu #434 hết hạn hôm nay; người dùng lập Dự án TKT từ nhu cầu này lúc 23:50.</t>
         </is>
       </c>
       <c r="G114" s="15" t="inlineStr">
         <is>
-          <t>1. Người 1 bấm Lưu form lập dự án</t>
+          <t>1. Chạy lệnh quét hạn nhu cầu sau đó
+2. Kiểm tra #434</t>
         </is>
       </c>
       <c r="H114" s="15" t="inlineStr">
@@ -7261,8 +7267,7 @@
       </c>
       <c r="I114" s="15" t="inlineStr">
         <is>
-          <t>- Bị chặn kèm thông báo nhu cầu đã đóng, không tạo dự án
-- Màn không treo</t>
+          <t>- Không bị đóng, trạng thái là 'Đã lập dự án TKT'</t>
         </is>
       </c>
       <c r="J114" s="15" t="inlineStr"/>
@@ -7299,12 +7304,12 @@
       </c>
       <c r="C115" s="16" t="inlineStr">
         <is>
-          <t>TC_09.006</t>
+          <t>TC_09.005</t>
         </is>
       </c>
       <c r="D115" s="15" t="inlineStr">
         <is>
-          <t>Quét chạy khi hệ thống chưa có cấu hình M</t>
+          <t>Hai người cùng thao tác trên một nhu cầu</t>
         </is>
       </c>
       <c r="E115" s="16" t="inlineStr">
@@ -7314,12 +7319,12 @@
       </c>
       <c r="F115" s="15" t="inlineStr">
         <is>
-          <t>Công ty của cuộc họp chưa từng lưu cấu hình hạn.</t>
+          <t>Người 1 đang mở form lập dự án từ nhu cầu #435; người 2 đóng tay nhu cầu đó.</t>
         </is>
       </c>
       <c r="G115" s="15" t="inlineStr">
         <is>
-          <t>1. Chạy lệnh quét hạn nhu cầu với 1 nhu cầu còn 2 ngày tới hạn (N = 30)</t>
+          <t>1. Người 1 bấm Lưu form lập dự án</t>
         </is>
       </c>
       <c r="H115" s="15" t="inlineStr">
@@ -7329,8 +7334,8 @@
       </c>
       <c r="I115" s="15" t="inlineStr">
         <is>
-          <t>- Hệ thống dùng mặc định 3 ngày: nhu cầu vẫn được cảnh báo
-- Không văng lỗi vì thiếu cấu hình</t>
+          <t>- Bị chặn kèm thông báo nhu cầu đã đóng, không tạo dự án
+- Màn không treo</t>
         </is>
       </c>
       <c r="J115" s="15" t="inlineStr"/>
@@ -7367,27 +7372,27 @@
       </c>
       <c r="C116" s="16" t="inlineStr">
         <is>
-          <t>TC_09.007</t>
+          <t>TC_09.006</t>
         </is>
       </c>
       <c r="D116" s="15" t="inlineStr">
         <is>
-          <t>Cuộc họp bị xoá hoặc thiếu người chủ trì</t>
+          <t>Quét chạy khi hệ thống chưa có cấu hình M</t>
         </is>
       </c>
       <c r="E116" s="16" t="inlineStr">
         <is>
-          <t>P2</t>
+          <t>P1</t>
         </is>
       </c>
       <c r="F116" s="15" t="inlineStr">
         <is>
-          <t>Nhu cầu #436 tới vùng cảnh báo nhưng cuộc họp không xác định được người chủ trì lẫn người tạo.</t>
+          <t>Công ty của cuộc họp chưa từng lưu cấu hình hạn.</t>
         </is>
       </c>
       <c r="G116" s="15" t="inlineStr">
         <is>
-          <t>1. Chạy lệnh quét hạn nhu cầu</t>
+          <t>1. Chạy lệnh quét hạn nhu cầu với 1 nhu cầu còn 2 ngày tới hạn (N = 30)</t>
         </is>
       </c>
       <c r="H116" s="15" t="inlineStr">
@@ -7397,7 +7402,8 @@
       </c>
       <c r="I116" s="15" t="inlineStr">
         <is>
-          <t>- Không gửi được thông báo nhưng lệnh vẫn chạy hết, các nhu cầu khác vẫn được xử lý bình thường</t>
+          <t>- Hệ thống dùng mặc định 3 ngày: nhu cầu vẫn được cảnh báo
+- Không văng lỗi vì thiếu cấu hình</t>
         </is>
       </c>
       <c r="J116" s="15" t="inlineStr"/>
@@ -7421,61 +7427,128 @@
       <c r="P116" s="16" t="inlineStr"/>
       <c r="Q116" s="16" t="inlineStr"/>
     </row>
-    <row r="117" ht="26" customHeight="1">
-      <c r="A117" s="13" t="n"/>
-      <c r="B117" s="13" t="n"/>
-      <c r="C117" s="14" t="inlineStr">
+    <row r="117" ht="34" customHeight="1">
+      <c r="A117" s="15" t="inlineStr">
+        <is>
+          <t>Hạn xử lý nhu cầu KH</t>
+        </is>
+      </c>
+      <c r="B117" s="15" t="inlineStr">
+        <is>
+          <t>CÔ LẬP DỮ LIỆU &amp; THAO TÁC ĐỒNG THỜI</t>
+        </is>
+      </c>
+      <c r="C117" s="16" t="inlineStr">
+        <is>
+          <t>TC_09.007</t>
+        </is>
+      </c>
+      <c r="D117" s="15" t="inlineStr">
+        <is>
+          <t>Cuộc họp bị xoá hoặc thiếu người chủ trì</t>
+        </is>
+      </c>
+      <c r="E117" s="16" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="F117" s="15" t="inlineStr">
+        <is>
+          <t>Nhu cầu #436 tới vùng cảnh báo nhưng cuộc họp không xác định được người chủ trì lẫn người tạo.</t>
+        </is>
+      </c>
+      <c r="G117" s="15" t="inlineStr">
+        <is>
+          <t>1. Chạy lệnh quét hạn nhu cầu</t>
+        </is>
+      </c>
+      <c r="H117" s="15" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I117" s="15" t="inlineStr">
+        <is>
+          <t>- Không gửi được thông báo nhưng lệnh vẫn chạy hết, các nhu cầu khác vẫn được xử lý bình thường</t>
+        </is>
+      </c>
+      <c r="J117" s="15" t="inlineStr"/>
+      <c r="K117" s="16" t="inlineStr">
+        <is>
+          <t>Not Executed</t>
+        </is>
+      </c>
+      <c r="L117" s="16" t="inlineStr">
+        <is>
+          <t>Not Executed</t>
+        </is>
+      </c>
+      <c r="M117" s="16" t="inlineStr">
+        <is>
+          <t>Not Executed</t>
+        </is>
+      </c>
+      <c r="N117" s="15" t="inlineStr"/>
+      <c r="O117" s="16" t="inlineStr"/>
+      <c r="P117" s="16" t="inlineStr"/>
+      <c r="Q117" s="16" t="inlineStr"/>
+    </row>
+    <row r="118" ht="26" customHeight="1">
+      <c r="A118" s="13" t="n"/>
+      <c r="B118" s="13" t="n"/>
+      <c r="C118" s="14" t="inlineStr">
         <is>
           <t>X. E2E FLOW</t>
         </is>
       </c>
-      <c r="D117" s="4" t="n"/>
-      <c r="E117" s="4" t="n"/>
-      <c r="F117" s="4" t="n"/>
-      <c r="G117" s="4" t="n"/>
-      <c r="H117" s="4" t="n"/>
-      <c r="I117" s="4" t="n"/>
-      <c r="J117" s="4" t="n"/>
-      <c r="K117" s="4" t="n"/>
-      <c r="L117" s="4" t="n"/>
-      <c r="M117" s="4" t="n"/>
-      <c r="N117" s="4" t="n"/>
-      <c r="O117" s="4" t="n"/>
-      <c r="P117" s="4" t="n"/>
-      <c r="Q117" s="5" t="n"/>
-    </row>
-    <row r="118" ht="87" customHeight="1">
-      <c r="A118" s="15" t="inlineStr">
-        <is>
-          <t>Hạn xử lý nhu cầu KH</t>
-        </is>
-      </c>
-      <c r="B118" s="15" t="inlineStr">
+      <c r="D118" s="4" t="n"/>
+      <c r="E118" s="4" t="n"/>
+      <c r="F118" s="4" t="n"/>
+      <c r="G118" s="4" t="n"/>
+      <c r="H118" s="4" t="n"/>
+      <c r="I118" s="4" t="n"/>
+      <c r="J118" s="4" t="n"/>
+      <c r="K118" s="4" t="n"/>
+      <c r="L118" s="4" t="n"/>
+      <c r="M118" s="4" t="n"/>
+      <c r="N118" s="4" t="n"/>
+      <c r="O118" s="4" t="n"/>
+      <c r="P118" s="4" t="n"/>
+      <c r="Q118" s="5" t="n"/>
+    </row>
+    <row r="119" ht="87" customHeight="1">
+      <c r="A119" s="15" t="inlineStr">
+        <is>
+          <t>Hạn xử lý nhu cầu KH</t>
+        </is>
+      </c>
+      <c r="B119" s="15" t="inlineStr">
         <is>
           <t>E2E FLOW</t>
         </is>
       </c>
-      <c r="C118" s="16" t="inlineStr">
+      <c r="C119" s="16" t="inlineStr">
         <is>
           <t>TC_10.001</t>
         </is>
       </c>
-      <c r="D118" s="15" t="inlineStr">
+      <c r="D119" s="15" t="inlineStr">
         <is>
           <t>Luồng đầy đủ: khai N và M -&gt; cảnh báo -&gt; tự đóng -&gt; chặn lập dự án</t>
         </is>
       </c>
-      <c r="E118" s="16" t="inlineStr">
+      <c r="E119" s="16" t="inlineStr">
         <is>
           <t>P0</t>
         </is>
       </c>
-      <c r="F118" s="15" t="inlineStr">
+      <c r="F119" s="15" t="inlineStr">
         <is>
           <t>Lĩnh vực LVCTKD.E2E đang N = 0; cuộc họp M-E2E có 1 nhu cầu, chưa Hoàn thành; M = 3.</t>
         </is>
       </c>
-      <c r="G118" s="15" t="inlineStr">
+      <c r="G119" s="15" t="inlineStr">
         <is>
           <t>1. Khai N = 5 cho lĩnh vực LVCTKD.E2E
 2. Chuyển cuộc họp M-E2E sang Hoàn thành
@@ -7485,12 +7558,12 @@
 6. Thử lập Dự án TKT từ nhu cầu đó</t>
         </is>
       </c>
-      <c r="H118" s="15" t="inlineStr">
+      <c r="H119" s="15" t="inlineStr">
         <is>
           <t>Thời gian hiệu lực nhu cầu: 5 · Cảnh báo trước khi đóng: 3</t>
         </is>
       </c>
-      <c r="I118" s="15" t="inlineStr">
+      <c r="I119" s="15" t="inlineStr">
         <is>
           <t>- Bước 3: cột hạn = ngày Hoàn thành + 5 ngày
 - Bước 4: người chủ trì nhận 1 thông báo, dòng tô cam '(còn 3 ngày)'
@@ -7498,59 +7571,59 @@
 - Bước 6: không còn nút Tạo Dự án TKT; gọi thẳng chức năng thì bị chặn đúng câu thông báo</t>
         </is>
       </c>
-      <c r="J118" s="15" t="inlineStr"/>
-      <c r="K118" s="16" t="inlineStr">
-        <is>
-          <t>Not Executed</t>
-        </is>
-      </c>
-      <c r="L118" s="16" t="inlineStr">
-        <is>
-          <t>Not Executed</t>
-        </is>
-      </c>
-      <c r="M118" s="16" t="inlineStr">
-        <is>
-          <t>Not Executed</t>
-        </is>
-      </c>
-      <c r="N118" s="15" t="inlineStr"/>
-      <c r="O118" s="16" t="inlineStr"/>
-      <c r="P118" s="16" t="inlineStr"/>
-      <c r="Q118" s="16" t="inlineStr"/>
-    </row>
-    <row r="119" ht="47" customHeight="1">
-      <c r="A119" s="15" t="inlineStr">
-        <is>
-          <t>Hạn xử lý nhu cầu KH</t>
-        </is>
-      </c>
-      <c r="B119" s="15" t="inlineStr">
+      <c r="J119" s="15" t="inlineStr"/>
+      <c r="K119" s="16" t="inlineStr">
+        <is>
+          <t>Not Executed</t>
+        </is>
+      </c>
+      <c r="L119" s="16" t="inlineStr">
+        <is>
+          <t>Not Executed</t>
+        </is>
+      </c>
+      <c r="M119" s="16" t="inlineStr">
+        <is>
+          <t>Not Executed</t>
+        </is>
+      </c>
+      <c r="N119" s="15" t="inlineStr"/>
+      <c r="O119" s="16" t="inlineStr"/>
+      <c r="P119" s="16" t="inlineStr"/>
+      <c r="Q119" s="16" t="inlineStr"/>
+    </row>
+    <row r="120" ht="47" customHeight="1">
+      <c r="A120" s="15" t="inlineStr">
+        <is>
+          <t>Hạn xử lý nhu cầu KH</t>
+        </is>
+      </c>
+      <c r="B120" s="15" t="inlineStr">
         <is>
           <t>E2E FLOW</t>
         </is>
       </c>
-      <c r="C119" s="16" t="inlineStr">
+      <c r="C120" s="16" t="inlineStr">
         <is>
           <t>TC_10.002</t>
         </is>
       </c>
-      <c r="D119" s="15" t="inlineStr">
+      <c r="D120" s="15" t="inlineStr">
         <is>
           <t>Luồng lập dự án kịp hạn</t>
         </is>
       </c>
-      <c r="E119" s="16" t="inlineStr">
+      <c r="E120" s="16" t="inlineStr">
         <is>
           <t>P0</t>
         </is>
       </c>
-      <c r="F119" s="15" t="inlineStr">
-        <is>
-          <t>Nhu cầu #501 còn 2 ngày tới hạn, đã nhận cảnh báo.</t>
-        </is>
-      </c>
-      <c r="G119" s="15" t="inlineStr">
+      <c r="F120" s="15" t="inlineStr">
+        <is>
+          <t>Nhu cầu #501 thuộc lĩnh vực có N = 30 (M = 3), còn 2 ngày tới hạn, đã nhận cảnh báo.</t>
+        </is>
+      </c>
+      <c r="G120" s="15" t="inlineStr">
         <is>
           <t>1. Bấm nút Tạo Dự án TKT từ nhu cầu #501
 2. Lập dự án và lưu
@@ -7558,84 +7631,15 @@
 4. Chạy lệnh quét hạn nhu cầu sau ngày hết hạn</t>
         </is>
       </c>
-      <c r="H119" s="15" t="inlineStr">
+      <c r="H120" s="15" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="I119" s="15" t="inlineStr">
+      <c r="I120" s="15" t="inlineStr">
         <is>
           <t>- Sau bước 2: nhu cầu chuyển 'Đã lập dự án TKT', cột hạn thành 'Không giới hạn thời gian hiệu lực'
 - Sau bước 4: nhu cầu KHÔNG bị đóng</t>
-        </is>
-      </c>
-      <c r="J119" s="15" t="inlineStr"/>
-      <c r="K119" s="16" t="inlineStr">
-        <is>
-          <t>Not Executed</t>
-        </is>
-      </c>
-      <c r="L119" s="16" t="inlineStr">
-        <is>
-          <t>Not Executed</t>
-        </is>
-      </c>
-      <c r="M119" s="16" t="inlineStr">
-        <is>
-          <t>Not Executed</t>
-        </is>
-      </c>
-      <c r="N119" s="15" t="inlineStr"/>
-      <c r="O119" s="16" t="inlineStr"/>
-      <c r="P119" s="16" t="inlineStr"/>
-      <c r="Q119" s="16" t="inlineStr"/>
-    </row>
-    <row r="120" ht="38" customHeight="1">
-      <c r="A120" s="15" t="inlineStr">
-        <is>
-          <t>Hạn xử lý nhu cầu KH</t>
-        </is>
-      </c>
-      <c r="B120" s="15" t="inlineStr">
-        <is>
-          <t>E2E FLOW</t>
-        </is>
-      </c>
-      <c r="C120" s="16" t="inlineStr">
-        <is>
-          <t>TC_10.003</t>
-        </is>
-      </c>
-      <c r="D120" s="15" t="inlineStr">
-        <is>
-          <t>Luồng lĩnh vực không đặt thời hạn</t>
-        </is>
-      </c>
-      <c r="E120" s="16" t="inlineStr">
-        <is>
-          <t>P1</t>
-        </is>
-      </c>
-      <c r="F120" s="15" t="inlineStr">
-        <is>
-          <t>Lĩnh vực LVCTKD.KHAC để N = 0, có 10 nhu cầu cũ từ nhiều tháng trước.</t>
-        </is>
-      </c>
-      <c r="G120" s="15" t="inlineStr">
-        <is>
-          <t>1. Chạy lệnh quét hạn nhu cầu
-2. Xem 10 nhu cầu đó trên màn danh sách</t>
-        </is>
-      </c>
-      <c r="H120" s="15" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="I120" s="15" t="inlineStr">
-        <is>
-          <t>- Không nhu cầu nào bị đóng, không thông báo nào được gửi
-- Cả 10 dòng đều ghi 'Không giới hạn thời gian hiệu lực'</t>
         </is>
       </c>
       <c r="J120" s="15" t="inlineStr"/>
@@ -7659,7 +7663,7 @@
       <c r="P120" s="16" t="inlineStr"/>
       <c r="Q120" s="16" t="inlineStr"/>
     </row>
-    <row r="121" ht="49" customHeight="1">
+    <row r="121" ht="38" customHeight="1">
       <c r="A121" s="15" t="inlineStr">
         <is>
           <t>Hạn xử lý nhu cầu KH</t>
@@ -7672,12 +7676,12 @@
       </c>
       <c r="C121" s="16" t="inlineStr">
         <is>
-          <t>TC_10.004</t>
+          <t>TC_10.003</t>
         </is>
       </c>
       <c r="D121" s="15" t="inlineStr">
         <is>
-          <t>Luồng hai lĩnh vực hạn khác nhau trong cùng cuộc họp</t>
+          <t>Luồng lĩnh vực không đặt thời hạn</t>
         </is>
       </c>
       <c r="E121" s="16" t="inlineStr">
@@ -7687,13 +7691,13 @@
       </c>
       <c r="F121" s="15" t="inlineStr">
         <is>
-          <t>Cuộc họp M-E2E2 Hoàn thành 01/09/2026, phát sinh 2 nhu cầu: một thuộc lĩnh vực N = 10, một thuộc lĩnh vực N = 40.</t>
+          <t>Lĩnh vực LVCTKD.KHAC để N = 0, có 10 nhu cầu cũ từ nhiều tháng trước.</t>
         </is>
       </c>
       <c r="G121" s="15" t="inlineStr">
         <is>
-          <t>1. Xem cột hạn của 2 nhu cầu
-2. Chạy lệnh quét hạn nhu cầu vào ngày 11/09/2026</t>
+          <t>1. Chạy lệnh quét hạn nhu cầu
+2. Xem 10 nhu cầu đó trên màn danh sách</t>
         </is>
       </c>
       <c r="H121" s="15" t="inlineStr">
@@ -7703,8 +7707,8 @@
       </c>
       <c r="I121" s="15" t="inlineStr">
         <is>
-          <t>- Nhu cầu thứ nhất hạn 11/09/2026, nhu cầu thứ hai hạn 11/10/2026
-- Lần quét ngày 11/09 chỉ đóng nhu cầu thứ nhất, nhu cầu thứ hai vẫn Đang theo dõi</t>
+          <t>- Không nhu cầu nào bị đóng, không thông báo nào được gửi
+- Cả 10 dòng đều ghi 'Không giới hạn thời gian hiệu lực'</t>
         </is>
       </c>
       <c r="J121" s="15" t="inlineStr"/>
@@ -7728,15 +7732,84 @@
       <c r="P121" s="16" t="inlineStr"/>
       <c r="Q121" s="16" t="inlineStr"/>
     </row>
+    <row r="122" ht="49" customHeight="1">
+      <c r="A122" s="15" t="inlineStr">
+        <is>
+          <t>Hạn xử lý nhu cầu KH</t>
+        </is>
+      </c>
+      <c r="B122" s="15" t="inlineStr">
+        <is>
+          <t>E2E FLOW</t>
+        </is>
+      </c>
+      <c r="C122" s="16" t="inlineStr">
+        <is>
+          <t>TC_10.004</t>
+        </is>
+      </c>
+      <c r="D122" s="15" t="inlineStr">
+        <is>
+          <t>Luồng hai lĩnh vực hạn khác nhau trong cùng cuộc họp</t>
+        </is>
+      </c>
+      <c r="E122" s="16" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="F122" s="15" t="inlineStr">
+        <is>
+          <t>Cuộc họp M-E2E2 Hoàn thành 01/09/2026, phát sinh 2 nhu cầu: một thuộc lĩnh vực N = 10, một thuộc lĩnh vực N = 40.</t>
+        </is>
+      </c>
+      <c r="G122" s="15" t="inlineStr">
+        <is>
+          <t>1. Xem cột hạn của 2 nhu cầu
+2. Chạy lệnh quét hạn nhu cầu vào ngày 11/09/2026</t>
+        </is>
+      </c>
+      <c r="H122" s="15" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I122" s="15" t="inlineStr">
+        <is>
+          <t>- Nhu cầu thứ nhất hạn 11/09/2026, nhu cầu thứ hai hạn 11/10/2026
+- Lần quét ngày 11/09 chỉ đóng nhu cầu thứ nhất, nhu cầu thứ hai vẫn Đang theo dõi</t>
+        </is>
+      </c>
+      <c r="J122" s="15" t="inlineStr"/>
+      <c r="K122" s="16" t="inlineStr">
+        <is>
+          <t>Not Executed</t>
+        </is>
+      </c>
+      <c r="L122" s="16" t="inlineStr">
+        <is>
+          <t>Not Executed</t>
+        </is>
+      </c>
+      <c r="M122" s="16" t="inlineStr">
+        <is>
+          <t>Not Executed</t>
+        </is>
+      </c>
+      <c r="N122" s="15" t="inlineStr"/>
+      <c r="O122" s="16" t="inlineStr"/>
+      <c r="P122" s="16" t="inlineStr"/>
+      <c r="Q122" s="16" t="inlineStr"/>
+    </row>
   </sheetData>
   <mergeCells count="43">
-    <mergeCell ref="C109:Q109"/>
     <mergeCell ref="B9:N9"/>
     <mergeCell ref="I15:J15"/>
+    <mergeCell ref="C99:Q99"/>
     <mergeCell ref="K15:L15"/>
     <mergeCell ref="A11:E11"/>
     <mergeCell ref="I11:J11"/>
-    <mergeCell ref="C117:Q117"/>
+    <mergeCell ref="C118:Q118"/>
     <mergeCell ref="B6:N6"/>
     <mergeCell ref="A1:N1"/>
     <mergeCell ref="B5:N5"/>
@@ -7747,38 +7820,38 @@
     <mergeCell ref="O12:Q12"/>
     <mergeCell ref="C27:Q27"/>
     <mergeCell ref="C52:Q52"/>
+    <mergeCell ref="C71:Q71"/>
+    <mergeCell ref="C110:Q110"/>
     <mergeCell ref="B7:N7"/>
-    <mergeCell ref="C70:Q70"/>
     <mergeCell ref="B3:N3"/>
     <mergeCell ref="O11:Q11"/>
     <mergeCell ref="M13:N13"/>
-    <mergeCell ref="C91:Q91"/>
+    <mergeCell ref="C82:Q82"/>
     <mergeCell ref="I12:J12"/>
     <mergeCell ref="O14:Q14"/>
     <mergeCell ref="M15:N15"/>
     <mergeCell ref="K12:L12"/>
-    <mergeCell ref="C81:Q81"/>
     <mergeCell ref="M12:N12"/>
     <mergeCell ref="O13:Q13"/>
     <mergeCell ref="I14:J14"/>
     <mergeCell ref="C18:Q18"/>
     <mergeCell ref="K14:L14"/>
     <mergeCell ref="B2:N2"/>
+    <mergeCell ref="C92:Q92"/>
     <mergeCell ref="O15:Q15"/>
     <mergeCell ref="B8:N8"/>
     <mergeCell ref="C58:Q58"/>
     <mergeCell ref="M14:N14"/>
-    <mergeCell ref="C98:Q98"/>
     <mergeCell ref="I13:J13"/>
     <mergeCell ref="F11:H15"/>
     <mergeCell ref="K13:L13"/>
     <mergeCell ref="B10:N10"/>
   </mergeCells>
   <dataValidations count="2">
-    <dataValidation sqref="K18:M171" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="K18:M172" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Passed,Failed,Pending,Not Executed"</formula1>
     </dataValidation>
-    <dataValidation sqref="O18:Q171" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="O18:Q172" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"P,F,PE"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>

<commit_message>
docs(11377): tach ro 2 luong - to cam man danh sach vs thong bao chuong
Ngoai le "N <= M thi bo qua" chi ap cho LUONG GUI THONG BAO (gach con cua
"Luong 1" trong mo ta Redmine), khong ap cho cot han o man danh sach.

- Mo ta nghiep vu: doi "luong CANH BAO" -> "luong GUI THONG BAO"
- Khoi "Ghi chu doc bang": viet lai thanh 2 muc (a) to cam - khong phu thuoc
  N > M, vung canh bao TICH LUY; (b) thong bao chuong - co ngoai le N <= M
- TC_04.011: bo ghi chu sai, them y "moi dong con duoi 7 ngay deu phai to cam"
- TC_04.012: viet lai han - truoc ghi "nang M vuot qua N thi canh bao TAT di"
  (sai), nay la "nhu cau co N nho hon M VAN to cam tren man hinh, chi khong
  nhan duoc thong bao chuong"
- design.md: them muc 1b ghi lai sai lam nay va bang luat dung cho tung noi

Refs #11377

Co-Authored-By: Claude Opus 5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/hrm/.plans/canh-bao-tu-dong-dong-nhu-cau/testcase.xlsx
+++ b/hrm/.plans/canh-bao-tu-dong-dong-nhu-cau/testcase.xlsx
@@ -667,7 +667,7 @@
 - Nhu cầu mà cuộc họp chưa Hoàn thành (chưa có mốc T);
 - Nhu cầu đã lập Dự án TKT;
 - Nhu cầu đã ở trạng thái Đóng (do người dùng đóng tay hoặc hệ thống đã đóng trước đó).
-Riêng luồng CẢNH BÁO còn bị bỏ qua khi N &lt;= M, hoặc khi M = 0, hoặc khi nhu cầu đó đã được cảnh báo một lần rồi (không nhắc lại mỗi ngày).</t>
+Riêng luồng GỬI THÔNG BÁO còn bị bỏ qua khi N &lt;= M, hoặc khi M = 0, hoặc khi nhu cầu đó đã được thông báo một lần rồi (không nhắc lại mỗi ngày).</t>
         </is>
       </c>
       <c r="C4" s="4" t="n"/>
@@ -817,7 +817,7 @@
       <c r="M9" s="4" t="n"/>
       <c r="N9" s="5" t="n"/>
     </row>
-    <row r="10" ht="185" customHeight="1">
+    <row r="10" ht="219" customHeight="1">
       <c r="A10" s="2" t="inlineStr">
         <is>
           <t>9. Ghi chú đọc bảng</t>
@@ -828,8 +828,10 @@
           <t>Bẫy dễ sai nhất của đợt này:
 - N = 0 nghĩa là KHÔNG đặt thời hạn, không phải 'hết hạn ngay'. Mặc định sau khi lên bản mới, mọi lĩnh vực đều là 0, tức chưa nhu cầu nào bị đóng cho tới khi người quản trị khai N.
 - N &lt;= M thì KHÔNG có bước cảnh báo, nhu cầu vẫn bị đóng đúng hạn. Đừng báo lỗi 'thiếu thông báo'.
-- MỌI testcase kỳ vọng CÓ cảnh báo đều đã chốt sẵn N &gt; M trong cột Điều kiện. Khi test trên dữ liệu thật, phải kiểm N của lĩnh vực trước: N &lt;= M mà không thấy cảnh báo là ĐÚNG, không phải lỗi.
-- Nâng M lên KHÔNG phải lúc nào cũng làm nhiều nhu cầu được cảnh báo hơn: M vượt quá N của lĩnh vực nào thì nhu cầu của lĩnh vực đó MẤT cảnh báo.
+- PHÂN BIỆT 2 LUỒNG, đây là chỗ dễ báo nhầm nhất:
+   (a) TÔ CAM + '(còn X ngày)' ở cột hạn màn danh sách: hiện cho MỌI nhu cầu còn dưới M ngày là hết hạn, KHÔNG phụ thuộc N lớn hay nhỏ hơn M. Vùng cảnh báo TÍCH LUỸ — đặt M = 3 thì còn 3, 2, 1 ngày và quá hạn đều tô cam, không phải chỉ đúng mốc 3 ngày.
+   (b) THÔNG BÁO CHUÔNG do lệnh quét gửi: có ngoại lệ, N &lt;= M thì KHÔNG gửi.
+   =&gt; Nhu cầu N &lt;= M sẽ tô cam trên màn hình nhưng không ai nhận chuông. Đúng yêu cầu, không phải lỗi.
 - Nhu cầu quá hạn vẫn nằm trong danh sách cho tới lần quét kế tiếp (01:20 hôm sau) mới chuyển sang Đóng — trong khoảng đó cột hạn hiện '(quá hạn X ngày)' là đúng.
 - Ngày đóng là ngày HẾT HẠN chứ không phải ngày chạy quét.
 - Sửa N ở danh mục làm hạn của mọi nhu cầu thuộc lĩnh vực đó đổi ngay, kể cả nhu cầu cũ.
@@ -4354,7 +4356,7 @@
       <c r="P68" s="16" t="inlineStr"/>
       <c r="Q68" s="16" t="inlineStr"/>
     </row>
-    <row r="69" ht="61" customHeight="1">
+    <row r="69" ht="41" customHeight="1">
       <c r="A69" s="15" t="inlineStr">
         <is>
           <t>Hạn xử lý nhu cầu KH</t>
@@ -4399,7 +4401,7 @@
       <c r="I69" s="15" t="inlineStr">
         <is>
           <t>- Dòng #108 chuyển sang tô cam kèm '(còn 5 ngày)'
-- LƯU Ý: kết quả này chỉ đúng vì N = 30 vẫn LỚN HƠN M = 7. Nâng M vượt quá N thì cảnh báo TẮT đi chứ không bật thêm — xem TC ngay dưới</t>
+- Mọi dòng còn DƯỚI 7 ngày đều phải tô cam, không phải chỉ dòng đúng 7 ngày</t>
         </is>
       </c>
       <c r="J69" s="15" t="inlineStr"/>
@@ -4423,7 +4425,7 @@
       <c r="P69" s="16" t="inlineStr"/>
       <c r="Q69" s="16" t="inlineStr"/>
     </row>
-    <row r="70" ht="75" customHeight="1">
+    <row r="70" ht="151" customHeight="1">
       <c r="A70" s="15" t="inlineStr">
         <is>
           <t>Hạn xử lý nhu cầu KH</t>
@@ -4441,7 +4443,7 @@
       </c>
       <c r="D70" s="15" t="inlineStr">
         <is>
-          <t>Nâng M vượt quá N thì cảnh báo TẮT đi</t>
+          <t>Nhu cầu có N nhỏ hơn M vẫn tô cam trên màn hình</t>
         </is>
       </c>
       <c r="E70" s="16" t="inlineStr">
@@ -4451,24 +4453,25 @@
       </c>
       <c r="F70" s="15" t="inlineStr">
         <is>
-          <t>M = 3, nhu cầu #109 thuộc lĩnh vực có N = 5, đang tô cam vì còn 2 ngày.</t>
+          <t>M = 7, nhu cầu #109 thuộc lĩnh vực có N = 5 (tức N nhỏ hơn M), còn 2 ngày là hết hạn.</t>
         </is>
       </c>
       <c r="G70" s="15" t="inlineStr">
         <is>
-          <t>1. Đổi M thành 7 ở Cấu hình chung, lưu
-2. Quay lại màn Nhu cầu khách hàng, tải lại</t>
+          <t>1. Mở màn Nhu cầu khách hàng, xem dòng #109
+2. Chạy lệnh quét hạn nhu cầu, xem chuông thông báo</t>
         </is>
       </c>
       <c r="H70" s="15" t="inlineStr">
         <is>
-          <t>Cảnh báo trước khi đóng nhu cầu: 3 -&gt; 7</t>
+          <t>Thời gian hiệu lực nhu cầu: 5 · Cảnh báo trước khi đóng: 7</t>
         </is>
       </c>
       <c r="I70" s="15" t="inlineStr">
         <is>
-          <t>- Dòng #109 HẾT tô cam, hết ghi chú số ngày, chỉ còn ngày hết hạn
-- LƯU Ý: đây là ĐÚNG yêu cầu, không phải lỗi. N = 5 nay nhỏ hơn M = 7 nên rơi vào ngoại lệ 'N &lt;= M thì bỏ qua cảnh báo'
+          <t>- Bước 1: dòng #109 CÓ tô cam kèm '(còn 2 ngày)' — cột hạn luôn cho biết nhu cầu còn mấy ngày nữa tự đóng, không phụ thuộc N lớn hay nhỏ hơn M
+- Bước 2: KHÔNG ai nhận thông báo chuông cho #109 — đúng ngoại lệ 'N &lt;= M thì bỏ qua bước gửi thông báo' của yêu cầu, không phải lỗi
+- LƯU Ý: đây là 2 luồng khác nhau. Tô cam trên màn hình nói 'sắp tự đóng'; thông báo chuông là một hành động riêng và có ngoại lệ riêng
 - Nhu cầu vẫn bị đóng đúng hạn như thường</t>
         </is>
       </c>

</xml_diff>